<commit_message>
feat(vidrios): composición, seguridad y pedidos sellados
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sistemas" sheetId="1" r:id="R8282c5d1a603453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfiles" sheetId="2" r:id="Rd340470f3e4a4478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles y reglas de corte" sheetId="3" r:id="Rbff0e0ad12b047f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refuerzos" sheetId="4" r:id="Rc4c543501bf34c42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Límites" sheetId="5" r:id="Rf3c66cfdf453469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colores y SKU por color" sheetId="6" r:id="R2c87e79595a24e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="7" r:id="R5ef2f5f5e9bd4ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="8" r:id="Rc4ab87be3d7a42cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="9" r:id="R2260f5d3412b4a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sistemas" sheetId="1" r:id="R30854f96d12d406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfiles" sheetId="2" r:id="R40436b429cea4077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles y reglas de corte" sheetId="3" r:id="R0cd932817b2547dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refuerzos" sheetId="4" r:id="R5a60c4d7d2ee42d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Límites" sheetId="5" r:id="R2135c857c9f24d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colores y SKU por color" sheetId="6" r:id="Rd5c5cb88fcaf45f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="7" r:id="R3452336fba5a4cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas de vidrio" sheetId="8" r:id="R64164b13a3714a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="9" r:id="R17f0a2acee47424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" r:id="R3cf28316dcb84cde"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1142,6 +1143,344 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Precios de costo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
+      <x:c r="A4" s="5" t="str">
+        <x:v>Código de sistema</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>SKU</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Lista de costo</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>Proveedor</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Moneda</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="str">
+        <x:v>Vigente desde (aaaa-mm-dd)</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Vigente hasta (aaaa-mm-dd)</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>Tipo de artículo</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="J4" s="5" t="str">
+        <x:v>Costo unitario</x:v>
+      </x:c>
+      <x:c r="K4" s="5" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="7"/>
+      <x:c r="B5" s="7"/>
+      <x:c r="C5" s="7"/>
+      <x:c r="D5" s="7"/>
+      <x:c r="E5" s="7"/>
+      <x:c r="F5" s="12"/>
+      <x:c r="G5" s="13"/>
+      <x:c r="H5" s="7"/>
+      <x:c r="I5" s="7"/>
+      <x:c r="J5" s="8"/>
+      <x:c r="K5" s="7"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="7"/>
+      <x:c r="B6" s="7"/>
+      <x:c r="C6" s="7"/>
+      <x:c r="D6" s="7"/>
+      <x:c r="E6" s="7"/>
+      <x:c r="F6" s="12"/>
+      <x:c r="G6" s="13"/>
+      <x:c r="H6" s="7"/>
+      <x:c r="I6" s="7"/>
+      <x:c r="J6" s="8"/>
+      <x:c r="K6" s="7"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="7"/>
+      <x:c r="B7" s="7"/>
+      <x:c r="C7" s="7"/>
+      <x:c r="D7" s="7"/>
+      <x:c r="E7" s="7"/>
+      <x:c r="F7" s="12"/>
+      <x:c r="G7" s="13"/>
+      <x:c r="H7" s="7"/>
+      <x:c r="I7" s="7"/>
+      <x:c r="J7" s="8"/>
+      <x:c r="K7" s="7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="7"/>
+      <x:c r="B8" s="7"/>
+      <x:c r="C8" s="7"/>
+      <x:c r="D8" s="7"/>
+      <x:c r="E8" s="7"/>
+      <x:c r="F8" s="12"/>
+      <x:c r="G8" s="13"/>
+      <x:c r="H8" s="7"/>
+      <x:c r="I8" s="7"/>
+      <x:c r="J8" s="8"/>
+      <x:c r="K8" s="7"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="7"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="7"/>
+      <x:c r="D9" s="7"/>
+      <x:c r="E9" s="7"/>
+      <x:c r="F9" s="12"/>
+      <x:c r="G9" s="13"/>
+      <x:c r="H9" s="7"/>
+      <x:c r="I9" s="7"/>
+      <x:c r="J9" s="8"/>
+      <x:c r="K9" s="7"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="7"/>
+      <x:c r="B10" s="7"/>
+      <x:c r="C10" s="7"/>
+      <x:c r="D10" s="7"/>
+      <x:c r="E10" s="7"/>
+      <x:c r="F10" s="12"/>
+      <x:c r="G10" s="13"/>
+      <x:c r="H10" s="7"/>
+      <x:c r="I10" s="7"/>
+      <x:c r="J10" s="8"/>
+      <x:c r="K10" s="7"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="7"/>
+      <x:c r="B11" s="7"/>
+      <x:c r="C11" s="7"/>
+      <x:c r="D11" s="7"/>
+      <x:c r="E11" s="7"/>
+      <x:c r="F11" s="12"/>
+      <x:c r="G11" s="13"/>
+      <x:c r="H11" s="7"/>
+      <x:c r="I11" s="7"/>
+      <x:c r="J11" s="8"/>
+      <x:c r="K11" s="7"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="7"/>
+      <x:c r="B12" s="7"/>
+      <x:c r="C12" s="7"/>
+      <x:c r="D12" s="7"/>
+      <x:c r="E12" s="7"/>
+      <x:c r="F12" s="12"/>
+      <x:c r="G12" s="13"/>
+      <x:c r="H12" s="7"/>
+      <x:c r="I12" s="7"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="7"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="7"/>
+      <x:c r="B13" s="7"/>
+      <x:c r="C13" s="7"/>
+      <x:c r="D13" s="7"/>
+      <x:c r="E13" s="7"/>
+      <x:c r="F13" s="12"/>
+      <x:c r="G13" s="13"/>
+      <x:c r="H13" s="7"/>
+      <x:c r="I13" s="7"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="7"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7"/>
+      <x:c r="B14" s="7"/>
+      <x:c r="C14" s="7"/>
+      <x:c r="D14" s="7"/>
+      <x:c r="E14" s="7"/>
+      <x:c r="F14" s="12"/>
+      <x:c r="G14" s="13"/>
+      <x:c r="H14" s="7"/>
+      <x:c r="I14" s="7"/>
+      <x:c r="J14" s="8"/>
+      <x:c r="K14" s="7"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="7"/>
+      <x:c r="B15" s="7"/>
+      <x:c r="C15" s="7"/>
+      <x:c r="D15" s="7"/>
+      <x:c r="E15" s="7"/>
+      <x:c r="F15" s="12"/>
+      <x:c r="G15" s="13"/>
+      <x:c r="H15" s="7"/>
+      <x:c r="I15" s="7"/>
+      <x:c r="J15" s="8"/>
+      <x:c r="K15" s="7"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="7"/>
+      <x:c r="B16" s="7"/>
+      <x:c r="C16" s="7"/>
+      <x:c r="D16" s="7"/>
+      <x:c r="E16" s="7"/>
+      <x:c r="F16" s="12"/>
+      <x:c r="G16" s="13"/>
+      <x:c r="H16" s="7"/>
+      <x:c r="I16" s="7"/>
+      <x:c r="J16" s="8"/>
+      <x:c r="K16" s="7"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="7"/>
+      <x:c r="B17" s="7"/>
+      <x:c r="C17" s="7"/>
+      <x:c r="D17" s="7"/>
+      <x:c r="E17" s="7"/>
+      <x:c r="F17" s="12"/>
+      <x:c r="G17" s="13"/>
+      <x:c r="H17" s="7"/>
+      <x:c r="I17" s="7"/>
+      <x:c r="J17" s="8"/>
+      <x:c r="K17" s="7"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="7"/>
+      <x:c r="B18" s="7"/>
+      <x:c r="C18" s="7"/>
+      <x:c r="D18" s="7"/>
+      <x:c r="E18" s="7"/>
+      <x:c r="F18" s="12"/>
+      <x:c r="G18" s="13"/>
+      <x:c r="H18" s="7"/>
+      <x:c r="I18" s="7"/>
+      <x:c r="J18" s="8"/>
+      <x:c r="K18" s="7"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="7"/>
+      <x:c r="B19" s="7"/>
+      <x:c r="C19" s="7"/>
+      <x:c r="D19" s="7"/>
+      <x:c r="E19" s="7"/>
+      <x:c r="F19" s="12"/>
+      <x:c r="G19" s="13"/>
+      <x:c r="H19" s="7"/>
+      <x:c r="I19" s="7"/>
+      <x:c r="J19" s="8"/>
+      <x:c r="K19" s="7"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="7"/>
+      <x:c r="B20" s="7"/>
+      <x:c r="C20" s="7"/>
+      <x:c r="D20" s="7"/>
+      <x:c r="E20" s="7"/>
+      <x:c r="F20" s="12"/>
+      <x:c r="G20" s="13"/>
+      <x:c r="H20" s="7"/>
+      <x:c r="I20" s="7"/>
+      <x:c r="J20" s="8"/>
+      <x:c r="K20" s="7"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="7"/>
+      <x:c r="B21" s="7"/>
+      <x:c r="C21" s="7"/>
+      <x:c r="D21" s="7"/>
+      <x:c r="E21" s="7"/>
+      <x:c r="F21" s="12"/>
+      <x:c r="G21" s="13"/>
+      <x:c r="H21" s="7"/>
+      <x:c r="I21" s="7"/>
+      <x:c r="J21" s="8"/>
+      <x:c r="K21" s="7"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="7"/>
+      <x:c r="B22" s="7"/>
+      <x:c r="C22" s="7"/>
+      <x:c r="D22" s="7"/>
+      <x:c r="E22" s="7"/>
+      <x:c r="F22" s="12"/>
+      <x:c r="G22" s="13"/>
+      <x:c r="H22" s="7"/>
+      <x:c r="I22" s="7"/>
+      <x:c r="J22" s="8"/>
+      <x:c r="K22" s="7"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="7"/>
+      <x:c r="B23" s="7"/>
+      <x:c r="C23" s="7"/>
+      <x:c r="D23" s="7"/>
+      <x:c r="E23" s="7"/>
+      <x:c r="F23" s="12"/>
+      <x:c r="G23" s="13"/>
+      <x:c r="H23" s="7"/>
+      <x:c r="I23" s="7"/>
+      <x:c r="J23" s="8"/>
+      <x:c r="K23" s="7"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="7"/>
+      <x:c r="B24" s="7"/>
+      <x:c r="C24" s="7"/>
+      <x:c r="D24" s="7"/>
+      <x:c r="E24" s="7"/>
+      <x:c r="F24" s="12"/>
+      <x:c r="G24" s="13"/>
+      <x:c r="H24" s="7"/>
+      <x:c r="I24" s="7"/>
+      <x:c r="J24" s="8"/>
+      <x:c r="K24" s="7"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="E5:E24">
+      <x:formula1>"CLP,USD"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H5:H24">
+      <x:formula1>"Perfil,Refuerzo,Vidrio,Herraje,Otro"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I24">
+      <x:formula1>"Barra,Metro,Metro cuadrado,Kit,Unidad"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -2646,12 +2985,31 @@
     <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="22" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="22" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="22" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="30" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="22" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="22" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="22" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="22" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="30" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2675,33 +3033,90 @@
         <x:v>Composición de vidrio</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
+        <x:v>Nombre comercial</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Ejemplo sintético</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="str">
+        <x:v>Ug de proveedor (W/m²K)</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Factor solar g de proveedor</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>Transmisión luminosa de proveedor</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Clase NCh 135 de proveedor</x:v>
+      </x:c>
+      <x:c r="J4" s="5" t="str">
+        <x:v>Peso declarado de proveedor (kg/m²)</x:v>
+      </x:c>
+      <x:c r="K4" s="5" t="str">
+        <x:v>Área mínima facturable (m²)</x:v>
+      </x:c>
+      <x:c r="L4" s="5" t="str">
+        <x:v>Ancho mínimo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="M4" s="5" t="str">
+        <x:v>Ancho máximo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="N4" s="5" t="str">
+        <x:v>Alto mínimo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="O4" s="5" t="str">
+        <x:v>Alto máximo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="P4" s="5" t="str">
+        <x:v>Área máxima de vidrio (m²)</x:v>
+      </x:c>
+      <x:c r="Q4" s="5" t="str">
+        <x:v>Relación de aspecto máxima de vidrio</x:v>
+      </x:c>
+      <x:c r="R4" s="5" t="str">
+        <x:v>SKU recargo templado</x:v>
+      </x:c>
+      <x:c r="S4" s="5" t="str">
+        <x:v>SKU recargo pulido</x:v>
+      </x:c>
+      <x:c r="T4" s="5" t="str">
+        <x:v>SKU recargo perforación</x:v>
+      </x:c>
+      <x:c r="U4" s="5" t="str">
+        <x:v>SKU palillaje por metro</x:v>
+      </x:c>
+      <x:c r="V4" s="5" t="str">
+        <x:v>SKU palillaje por cruce</x:v>
+      </x:c>
+      <x:c r="W4" s="5" t="str">
         <x:v>SKU de compra</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="str">
+      <x:c r="X4" s="5" t="str">
         <x:v>Fabricante</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="str">
+      <x:c r="Y4" s="5" t="str">
         <x:v>Versión</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="str">
+      <x:c r="Z4" s="5" t="str">
         <x:v>Espesor para junquillo (mm)</x:v>
       </x:c>
-      <x:c r="H4" s="5" t="str">
+      <x:c r="AA4" s="5" t="str">
         <x:v>SKU de junquillo</x:v>
       </x:c>
-      <x:c r="I4" s="5" t="str">
+      <x:c r="AB4" s="5" t="str">
         <x:v>Ancho de junquillo (mm)</x:v>
       </x:c>
-      <x:c r="J4" s="5" t="str">
+      <x:c r="AC4" s="5" t="str">
         <x:v>Junta interior (mm)</x:v>
       </x:c>
-      <x:c r="K4" s="5" t="str">
+      <x:c r="AD4" s="5" t="str">
         <x:v>Junta exterior (mm)</x:v>
       </x:c>
-      <x:c r="L4" s="5" t="str">
+      <x:c r="AE4" s="5" t="str">
         <x:v>Adición al corte de junquillo (mm)</x:v>
       </x:c>
-      <x:c r="M4" s="5" t="str">
+      <x:c r="AF4" s="5" t="str">
         <x:v>Fuente</x:v>
       </x:c>
     </x:row>
@@ -2709,308 +3124,986 @@
       <x:c r="A5" s="7"/>
       <x:c r="B5" s="7"/>
       <x:c r="C5" s="7"/>
-      <x:c r="D5" s="7"/>
-      <x:c r="E5" s="7"/>
-      <x:c r="F5" s="9"/>
+      <x:c r="D5" s="6"/>
+      <x:c r="E5" s="6"/>
+      <x:c r="F5" s="10"/>
       <x:c r="G5" s="10"/>
-      <x:c r="H5" s="6"/>
-      <x:c r="I5" s="10"/>
+      <x:c r="H5" s="10"/>
+      <x:c r="I5" s="6"/>
       <x:c r="J5" s="10"/>
       <x:c r="K5" s="10"/>
       <x:c r="L5" s="10"/>
-      <x:c r="M5" s="7"/>
+      <x:c r="M5" s="10"/>
+      <x:c r="N5" s="10"/>
+      <x:c r="O5" s="10"/>
+      <x:c r="P5" s="10"/>
+      <x:c r="Q5" s="10"/>
+      <x:c r="R5" s="6"/>
+      <x:c r="S5" s="6"/>
+      <x:c r="T5" s="6"/>
+      <x:c r="U5" s="6"/>
+      <x:c r="V5" s="6"/>
+      <x:c r="W5" s="7"/>
+      <x:c r="X5" s="7"/>
+      <x:c r="Y5" s="9"/>
+      <x:c r="Z5" s="10"/>
+      <x:c r="AA5" s="6"/>
+      <x:c r="AB5" s="10"/>
+      <x:c r="AC5" s="10"/>
+      <x:c r="AD5" s="10"/>
+      <x:c r="AE5" s="10"/>
+      <x:c r="AF5" s="7"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7"/>
       <x:c r="B6" s="7"/>
       <x:c r="C6" s="7"/>
-      <x:c r="D6" s="7"/>
-      <x:c r="E6" s="7"/>
-      <x:c r="F6" s="9"/>
+      <x:c r="D6" s="6"/>
+      <x:c r="E6" s="6"/>
+      <x:c r="F6" s="10"/>
       <x:c r="G6" s="10"/>
-      <x:c r="H6" s="6"/>
-      <x:c r="I6" s="10"/>
+      <x:c r="H6" s="10"/>
+      <x:c r="I6" s="6"/>
       <x:c r="J6" s="10"/>
       <x:c r="K6" s="10"/>
       <x:c r="L6" s="10"/>
-      <x:c r="M6" s="7"/>
+      <x:c r="M6" s="10"/>
+      <x:c r="N6" s="10"/>
+      <x:c r="O6" s="10"/>
+      <x:c r="P6" s="10"/>
+      <x:c r="Q6" s="10"/>
+      <x:c r="R6" s="6"/>
+      <x:c r="S6" s="6"/>
+      <x:c r="T6" s="6"/>
+      <x:c r="U6" s="6"/>
+      <x:c r="V6" s="6"/>
+      <x:c r="W6" s="7"/>
+      <x:c r="X6" s="7"/>
+      <x:c r="Y6" s="9"/>
+      <x:c r="Z6" s="10"/>
+      <x:c r="AA6" s="6"/>
+      <x:c r="AB6" s="10"/>
+      <x:c r="AC6" s="10"/>
+      <x:c r="AD6" s="10"/>
+      <x:c r="AE6" s="10"/>
+      <x:c r="AF6" s="7"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7"/>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
-      <x:c r="D7" s="7"/>
-      <x:c r="E7" s="7"/>
-      <x:c r="F7" s="9"/>
+      <x:c r="D7" s="6"/>
+      <x:c r="E7" s="6"/>
+      <x:c r="F7" s="10"/>
       <x:c r="G7" s="10"/>
-      <x:c r="H7" s="6"/>
-      <x:c r="I7" s="10"/>
+      <x:c r="H7" s="10"/>
+      <x:c r="I7" s="6"/>
       <x:c r="J7" s="10"/>
       <x:c r="K7" s="10"/>
       <x:c r="L7" s="10"/>
-      <x:c r="M7" s="7"/>
+      <x:c r="M7" s="10"/>
+      <x:c r="N7" s="10"/>
+      <x:c r="O7" s="10"/>
+      <x:c r="P7" s="10"/>
+      <x:c r="Q7" s="10"/>
+      <x:c r="R7" s="6"/>
+      <x:c r="S7" s="6"/>
+      <x:c r="T7" s="6"/>
+      <x:c r="U7" s="6"/>
+      <x:c r="V7" s="6"/>
+      <x:c r="W7" s="7"/>
+      <x:c r="X7" s="7"/>
+      <x:c r="Y7" s="9"/>
+      <x:c r="Z7" s="10"/>
+      <x:c r="AA7" s="6"/>
+      <x:c r="AB7" s="10"/>
+      <x:c r="AC7" s="10"/>
+      <x:c r="AD7" s="10"/>
+      <x:c r="AE7" s="10"/>
+      <x:c r="AF7" s="7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7"/>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
-      <x:c r="D8" s="7"/>
-      <x:c r="E8" s="7"/>
-      <x:c r="F8" s="9"/>
+      <x:c r="D8" s="6"/>
+      <x:c r="E8" s="6"/>
+      <x:c r="F8" s="10"/>
       <x:c r="G8" s="10"/>
-      <x:c r="H8" s="6"/>
-      <x:c r="I8" s="10"/>
+      <x:c r="H8" s="10"/>
+      <x:c r="I8" s="6"/>
       <x:c r="J8" s="10"/>
       <x:c r="K8" s="10"/>
       <x:c r="L8" s="10"/>
-      <x:c r="M8" s="7"/>
+      <x:c r="M8" s="10"/>
+      <x:c r="N8" s="10"/>
+      <x:c r="O8" s="10"/>
+      <x:c r="P8" s="10"/>
+      <x:c r="Q8" s="10"/>
+      <x:c r="R8" s="6"/>
+      <x:c r="S8" s="6"/>
+      <x:c r="T8" s="6"/>
+      <x:c r="U8" s="6"/>
+      <x:c r="V8" s="6"/>
+      <x:c r="W8" s="7"/>
+      <x:c r="X8" s="7"/>
+      <x:c r="Y8" s="9"/>
+      <x:c r="Z8" s="10"/>
+      <x:c r="AA8" s="6"/>
+      <x:c r="AB8" s="10"/>
+      <x:c r="AC8" s="10"/>
+      <x:c r="AD8" s="10"/>
+      <x:c r="AE8" s="10"/>
+      <x:c r="AF8" s="7"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7"/>
       <x:c r="B9" s="7"/>
       <x:c r="C9" s="7"/>
-      <x:c r="D9" s="7"/>
-      <x:c r="E9" s="7"/>
-      <x:c r="F9" s="9"/>
+      <x:c r="D9" s="6"/>
+      <x:c r="E9" s="6"/>
+      <x:c r="F9" s="10"/>
       <x:c r="G9" s="10"/>
-      <x:c r="H9" s="6"/>
-      <x:c r="I9" s="10"/>
+      <x:c r="H9" s="10"/>
+      <x:c r="I9" s="6"/>
       <x:c r="J9" s="10"/>
       <x:c r="K9" s="10"/>
       <x:c r="L9" s="10"/>
-      <x:c r="M9" s="7"/>
+      <x:c r="M9" s="10"/>
+      <x:c r="N9" s="10"/>
+      <x:c r="O9" s="10"/>
+      <x:c r="P9" s="10"/>
+      <x:c r="Q9" s="10"/>
+      <x:c r="R9" s="6"/>
+      <x:c r="S9" s="6"/>
+      <x:c r="T9" s="6"/>
+      <x:c r="U9" s="6"/>
+      <x:c r="V9" s="6"/>
+      <x:c r="W9" s="7"/>
+      <x:c r="X9" s="7"/>
+      <x:c r="Y9" s="9"/>
+      <x:c r="Z9" s="10"/>
+      <x:c r="AA9" s="6"/>
+      <x:c r="AB9" s="10"/>
+      <x:c r="AC9" s="10"/>
+      <x:c r="AD9" s="10"/>
+      <x:c r="AE9" s="10"/>
+      <x:c r="AF9" s="7"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7"/>
       <x:c r="B10" s="7"/>
       <x:c r="C10" s="7"/>
-      <x:c r="D10" s="7"/>
-      <x:c r="E10" s="7"/>
-      <x:c r="F10" s="9"/>
+      <x:c r="D10" s="6"/>
+      <x:c r="E10" s="6"/>
+      <x:c r="F10" s="10"/>
       <x:c r="G10" s="10"/>
-      <x:c r="H10" s="6"/>
-      <x:c r="I10" s="10"/>
+      <x:c r="H10" s="10"/>
+      <x:c r="I10" s="6"/>
       <x:c r="J10" s="10"/>
       <x:c r="K10" s="10"/>
       <x:c r="L10" s="10"/>
-      <x:c r="M10" s="7"/>
+      <x:c r="M10" s="10"/>
+      <x:c r="N10" s="10"/>
+      <x:c r="O10" s="10"/>
+      <x:c r="P10" s="10"/>
+      <x:c r="Q10" s="10"/>
+      <x:c r="R10" s="6"/>
+      <x:c r="S10" s="6"/>
+      <x:c r="T10" s="6"/>
+      <x:c r="U10" s="6"/>
+      <x:c r="V10" s="6"/>
+      <x:c r="W10" s="7"/>
+      <x:c r="X10" s="7"/>
+      <x:c r="Y10" s="9"/>
+      <x:c r="Z10" s="10"/>
+      <x:c r="AA10" s="6"/>
+      <x:c r="AB10" s="10"/>
+      <x:c r="AC10" s="10"/>
+      <x:c r="AD10" s="10"/>
+      <x:c r="AE10" s="10"/>
+      <x:c r="AF10" s="7"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7"/>
       <x:c r="B11" s="7"/>
       <x:c r="C11" s="7"/>
-      <x:c r="D11" s="7"/>
-      <x:c r="E11" s="7"/>
-      <x:c r="F11" s="9"/>
+      <x:c r="D11" s="6"/>
+      <x:c r="E11" s="6"/>
+      <x:c r="F11" s="10"/>
       <x:c r="G11" s="10"/>
-      <x:c r="H11" s="6"/>
-      <x:c r="I11" s="10"/>
+      <x:c r="H11" s="10"/>
+      <x:c r="I11" s="6"/>
       <x:c r="J11" s="10"/>
       <x:c r="K11" s="10"/>
       <x:c r="L11" s="10"/>
-      <x:c r="M11" s="7"/>
+      <x:c r="M11" s="10"/>
+      <x:c r="N11" s="10"/>
+      <x:c r="O11" s="10"/>
+      <x:c r="P11" s="10"/>
+      <x:c r="Q11" s="10"/>
+      <x:c r="R11" s="6"/>
+      <x:c r="S11" s="6"/>
+      <x:c r="T11" s="6"/>
+      <x:c r="U11" s="6"/>
+      <x:c r="V11" s="6"/>
+      <x:c r="W11" s="7"/>
+      <x:c r="X11" s="7"/>
+      <x:c r="Y11" s="9"/>
+      <x:c r="Z11" s="10"/>
+      <x:c r="AA11" s="6"/>
+      <x:c r="AB11" s="10"/>
+      <x:c r="AC11" s="10"/>
+      <x:c r="AD11" s="10"/>
+      <x:c r="AE11" s="10"/>
+      <x:c r="AF11" s="7"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7"/>
       <x:c r="B12" s="7"/>
       <x:c r="C12" s="7"/>
-      <x:c r="D12" s="7"/>
-      <x:c r="E12" s="7"/>
-      <x:c r="F12" s="9"/>
+      <x:c r="D12" s="6"/>
+      <x:c r="E12" s="6"/>
+      <x:c r="F12" s="10"/>
       <x:c r="G12" s="10"/>
-      <x:c r="H12" s="6"/>
-      <x:c r="I12" s="10"/>
+      <x:c r="H12" s="10"/>
+      <x:c r="I12" s="6"/>
       <x:c r="J12" s="10"/>
       <x:c r="K12" s="10"/>
       <x:c r="L12" s="10"/>
-      <x:c r="M12" s="7"/>
+      <x:c r="M12" s="10"/>
+      <x:c r="N12" s="10"/>
+      <x:c r="O12" s="10"/>
+      <x:c r="P12" s="10"/>
+      <x:c r="Q12" s="10"/>
+      <x:c r="R12" s="6"/>
+      <x:c r="S12" s="6"/>
+      <x:c r="T12" s="6"/>
+      <x:c r="U12" s="6"/>
+      <x:c r="V12" s="6"/>
+      <x:c r="W12" s="7"/>
+      <x:c r="X12" s="7"/>
+      <x:c r="Y12" s="9"/>
+      <x:c r="Z12" s="10"/>
+      <x:c r="AA12" s="6"/>
+      <x:c r="AB12" s="10"/>
+      <x:c r="AC12" s="10"/>
+      <x:c r="AD12" s="10"/>
+      <x:c r="AE12" s="10"/>
+      <x:c r="AF12" s="7"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7"/>
       <x:c r="B13" s="7"/>
       <x:c r="C13" s="7"/>
-      <x:c r="D13" s="7"/>
-      <x:c r="E13" s="7"/>
-      <x:c r="F13" s="9"/>
+      <x:c r="D13" s="6"/>
+      <x:c r="E13" s="6"/>
+      <x:c r="F13" s="10"/>
       <x:c r="G13" s="10"/>
-      <x:c r="H13" s="6"/>
-      <x:c r="I13" s="10"/>
+      <x:c r="H13" s="10"/>
+      <x:c r="I13" s="6"/>
       <x:c r="J13" s="10"/>
       <x:c r="K13" s="10"/>
       <x:c r="L13" s="10"/>
-      <x:c r="M13" s="7"/>
+      <x:c r="M13" s="10"/>
+      <x:c r="N13" s="10"/>
+      <x:c r="O13" s="10"/>
+      <x:c r="P13" s="10"/>
+      <x:c r="Q13" s="10"/>
+      <x:c r="R13" s="6"/>
+      <x:c r="S13" s="6"/>
+      <x:c r="T13" s="6"/>
+      <x:c r="U13" s="6"/>
+      <x:c r="V13" s="6"/>
+      <x:c r="W13" s="7"/>
+      <x:c r="X13" s="7"/>
+      <x:c r="Y13" s="9"/>
+      <x:c r="Z13" s="10"/>
+      <x:c r="AA13" s="6"/>
+      <x:c r="AB13" s="10"/>
+      <x:c r="AC13" s="10"/>
+      <x:c r="AD13" s="10"/>
+      <x:c r="AE13" s="10"/>
+      <x:c r="AF13" s="7"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7"/>
       <x:c r="B14" s="7"/>
       <x:c r="C14" s="7"/>
-      <x:c r="D14" s="7"/>
-      <x:c r="E14" s="7"/>
-      <x:c r="F14" s="9"/>
+      <x:c r="D14" s="6"/>
+      <x:c r="E14" s="6"/>
+      <x:c r="F14" s="10"/>
       <x:c r="G14" s="10"/>
-      <x:c r="H14" s="6"/>
-      <x:c r="I14" s="10"/>
+      <x:c r="H14" s="10"/>
+      <x:c r="I14" s="6"/>
       <x:c r="J14" s="10"/>
       <x:c r="K14" s="10"/>
       <x:c r="L14" s="10"/>
-      <x:c r="M14" s="7"/>
+      <x:c r="M14" s="10"/>
+      <x:c r="N14" s="10"/>
+      <x:c r="O14" s="10"/>
+      <x:c r="P14" s="10"/>
+      <x:c r="Q14" s="10"/>
+      <x:c r="R14" s="6"/>
+      <x:c r="S14" s="6"/>
+      <x:c r="T14" s="6"/>
+      <x:c r="U14" s="6"/>
+      <x:c r="V14" s="6"/>
+      <x:c r="W14" s="7"/>
+      <x:c r="X14" s="7"/>
+      <x:c r="Y14" s="9"/>
+      <x:c r="Z14" s="10"/>
+      <x:c r="AA14" s="6"/>
+      <x:c r="AB14" s="10"/>
+      <x:c r="AC14" s="10"/>
+      <x:c r="AD14" s="10"/>
+      <x:c r="AE14" s="10"/>
+      <x:c r="AF14" s="7"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7"/>
       <x:c r="B15" s="7"/>
       <x:c r="C15" s="7"/>
-      <x:c r="D15" s="7"/>
-      <x:c r="E15" s="7"/>
-      <x:c r="F15" s="9"/>
+      <x:c r="D15" s="6"/>
+      <x:c r="E15" s="6"/>
+      <x:c r="F15" s="10"/>
       <x:c r="G15" s="10"/>
-      <x:c r="H15" s="6"/>
-      <x:c r="I15" s="10"/>
+      <x:c r="H15" s="10"/>
+      <x:c r="I15" s="6"/>
       <x:c r="J15" s="10"/>
       <x:c r="K15" s="10"/>
       <x:c r="L15" s="10"/>
-      <x:c r="M15" s="7"/>
+      <x:c r="M15" s="10"/>
+      <x:c r="N15" s="10"/>
+      <x:c r="O15" s="10"/>
+      <x:c r="P15" s="10"/>
+      <x:c r="Q15" s="10"/>
+      <x:c r="R15" s="6"/>
+      <x:c r="S15" s="6"/>
+      <x:c r="T15" s="6"/>
+      <x:c r="U15" s="6"/>
+      <x:c r="V15" s="6"/>
+      <x:c r="W15" s="7"/>
+      <x:c r="X15" s="7"/>
+      <x:c r="Y15" s="9"/>
+      <x:c r="Z15" s="10"/>
+      <x:c r="AA15" s="6"/>
+      <x:c r="AB15" s="10"/>
+      <x:c r="AC15" s="10"/>
+      <x:c r="AD15" s="10"/>
+      <x:c r="AE15" s="10"/>
+      <x:c r="AF15" s="7"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7"/>
       <x:c r="B16" s="7"/>
       <x:c r="C16" s="7"/>
-      <x:c r="D16" s="7"/>
-      <x:c r="E16" s="7"/>
-      <x:c r="F16" s="9"/>
+      <x:c r="D16" s="6"/>
+      <x:c r="E16" s="6"/>
+      <x:c r="F16" s="10"/>
       <x:c r="G16" s="10"/>
-      <x:c r="H16" s="6"/>
-      <x:c r="I16" s="10"/>
+      <x:c r="H16" s="10"/>
+      <x:c r="I16" s="6"/>
       <x:c r="J16" s="10"/>
       <x:c r="K16" s="10"/>
       <x:c r="L16" s="10"/>
-      <x:c r="M16" s="7"/>
+      <x:c r="M16" s="10"/>
+      <x:c r="N16" s="10"/>
+      <x:c r="O16" s="10"/>
+      <x:c r="P16" s="10"/>
+      <x:c r="Q16" s="10"/>
+      <x:c r="R16" s="6"/>
+      <x:c r="S16" s="6"/>
+      <x:c r="T16" s="6"/>
+      <x:c r="U16" s="6"/>
+      <x:c r="V16" s="6"/>
+      <x:c r="W16" s="7"/>
+      <x:c r="X16" s="7"/>
+      <x:c r="Y16" s="9"/>
+      <x:c r="Z16" s="10"/>
+      <x:c r="AA16" s="6"/>
+      <x:c r="AB16" s="10"/>
+      <x:c r="AC16" s="10"/>
+      <x:c r="AD16" s="10"/>
+      <x:c r="AE16" s="10"/>
+      <x:c r="AF16" s="7"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7"/>
       <x:c r="B17" s="7"/>
       <x:c r="C17" s="7"/>
-      <x:c r="D17" s="7"/>
-      <x:c r="E17" s="7"/>
-      <x:c r="F17" s="9"/>
+      <x:c r="D17" s="6"/>
+      <x:c r="E17" s="6"/>
+      <x:c r="F17" s="10"/>
       <x:c r="G17" s="10"/>
-      <x:c r="H17" s="6"/>
-      <x:c r="I17" s="10"/>
+      <x:c r="H17" s="10"/>
+      <x:c r="I17" s="6"/>
       <x:c r="J17" s="10"/>
       <x:c r="K17" s="10"/>
       <x:c r="L17" s="10"/>
-      <x:c r="M17" s="7"/>
+      <x:c r="M17" s="10"/>
+      <x:c r="N17" s="10"/>
+      <x:c r="O17" s="10"/>
+      <x:c r="P17" s="10"/>
+      <x:c r="Q17" s="10"/>
+      <x:c r="R17" s="6"/>
+      <x:c r="S17" s="6"/>
+      <x:c r="T17" s="6"/>
+      <x:c r="U17" s="6"/>
+      <x:c r="V17" s="6"/>
+      <x:c r="W17" s="7"/>
+      <x:c r="X17" s="7"/>
+      <x:c r="Y17" s="9"/>
+      <x:c r="Z17" s="10"/>
+      <x:c r="AA17" s="6"/>
+      <x:c r="AB17" s="10"/>
+      <x:c r="AC17" s="10"/>
+      <x:c r="AD17" s="10"/>
+      <x:c r="AE17" s="10"/>
+      <x:c r="AF17" s="7"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7"/>
       <x:c r="B18" s="7"/>
       <x:c r="C18" s="7"/>
-      <x:c r="D18" s="7"/>
-      <x:c r="E18" s="7"/>
-      <x:c r="F18" s="9"/>
+      <x:c r="D18" s="6"/>
+      <x:c r="E18" s="6"/>
+      <x:c r="F18" s="10"/>
       <x:c r="G18" s="10"/>
-      <x:c r="H18" s="6"/>
-      <x:c r="I18" s="10"/>
+      <x:c r="H18" s="10"/>
+      <x:c r="I18" s="6"/>
       <x:c r="J18" s="10"/>
       <x:c r="K18" s="10"/>
       <x:c r="L18" s="10"/>
-      <x:c r="M18" s="7"/>
+      <x:c r="M18" s="10"/>
+      <x:c r="N18" s="10"/>
+      <x:c r="O18" s="10"/>
+      <x:c r="P18" s="10"/>
+      <x:c r="Q18" s="10"/>
+      <x:c r="R18" s="6"/>
+      <x:c r="S18" s="6"/>
+      <x:c r="T18" s="6"/>
+      <x:c r="U18" s="6"/>
+      <x:c r="V18" s="6"/>
+      <x:c r="W18" s="7"/>
+      <x:c r="X18" s="7"/>
+      <x:c r="Y18" s="9"/>
+      <x:c r="Z18" s="10"/>
+      <x:c r="AA18" s="6"/>
+      <x:c r="AB18" s="10"/>
+      <x:c r="AC18" s="10"/>
+      <x:c r="AD18" s="10"/>
+      <x:c r="AE18" s="10"/>
+      <x:c r="AF18" s="7"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7"/>
       <x:c r="B19" s="7"/>
       <x:c r="C19" s="7"/>
-      <x:c r="D19" s="7"/>
-      <x:c r="E19" s="7"/>
-      <x:c r="F19" s="9"/>
+      <x:c r="D19" s="6"/>
+      <x:c r="E19" s="6"/>
+      <x:c r="F19" s="10"/>
       <x:c r="G19" s="10"/>
-      <x:c r="H19" s="6"/>
-      <x:c r="I19" s="10"/>
+      <x:c r="H19" s="10"/>
+      <x:c r="I19" s="6"/>
       <x:c r="J19" s="10"/>
       <x:c r="K19" s="10"/>
       <x:c r="L19" s="10"/>
-      <x:c r="M19" s="7"/>
+      <x:c r="M19" s="10"/>
+      <x:c r="N19" s="10"/>
+      <x:c r="O19" s="10"/>
+      <x:c r="P19" s="10"/>
+      <x:c r="Q19" s="10"/>
+      <x:c r="R19" s="6"/>
+      <x:c r="S19" s="6"/>
+      <x:c r="T19" s="6"/>
+      <x:c r="U19" s="6"/>
+      <x:c r="V19" s="6"/>
+      <x:c r="W19" s="7"/>
+      <x:c r="X19" s="7"/>
+      <x:c r="Y19" s="9"/>
+      <x:c r="Z19" s="10"/>
+      <x:c r="AA19" s="6"/>
+      <x:c r="AB19" s="10"/>
+      <x:c r="AC19" s="10"/>
+      <x:c r="AD19" s="10"/>
+      <x:c r="AE19" s="10"/>
+      <x:c r="AF19" s="7"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7"/>
       <x:c r="B20" s="7"/>
       <x:c r="C20" s="7"/>
-      <x:c r="D20" s="7"/>
-      <x:c r="E20" s="7"/>
-      <x:c r="F20" s="9"/>
+      <x:c r="D20" s="6"/>
+      <x:c r="E20" s="6"/>
+      <x:c r="F20" s="10"/>
       <x:c r="G20" s="10"/>
-      <x:c r="H20" s="6"/>
-      <x:c r="I20" s="10"/>
+      <x:c r="H20" s="10"/>
+      <x:c r="I20" s="6"/>
       <x:c r="J20" s="10"/>
       <x:c r="K20" s="10"/>
       <x:c r="L20" s="10"/>
-      <x:c r="M20" s="7"/>
+      <x:c r="M20" s="10"/>
+      <x:c r="N20" s="10"/>
+      <x:c r="O20" s="10"/>
+      <x:c r="P20" s="10"/>
+      <x:c r="Q20" s="10"/>
+      <x:c r="R20" s="6"/>
+      <x:c r="S20" s="6"/>
+      <x:c r="T20" s="6"/>
+      <x:c r="U20" s="6"/>
+      <x:c r="V20" s="6"/>
+      <x:c r="W20" s="7"/>
+      <x:c r="X20" s="7"/>
+      <x:c r="Y20" s="9"/>
+      <x:c r="Z20" s="10"/>
+      <x:c r="AA20" s="6"/>
+      <x:c r="AB20" s="10"/>
+      <x:c r="AC20" s="10"/>
+      <x:c r="AD20" s="10"/>
+      <x:c r="AE20" s="10"/>
+      <x:c r="AF20" s="7"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7"/>
       <x:c r="B21" s="7"/>
       <x:c r="C21" s="7"/>
-      <x:c r="D21" s="7"/>
-      <x:c r="E21" s="7"/>
-      <x:c r="F21" s="9"/>
+      <x:c r="D21" s="6"/>
+      <x:c r="E21" s="6"/>
+      <x:c r="F21" s="10"/>
       <x:c r="G21" s="10"/>
-      <x:c r="H21" s="6"/>
-      <x:c r="I21" s="10"/>
+      <x:c r="H21" s="10"/>
+      <x:c r="I21" s="6"/>
       <x:c r="J21" s="10"/>
       <x:c r="K21" s="10"/>
       <x:c r="L21" s="10"/>
-      <x:c r="M21" s="7"/>
+      <x:c r="M21" s="10"/>
+      <x:c r="N21" s="10"/>
+      <x:c r="O21" s="10"/>
+      <x:c r="P21" s="10"/>
+      <x:c r="Q21" s="10"/>
+      <x:c r="R21" s="6"/>
+      <x:c r="S21" s="6"/>
+      <x:c r="T21" s="6"/>
+      <x:c r="U21" s="6"/>
+      <x:c r="V21" s="6"/>
+      <x:c r="W21" s="7"/>
+      <x:c r="X21" s="7"/>
+      <x:c r="Y21" s="9"/>
+      <x:c r="Z21" s="10"/>
+      <x:c r="AA21" s="6"/>
+      <x:c r="AB21" s="10"/>
+      <x:c r="AC21" s="10"/>
+      <x:c r="AD21" s="10"/>
+      <x:c r="AE21" s="10"/>
+      <x:c r="AF21" s="7"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="7"/>
       <x:c r="B22" s="7"/>
       <x:c r="C22" s="7"/>
-      <x:c r="D22" s="7"/>
-      <x:c r="E22" s="7"/>
-      <x:c r="F22" s="9"/>
+      <x:c r="D22" s="6"/>
+      <x:c r="E22" s="6"/>
+      <x:c r="F22" s="10"/>
       <x:c r="G22" s="10"/>
-      <x:c r="H22" s="6"/>
-      <x:c r="I22" s="10"/>
+      <x:c r="H22" s="10"/>
+      <x:c r="I22" s="6"/>
       <x:c r="J22" s="10"/>
       <x:c r="K22" s="10"/>
       <x:c r="L22" s="10"/>
-      <x:c r="M22" s="7"/>
+      <x:c r="M22" s="10"/>
+      <x:c r="N22" s="10"/>
+      <x:c r="O22" s="10"/>
+      <x:c r="P22" s="10"/>
+      <x:c r="Q22" s="10"/>
+      <x:c r="R22" s="6"/>
+      <x:c r="S22" s="6"/>
+      <x:c r="T22" s="6"/>
+      <x:c r="U22" s="6"/>
+      <x:c r="V22" s="6"/>
+      <x:c r="W22" s="7"/>
+      <x:c r="X22" s="7"/>
+      <x:c r="Y22" s="9"/>
+      <x:c r="Z22" s="10"/>
+      <x:c r="AA22" s="6"/>
+      <x:c r="AB22" s="10"/>
+      <x:c r="AC22" s="10"/>
+      <x:c r="AD22" s="10"/>
+      <x:c r="AE22" s="10"/>
+      <x:c r="AF22" s="7"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7"/>
       <x:c r="B23" s="7"/>
       <x:c r="C23" s="7"/>
-      <x:c r="D23" s="7"/>
-      <x:c r="E23" s="7"/>
-      <x:c r="F23" s="9"/>
+      <x:c r="D23" s="6"/>
+      <x:c r="E23" s="6"/>
+      <x:c r="F23" s="10"/>
       <x:c r="G23" s="10"/>
-      <x:c r="H23" s="6"/>
-      <x:c r="I23" s="10"/>
+      <x:c r="H23" s="10"/>
+      <x:c r="I23" s="6"/>
       <x:c r="J23" s="10"/>
       <x:c r="K23" s="10"/>
       <x:c r="L23" s="10"/>
-      <x:c r="M23" s="7"/>
+      <x:c r="M23" s="10"/>
+      <x:c r="N23" s="10"/>
+      <x:c r="O23" s="10"/>
+      <x:c r="P23" s="10"/>
+      <x:c r="Q23" s="10"/>
+      <x:c r="R23" s="6"/>
+      <x:c r="S23" s="6"/>
+      <x:c r="T23" s="6"/>
+      <x:c r="U23" s="6"/>
+      <x:c r="V23" s="6"/>
+      <x:c r="W23" s="7"/>
+      <x:c r="X23" s="7"/>
+      <x:c r="Y23" s="9"/>
+      <x:c r="Z23" s="10"/>
+      <x:c r="AA23" s="6"/>
+      <x:c r="AB23" s="10"/>
+      <x:c r="AC23" s="10"/>
+      <x:c r="AD23" s="10"/>
+      <x:c r="AE23" s="10"/>
+      <x:c r="AF23" s="7"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7"/>
       <x:c r="B24" s="7"/>
       <x:c r="C24" s="7"/>
-      <x:c r="D24" s="7"/>
-      <x:c r="E24" s="7"/>
-      <x:c r="F24" s="9"/>
+      <x:c r="D24" s="6"/>
+      <x:c r="E24" s="6"/>
+      <x:c r="F24" s="10"/>
       <x:c r="G24" s="10"/>
-      <x:c r="H24" s="6"/>
-      <x:c r="I24" s="10"/>
+      <x:c r="H24" s="10"/>
+      <x:c r="I24" s="6"/>
       <x:c r="J24" s="10"/>
       <x:c r="K24" s="10"/>
       <x:c r="L24" s="10"/>
-      <x:c r="M24" s="7"/>
+      <x:c r="M24" s="10"/>
+      <x:c r="N24" s="10"/>
+      <x:c r="O24" s="10"/>
+      <x:c r="P24" s="10"/>
+      <x:c r="Q24" s="10"/>
+      <x:c r="R24" s="6"/>
+      <x:c r="S24" s="6"/>
+      <x:c r="T24" s="6"/>
+      <x:c r="U24" s="6"/>
+      <x:c r="V24" s="6"/>
+      <x:c r="W24" s="7"/>
+      <x:c r="X24" s="7"/>
+      <x:c r="Y24" s="9"/>
+      <x:c r="Z24" s="10"/>
+      <x:c r="AA24" s="6"/>
+      <x:c r="AB24" s="10"/>
+      <x:c r="AC24" s="10"/>
+      <x:c r="AD24" s="10"/>
+      <x:c r="AE24" s="10"/>
+      <x:c r="AF24" s="7"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="E5:E24">
+      <x:formula1>"Sí,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I24">
+      <x:formula1>"A,B,C"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Reglas de vidrio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
+      <x:c r="A4" s="5" t="str">
+        <x:v>Código de regla</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>Nombre</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Zona de riesgo</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>Antepecho de referencia (mm)</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Área de referencia (m²)</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="str">
+        <x:v>Clases admitidas separadas por |</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Obligatoria</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>Ejemplo sintético</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="7"/>
+      <x:c r="B5" s="7"/>
+      <x:c r="C5" s="7"/>
+      <x:c r="D5" s="10"/>
+      <x:c r="E5" s="10"/>
+      <x:c r="F5" s="7"/>
+      <x:c r="G5" s="7"/>
+      <x:c r="H5" s="7"/>
+      <x:c r="I5" s="7"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="7"/>
+      <x:c r="B6" s="7"/>
+      <x:c r="C6" s="7"/>
+      <x:c r="D6" s="10"/>
+      <x:c r="E6" s="10"/>
+      <x:c r="F6" s="7"/>
+      <x:c r="G6" s="7"/>
+      <x:c r="H6" s="7"/>
+      <x:c r="I6" s="7"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="7"/>
+      <x:c r="B7" s="7"/>
+      <x:c r="C7" s="7"/>
+      <x:c r="D7" s="10"/>
+      <x:c r="E7" s="10"/>
+      <x:c r="F7" s="7"/>
+      <x:c r="G7" s="7"/>
+      <x:c r="H7" s="7"/>
+      <x:c r="I7" s="7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="7"/>
+      <x:c r="B8" s="7"/>
+      <x:c r="C8" s="7"/>
+      <x:c r="D8" s="10"/>
+      <x:c r="E8" s="10"/>
+      <x:c r="F8" s="7"/>
+      <x:c r="G8" s="7"/>
+      <x:c r="H8" s="7"/>
+      <x:c r="I8" s="7"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="7"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="7"/>
+      <x:c r="D9" s="10"/>
+      <x:c r="E9" s="10"/>
+      <x:c r="F9" s="7"/>
+      <x:c r="G9" s="7"/>
+      <x:c r="H9" s="7"/>
+      <x:c r="I9" s="7"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="7"/>
+      <x:c r="B10" s="7"/>
+      <x:c r="C10" s="7"/>
+      <x:c r="D10" s="10"/>
+      <x:c r="E10" s="10"/>
+      <x:c r="F10" s="7"/>
+      <x:c r="G10" s="7"/>
+      <x:c r="H10" s="7"/>
+      <x:c r="I10" s="7"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="7"/>
+      <x:c r="B11" s="7"/>
+      <x:c r="C11" s="7"/>
+      <x:c r="D11" s="10"/>
+      <x:c r="E11" s="10"/>
+      <x:c r="F11" s="7"/>
+      <x:c r="G11" s="7"/>
+      <x:c r="H11" s="7"/>
+      <x:c r="I11" s="7"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="7"/>
+      <x:c r="B12" s="7"/>
+      <x:c r="C12" s="7"/>
+      <x:c r="D12" s="10"/>
+      <x:c r="E12" s="10"/>
+      <x:c r="F12" s="7"/>
+      <x:c r="G12" s="7"/>
+      <x:c r="H12" s="7"/>
+      <x:c r="I12" s="7"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="7"/>
+      <x:c r="B13" s="7"/>
+      <x:c r="C13" s="7"/>
+      <x:c r="D13" s="10"/>
+      <x:c r="E13" s="10"/>
+      <x:c r="F13" s="7"/>
+      <x:c r="G13" s="7"/>
+      <x:c r="H13" s="7"/>
+      <x:c r="I13" s="7"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7"/>
+      <x:c r="B14" s="7"/>
+      <x:c r="C14" s="7"/>
+      <x:c r="D14" s="10"/>
+      <x:c r="E14" s="10"/>
+      <x:c r="F14" s="7"/>
+      <x:c r="G14" s="7"/>
+      <x:c r="H14" s="7"/>
+      <x:c r="I14" s="7"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="7"/>
+      <x:c r="B15" s="7"/>
+      <x:c r="C15" s="7"/>
+      <x:c r="D15" s="10"/>
+      <x:c r="E15" s="10"/>
+      <x:c r="F15" s="7"/>
+      <x:c r="G15" s="7"/>
+      <x:c r="H15" s="7"/>
+      <x:c r="I15" s="7"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="7"/>
+      <x:c r="B16" s="7"/>
+      <x:c r="C16" s="7"/>
+      <x:c r="D16" s="10"/>
+      <x:c r="E16" s="10"/>
+      <x:c r="F16" s="7"/>
+      <x:c r="G16" s="7"/>
+      <x:c r="H16" s="7"/>
+      <x:c r="I16" s="7"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="7"/>
+      <x:c r="B17" s="7"/>
+      <x:c r="C17" s="7"/>
+      <x:c r="D17" s="10"/>
+      <x:c r="E17" s="10"/>
+      <x:c r="F17" s="7"/>
+      <x:c r="G17" s="7"/>
+      <x:c r="H17" s="7"/>
+      <x:c r="I17" s="7"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="7"/>
+      <x:c r="B18" s="7"/>
+      <x:c r="C18" s="7"/>
+      <x:c r="D18" s="10"/>
+      <x:c r="E18" s="10"/>
+      <x:c r="F18" s="7"/>
+      <x:c r="G18" s="7"/>
+      <x:c r="H18" s="7"/>
+      <x:c r="I18" s="7"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="7"/>
+      <x:c r="B19" s="7"/>
+      <x:c r="C19" s="7"/>
+      <x:c r="D19" s="10"/>
+      <x:c r="E19" s="10"/>
+      <x:c r="F19" s="7"/>
+      <x:c r="G19" s="7"/>
+      <x:c r="H19" s="7"/>
+      <x:c r="I19" s="7"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="7"/>
+      <x:c r="B20" s="7"/>
+      <x:c r="C20" s="7"/>
+      <x:c r="D20" s="10"/>
+      <x:c r="E20" s="10"/>
+      <x:c r="F20" s="7"/>
+      <x:c r="G20" s="7"/>
+      <x:c r="H20" s="7"/>
+      <x:c r="I20" s="7"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="7"/>
+      <x:c r="B21" s="7"/>
+      <x:c r="C21" s="7"/>
+      <x:c r="D21" s="10"/>
+      <x:c r="E21" s="10"/>
+      <x:c r="F21" s="7"/>
+      <x:c r="G21" s="7"/>
+      <x:c r="H21" s="7"/>
+      <x:c r="I21" s="7"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="7"/>
+      <x:c r="B22" s="7"/>
+      <x:c r="C22" s="7"/>
+      <x:c r="D22" s="10"/>
+      <x:c r="E22" s="10"/>
+      <x:c r="F22" s="7"/>
+      <x:c r="G22" s="7"/>
+      <x:c r="H22" s="7"/>
+      <x:c r="I22" s="7"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="7"/>
+      <x:c r="B23" s="7"/>
+      <x:c r="C23" s="7"/>
+      <x:c r="D23" s="10"/>
+      <x:c r="E23" s="10"/>
+      <x:c r="F23" s="7"/>
+      <x:c r="G23" s="7"/>
+      <x:c r="H23" s="7"/>
+      <x:c r="I23" s="7"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="7"/>
+      <x:c r="B24" s="7"/>
+      <x:c r="C24" s="7"/>
+      <x:c r="D24" s="10"/>
+      <x:c r="E24" s="10"/>
+      <x:c r="F24" s="7"/>
+      <x:c r="G24" s="7"/>
+      <x:c r="H24" s="7"/>
+      <x:c r="I24" s="7"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="C5:C24">
+      <x:formula1>"Puerta,Panel lateral,Paño bajo,Gran ventanal"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G5:G24">
+      <x:formula1>"Sí,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H5:H24">
+      <x:formula1>"Sí,No"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3490,342 +4583,4 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>Precios de costo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="2" t="str">
-        <x:v>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="48" customHeight="1">
-      <x:c r="A4" s="5" t="str">
-        <x:v>Código de sistema</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>SKU</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>Lista de costo</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="str">
-        <x:v>Proveedor</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="str">
-        <x:v>Moneda</x:v>
-      </x:c>
-      <x:c r="F4" s="5" t="str">
-        <x:v>Vigente desde (aaaa-mm-dd)</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="str">
-        <x:v>Vigente hasta (aaaa-mm-dd)</x:v>
-      </x:c>
-      <x:c r="H4" s="5" t="str">
-        <x:v>Tipo de artículo</x:v>
-      </x:c>
-      <x:c r="I4" s="5" t="str">
-        <x:v>Unidad</x:v>
-      </x:c>
-      <x:c r="J4" s="5" t="str">
-        <x:v>Costo unitario</x:v>
-      </x:c>
-      <x:c r="K4" s="5" t="str">
-        <x:v>Fuente</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="7"/>
-      <x:c r="B5" s="7"/>
-      <x:c r="C5" s="7"/>
-      <x:c r="D5" s="7"/>
-      <x:c r="E5" s="7"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="13"/>
-      <x:c r="H5" s="7"/>
-      <x:c r="I5" s="7"/>
-      <x:c r="J5" s="8"/>
-      <x:c r="K5" s="7"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="7"/>
-      <x:c r="B6" s="7"/>
-      <x:c r="C6" s="7"/>
-      <x:c r="D6" s="7"/>
-      <x:c r="E6" s="7"/>
-      <x:c r="F6" s="12"/>
-      <x:c r="G6" s="13"/>
-      <x:c r="H6" s="7"/>
-      <x:c r="I6" s="7"/>
-      <x:c r="J6" s="8"/>
-      <x:c r="K6" s="7"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="7"/>
-      <x:c r="B7" s="7"/>
-      <x:c r="C7" s="7"/>
-      <x:c r="D7" s="7"/>
-      <x:c r="E7" s="7"/>
-      <x:c r="F7" s="12"/>
-      <x:c r="G7" s="13"/>
-      <x:c r="H7" s="7"/>
-      <x:c r="I7" s="7"/>
-      <x:c r="J7" s="8"/>
-      <x:c r="K7" s="7"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7"/>
-      <x:c r="C8" s="7"/>
-      <x:c r="D8" s="7"/>
-      <x:c r="E8" s="7"/>
-      <x:c r="F8" s="12"/>
-      <x:c r="G8" s="13"/>
-      <x:c r="H8" s="7"/>
-      <x:c r="I8" s="7"/>
-      <x:c r="J8" s="8"/>
-      <x:c r="K8" s="7"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="7"/>
-      <x:c r="B9" s="7"/>
-      <x:c r="C9" s="7"/>
-      <x:c r="D9" s="7"/>
-      <x:c r="E9" s="7"/>
-      <x:c r="F9" s="12"/>
-      <x:c r="G9" s="13"/>
-      <x:c r="H9" s="7"/>
-      <x:c r="I9" s="7"/>
-      <x:c r="J9" s="8"/>
-      <x:c r="K9" s="7"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="7"/>
-      <x:c r="B10" s="7"/>
-      <x:c r="C10" s="7"/>
-      <x:c r="D10" s="7"/>
-      <x:c r="E10" s="7"/>
-      <x:c r="F10" s="12"/>
-      <x:c r="G10" s="13"/>
-      <x:c r="H10" s="7"/>
-      <x:c r="I10" s="7"/>
-      <x:c r="J10" s="8"/>
-      <x:c r="K10" s="7"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="7"/>
-      <x:c r="B11" s="7"/>
-      <x:c r="C11" s="7"/>
-      <x:c r="D11" s="7"/>
-      <x:c r="E11" s="7"/>
-      <x:c r="F11" s="12"/>
-      <x:c r="G11" s="13"/>
-      <x:c r="H11" s="7"/>
-      <x:c r="I11" s="7"/>
-      <x:c r="J11" s="8"/>
-      <x:c r="K11" s="7"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="7"/>
-      <x:c r="B12" s="7"/>
-      <x:c r="C12" s="7"/>
-      <x:c r="D12" s="7"/>
-      <x:c r="E12" s="7"/>
-      <x:c r="F12" s="12"/>
-      <x:c r="G12" s="13"/>
-      <x:c r="H12" s="7"/>
-      <x:c r="I12" s="7"/>
-      <x:c r="J12" s="8"/>
-      <x:c r="K12" s="7"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="7"/>
-      <x:c r="B13" s="7"/>
-      <x:c r="C13" s="7"/>
-      <x:c r="D13" s="7"/>
-      <x:c r="E13" s="7"/>
-      <x:c r="F13" s="12"/>
-      <x:c r="G13" s="13"/>
-      <x:c r="H13" s="7"/>
-      <x:c r="I13" s="7"/>
-      <x:c r="J13" s="8"/>
-      <x:c r="K13" s="7"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="7"/>
-      <x:c r="B14" s="7"/>
-      <x:c r="C14" s="7"/>
-      <x:c r="D14" s="7"/>
-      <x:c r="E14" s="7"/>
-      <x:c r="F14" s="12"/>
-      <x:c r="G14" s="13"/>
-      <x:c r="H14" s="7"/>
-      <x:c r="I14" s="7"/>
-      <x:c r="J14" s="8"/>
-      <x:c r="K14" s="7"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="7"/>
-      <x:c r="B15" s="7"/>
-      <x:c r="C15" s="7"/>
-      <x:c r="D15" s="7"/>
-      <x:c r="E15" s="7"/>
-      <x:c r="F15" s="12"/>
-      <x:c r="G15" s="13"/>
-      <x:c r="H15" s="7"/>
-      <x:c r="I15" s="7"/>
-      <x:c r="J15" s="8"/>
-      <x:c r="K15" s="7"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="7"/>
-      <x:c r="B16" s="7"/>
-      <x:c r="C16" s="7"/>
-      <x:c r="D16" s="7"/>
-      <x:c r="E16" s="7"/>
-      <x:c r="F16" s="12"/>
-      <x:c r="G16" s="13"/>
-      <x:c r="H16" s="7"/>
-      <x:c r="I16" s="7"/>
-      <x:c r="J16" s="8"/>
-      <x:c r="K16" s="7"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="7"/>
-      <x:c r="B17" s="7"/>
-      <x:c r="C17" s="7"/>
-      <x:c r="D17" s="7"/>
-      <x:c r="E17" s="7"/>
-      <x:c r="F17" s="12"/>
-      <x:c r="G17" s="13"/>
-      <x:c r="H17" s="7"/>
-      <x:c r="I17" s="7"/>
-      <x:c r="J17" s="8"/>
-      <x:c r="K17" s="7"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="7"/>
-      <x:c r="B18" s="7"/>
-      <x:c r="C18" s="7"/>
-      <x:c r="D18" s="7"/>
-      <x:c r="E18" s="7"/>
-      <x:c r="F18" s="12"/>
-      <x:c r="G18" s="13"/>
-      <x:c r="H18" s="7"/>
-      <x:c r="I18" s="7"/>
-      <x:c r="J18" s="8"/>
-      <x:c r="K18" s="7"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="7"/>
-      <x:c r="B19" s="7"/>
-      <x:c r="C19" s="7"/>
-      <x:c r="D19" s="7"/>
-      <x:c r="E19" s="7"/>
-      <x:c r="F19" s="12"/>
-      <x:c r="G19" s="13"/>
-      <x:c r="H19" s="7"/>
-      <x:c r="I19" s="7"/>
-      <x:c r="J19" s="8"/>
-      <x:c r="K19" s="7"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="7"/>
-      <x:c r="B20" s="7"/>
-      <x:c r="C20" s="7"/>
-      <x:c r="D20" s="7"/>
-      <x:c r="E20" s="7"/>
-      <x:c r="F20" s="12"/>
-      <x:c r="G20" s="13"/>
-      <x:c r="H20" s="7"/>
-      <x:c r="I20" s="7"/>
-      <x:c r="J20" s="8"/>
-      <x:c r="K20" s="7"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="7"/>
-      <x:c r="B21" s="7"/>
-      <x:c r="C21" s="7"/>
-      <x:c r="D21" s="7"/>
-      <x:c r="E21" s="7"/>
-      <x:c r="F21" s="12"/>
-      <x:c r="G21" s="13"/>
-      <x:c r="H21" s="7"/>
-      <x:c r="I21" s="7"/>
-      <x:c r="J21" s="8"/>
-      <x:c r="K21" s="7"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="7"/>
-      <x:c r="B22" s="7"/>
-      <x:c r="C22" s="7"/>
-      <x:c r="D22" s="7"/>
-      <x:c r="E22" s="7"/>
-      <x:c r="F22" s="12"/>
-      <x:c r="G22" s="13"/>
-      <x:c r="H22" s="7"/>
-      <x:c r="I22" s="7"/>
-      <x:c r="J22" s="8"/>
-      <x:c r="K22" s="7"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="7"/>
-      <x:c r="B23" s="7"/>
-      <x:c r="C23" s="7"/>
-      <x:c r="D23" s="7"/>
-      <x:c r="E23" s="7"/>
-      <x:c r="F23" s="12"/>
-      <x:c r="G23" s="13"/>
-      <x:c r="H23" s="7"/>
-      <x:c r="I23" s="7"/>
-      <x:c r="J23" s="8"/>
-      <x:c r="K23" s="7"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="7"/>
-      <x:c r="B24" s="7"/>
-      <x:c r="C24" s="7"/>
-      <x:c r="D24" s="7"/>
-      <x:c r="E24" s="7"/>
-      <x:c r="F24" s="12"/>
-      <x:c r="G24" s="13"/>
-      <x:c r="H24" s="7"/>
-      <x:c r="I24" s="7"/>
-      <x:c r="J24" s="8"/>
-      <x:c r="K24" s="7"/>
-    </x:row>
-  </x:sheetData>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="E5:E24">
-      <x:formula1>"CLP,USD"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="H5:H24">
-      <x:formula1>"Perfil,Refuerzo,Vidrio,Herraje,Otro"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="I5:I24">
-      <x:formula1>"Barra,Metro,Metro cuadrado,Kit,Unidad"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(vidrios): composición, seguridad y pedidos sellados (#120)
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sistemas" sheetId="1" r:id="R8282c5d1a603453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfiles" sheetId="2" r:id="Rd340470f3e4a4478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles y reglas de corte" sheetId="3" r:id="Rbff0e0ad12b047f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refuerzos" sheetId="4" r:id="Rc4c543501bf34c42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Límites" sheetId="5" r:id="Rf3c66cfdf453469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colores y SKU por color" sheetId="6" r:id="R2c87e79595a24e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="7" r:id="R5ef2f5f5e9bd4ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="8" r:id="Rc4ab87be3d7a42cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="9" r:id="R2260f5d3412b4a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sistemas" sheetId="1" r:id="R30854f96d12d406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfiles" sheetId="2" r:id="R40436b429cea4077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles y reglas de corte" sheetId="3" r:id="R0cd932817b2547dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refuerzos" sheetId="4" r:id="R5a60c4d7d2ee42d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Límites" sheetId="5" r:id="R2135c857c9f24d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colores y SKU por color" sheetId="6" r:id="Rd5c5cb88fcaf45f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="7" r:id="R3452336fba5a4cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas de vidrio" sheetId="8" r:id="R64164b13a3714a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="9" r:id="R17f0a2acee47424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" r:id="R3cf28316dcb84cde"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1142,6 +1143,344 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Precios de costo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
+      <x:c r="A4" s="5" t="str">
+        <x:v>Código de sistema</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>SKU</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Lista de costo</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>Proveedor</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Moneda</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="str">
+        <x:v>Vigente desde (aaaa-mm-dd)</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Vigente hasta (aaaa-mm-dd)</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>Tipo de artículo</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="J4" s="5" t="str">
+        <x:v>Costo unitario</x:v>
+      </x:c>
+      <x:c r="K4" s="5" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="7"/>
+      <x:c r="B5" s="7"/>
+      <x:c r="C5" s="7"/>
+      <x:c r="D5" s="7"/>
+      <x:c r="E5" s="7"/>
+      <x:c r="F5" s="12"/>
+      <x:c r="G5" s="13"/>
+      <x:c r="H5" s="7"/>
+      <x:c r="I5" s="7"/>
+      <x:c r="J5" s="8"/>
+      <x:c r="K5" s="7"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="7"/>
+      <x:c r="B6" s="7"/>
+      <x:c r="C6" s="7"/>
+      <x:c r="D6" s="7"/>
+      <x:c r="E6" s="7"/>
+      <x:c r="F6" s="12"/>
+      <x:c r="G6" s="13"/>
+      <x:c r="H6" s="7"/>
+      <x:c r="I6" s="7"/>
+      <x:c r="J6" s="8"/>
+      <x:c r="K6" s="7"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="7"/>
+      <x:c r="B7" s="7"/>
+      <x:c r="C7" s="7"/>
+      <x:c r="D7" s="7"/>
+      <x:c r="E7" s="7"/>
+      <x:c r="F7" s="12"/>
+      <x:c r="G7" s="13"/>
+      <x:c r="H7" s="7"/>
+      <x:c r="I7" s="7"/>
+      <x:c r="J7" s="8"/>
+      <x:c r="K7" s="7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="7"/>
+      <x:c r="B8" s="7"/>
+      <x:c r="C8" s="7"/>
+      <x:c r="D8" s="7"/>
+      <x:c r="E8" s="7"/>
+      <x:c r="F8" s="12"/>
+      <x:c r="G8" s="13"/>
+      <x:c r="H8" s="7"/>
+      <x:c r="I8" s="7"/>
+      <x:c r="J8" s="8"/>
+      <x:c r="K8" s="7"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="7"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="7"/>
+      <x:c r="D9" s="7"/>
+      <x:c r="E9" s="7"/>
+      <x:c r="F9" s="12"/>
+      <x:c r="G9" s="13"/>
+      <x:c r="H9" s="7"/>
+      <x:c r="I9" s="7"/>
+      <x:c r="J9" s="8"/>
+      <x:c r="K9" s="7"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="7"/>
+      <x:c r="B10" s="7"/>
+      <x:c r="C10" s="7"/>
+      <x:c r="D10" s="7"/>
+      <x:c r="E10" s="7"/>
+      <x:c r="F10" s="12"/>
+      <x:c r="G10" s="13"/>
+      <x:c r="H10" s="7"/>
+      <x:c r="I10" s="7"/>
+      <x:c r="J10" s="8"/>
+      <x:c r="K10" s="7"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="7"/>
+      <x:c r="B11" s="7"/>
+      <x:c r="C11" s="7"/>
+      <x:c r="D11" s="7"/>
+      <x:c r="E11" s="7"/>
+      <x:c r="F11" s="12"/>
+      <x:c r="G11" s="13"/>
+      <x:c r="H11" s="7"/>
+      <x:c r="I11" s="7"/>
+      <x:c r="J11" s="8"/>
+      <x:c r="K11" s="7"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="7"/>
+      <x:c r="B12" s="7"/>
+      <x:c r="C12" s="7"/>
+      <x:c r="D12" s="7"/>
+      <x:c r="E12" s="7"/>
+      <x:c r="F12" s="12"/>
+      <x:c r="G12" s="13"/>
+      <x:c r="H12" s="7"/>
+      <x:c r="I12" s="7"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="7"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="7"/>
+      <x:c r="B13" s="7"/>
+      <x:c r="C13" s="7"/>
+      <x:c r="D13" s="7"/>
+      <x:c r="E13" s="7"/>
+      <x:c r="F13" s="12"/>
+      <x:c r="G13" s="13"/>
+      <x:c r="H13" s="7"/>
+      <x:c r="I13" s="7"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="7"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7"/>
+      <x:c r="B14" s="7"/>
+      <x:c r="C14" s="7"/>
+      <x:c r="D14" s="7"/>
+      <x:c r="E14" s="7"/>
+      <x:c r="F14" s="12"/>
+      <x:c r="G14" s="13"/>
+      <x:c r="H14" s="7"/>
+      <x:c r="I14" s="7"/>
+      <x:c r="J14" s="8"/>
+      <x:c r="K14" s="7"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="7"/>
+      <x:c r="B15" s="7"/>
+      <x:c r="C15" s="7"/>
+      <x:c r="D15" s="7"/>
+      <x:c r="E15" s="7"/>
+      <x:c r="F15" s="12"/>
+      <x:c r="G15" s="13"/>
+      <x:c r="H15" s="7"/>
+      <x:c r="I15" s="7"/>
+      <x:c r="J15" s="8"/>
+      <x:c r="K15" s="7"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="7"/>
+      <x:c r="B16" s="7"/>
+      <x:c r="C16" s="7"/>
+      <x:c r="D16" s="7"/>
+      <x:c r="E16" s="7"/>
+      <x:c r="F16" s="12"/>
+      <x:c r="G16" s="13"/>
+      <x:c r="H16" s="7"/>
+      <x:c r="I16" s="7"/>
+      <x:c r="J16" s="8"/>
+      <x:c r="K16" s="7"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="7"/>
+      <x:c r="B17" s="7"/>
+      <x:c r="C17" s="7"/>
+      <x:c r="D17" s="7"/>
+      <x:c r="E17" s="7"/>
+      <x:c r="F17" s="12"/>
+      <x:c r="G17" s="13"/>
+      <x:c r="H17" s="7"/>
+      <x:c r="I17" s="7"/>
+      <x:c r="J17" s="8"/>
+      <x:c r="K17" s="7"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="7"/>
+      <x:c r="B18" s="7"/>
+      <x:c r="C18" s="7"/>
+      <x:c r="D18" s="7"/>
+      <x:c r="E18" s="7"/>
+      <x:c r="F18" s="12"/>
+      <x:c r="G18" s="13"/>
+      <x:c r="H18" s="7"/>
+      <x:c r="I18" s="7"/>
+      <x:c r="J18" s="8"/>
+      <x:c r="K18" s="7"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="7"/>
+      <x:c r="B19" s="7"/>
+      <x:c r="C19" s="7"/>
+      <x:c r="D19" s="7"/>
+      <x:c r="E19" s="7"/>
+      <x:c r="F19" s="12"/>
+      <x:c r="G19" s="13"/>
+      <x:c r="H19" s="7"/>
+      <x:c r="I19" s="7"/>
+      <x:c r="J19" s="8"/>
+      <x:c r="K19" s="7"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="7"/>
+      <x:c r="B20" s="7"/>
+      <x:c r="C20" s="7"/>
+      <x:c r="D20" s="7"/>
+      <x:c r="E20" s="7"/>
+      <x:c r="F20" s="12"/>
+      <x:c r="G20" s="13"/>
+      <x:c r="H20" s="7"/>
+      <x:c r="I20" s="7"/>
+      <x:c r="J20" s="8"/>
+      <x:c r="K20" s="7"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="7"/>
+      <x:c r="B21" s="7"/>
+      <x:c r="C21" s="7"/>
+      <x:c r="D21" s="7"/>
+      <x:c r="E21" s="7"/>
+      <x:c r="F21" s="12"/>
+      <x:c r="G21" s="13"/>
+      <x:c r="H21" s="7"/>
+      <x:c r="I21" s="7"/>
+      <x:c r="J21" s="8"/>
+      <x:c r="K21" s="7"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="7"/>
+      <x:c r="B22" s="7"/>
+      <x:c r="C22" s="7"/>
+      <x:c r="D22" s="7"/>
+      <x:c r="E22" s="7"/>
+      <x:c r="F22" s="12"/>
+      <x:c r="G22" s="13"/>
+      <x:c r="H22" s="7"/>
+      <x:c r="I22" s="7"/>
+      <x:c r="J22" s="8"/>
+      <x:c r="K22" s="7"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="7"/>
+      <x:c r="B23" s="7"/>
+      <x:c r="C23" s="7"/>
+      <x:c r="D23" s="7"/>
+      <x:c r="E23" s="7"/>
+      <x:c r="F23" s="12"/>
+      <x:c r="G23" s="13"/>
+      <x:c r="H23" s="7"/>
+      <x:c r="I23" s="7"/>
+      <x:c r="J23" s="8"/>
+      <x:c r="K23" s="7"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="7"/>
+      <x:c r="B24" s="7"/>
+      <x:c r="C24" s="7"/>
+      <x:c r="D24" s="7"/>
+      <x:c r="E24" s="7"/>
+      <x:c r="F24" s="12"/>
+      <x:c r="G24" s="13"/>
+      <x:c r="H24" s="7"/>
+      <x:c r="I24" s="7"/>
+      <x:c r="J24" s="8"/>
+      <x:c r="K24" s="7"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="E5:E24">
+      <x:formula1>"CLP,USD"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H5:H24">
+      <x:formula1>"Perfil,Refuerzo,Vidrio,Herraje,Otro"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I24">
+      <x:formula1>"Barra,Metro,Metro cuadrado,Kit,Unidad"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -2646,12 +2985,31 @@
     <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="22" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="22" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="22" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="22" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="30" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="22" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="22" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="22" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="22" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="30" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2675,33 +3033,90 @@
         <x:v>Composición de vidrio</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
+        <x:v>Nombre comercial</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Ejemplo sintético</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="str">
+        <x:v>Ug de proveedor (W/m²K)</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Factor solar g de proveedor</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>Transmisión luminosa de proveedor</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Clase NCh 135 de proveedor</x:v>
+      </x:c>
+      <x:c r="J4" s="5" t="str">
+        <x:v>Peso declarado de proveedor (kg/m²)</x:v>
+      </x:c>
+      <x:c r="K4" s="5" t="str">
+        <x:v>Área mínima facturable (m²)</x:v>
+      </x:c>
+      <x:c r="L4" s="5" t="str">
+        <x:v>Ancho mínimo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="M4" s="5" t="str">
+        <x:v>Ancho máximo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="N4" s="5" t="str">
+        <x:v>Alto mínimo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="O4" s="5" t="str">
+        <x:v>Alto máximo de vidrio (mm)</x:v>
+      </x:c>
+      <x:c r="P4" s="5" t="str">
+        <x:v>Área máxima de vidrio (m²)</x:v>
+      </x:c>
+      <x:c r="Q4" s="5" t="str">
+        <x:v>Relación de aspecto máxima de vidrio</x:v>
+      </x:c>
+      <x:c r="R4" s="5" t="str">
+        <x:v>SKU recargo templado</x:v>
+      </x:c>
+      <x:c r="S4" s="5" t="str">
+        <x:v>SKU recargo pulido</x:v>
+      </x:c>
+      <x:c r="T4" s="5" t="str">
+        <x:v>SKU recargo perforación</x:v>
+      </x:c>
+      <x:c r="U4" s="5" t="str">
+        <x:v>SKU palillaje por metro</x:v>
+      </x:c>
+      <x:c r="V4" s="5" t="str">
+        <x:v>SKU palillaje por cruce</x:v>
+      </x:c>
+      <x:c r="W4" s="5" t="str">
         <x:v>SKU de compra</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="str">
+      <x:c r="X4" s="5" t="str">
         <x:v>Fabricante</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="str">
+      <x:c r="Y4" s="5" t="str">
         <x:v>Versión</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="str">
+      <x:c r="Z4" s="5" t="str">
         <x:v>Espesor para junquillo (mm)</x:v>
       </x:c>
-      <x:c r="H4" s="5" t="str">
+      <x:c r="AA4" s="5" t="str">
         <x:v>SKU de junquillo</x:v>
       </x:c>
-      <x:c r="I4" s="5" t="str">
+      <x:c r="AB4" s="5" t="str">
         <x:v>Ancho de junquillo (mm)</x:v>
       </x:c>
-      <x:c r="J4" s="5" t="str">
+      <x:c r="AC4" s="5" t="str">
         <x:v>Junta interior (mm)</x:v>
       </x:c>
-      <x:c r="K4" s="5" t="str">
+      <x:c r="AD4" s="5" t="str">
         <x:v>Junta exterior (mm)</x:v>
       </x:c>
-      <x:c r="L4" s="5" t="str">
+      <x:c r="AE4" s="5" t="str">
         <x:v>Adición al corte de junquillo (mm)</x:v>
       </x:c>
-      <x:c r="M4" s="5" t="str">
+      <x:c r="AF4" s="5" t="str">
         <x:v>Fuente</x:v>
       </x:c>
     </x:row>
@@ -2709,308 +3124,986 @@
       <x:c r="A5" s="7"/>
       <x:c r="B5" s="7"/>
       <x:c r="C5" s="7"/>
-      <x:c r="D5" s="7"/>
-      <x:c r="E5" s="7"/>
-      <x:c r="F5" s="9"/>
+      <x:c r="D5" s="6"/>
+      <x:c r="E5" s="6"/>
+      <x:c r="F5" s="10"/>
       <x:c r="G5" s="10"/>
-      <x:c r="H5" s="6"/>
-      <x:c r="I5" s="10"/>
+      <x:c r="H5" s="10"/>
+      <x:c r="I5" s="6"/>
       <x:c r="J5" s="10"/>
       <x:c r="K5" s="10"/>
       <x:c r="L5" s="10"/>
-      <x:c r="M5" s="7"/>
+      <x:c r="M5" s="10"/>
+      <x:c r="N5" s="10"/>
+      <x:c r="O5" s="10"/>
+      <x:c r="P5" s="10"/>
+      <x:c r="Q5" s="10"/>
+      <x:c r="R5" s="6"/>
+      <x:c r="S5" s="6"/>
+      <x:c r="T5" s="6"/>
+      <x:c r="U5" s="6"/>
+      <x:c r="V5" s="6"/>
+      <x:c r="W5" s="7"/>
+      <x:c r="X5" s="7"/>
+      <x:c r="Y5" s="9"/>
+      <x:c r="Z5" s="10"/>
+      <x:c r="AA5" s="6"/>
+      <x:c r="AB5" s="10"/>
+      <x:c r="AC5" s="10"/>
+      <x:c r="AD5" s="10"/>
+      <x:c r="AE5" s="10"/>
+      <x:c r="AF5" s="7"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7"/>
       <x:c r="B6" s="7"/>
       <x:c r="C6" s="7"/>
-      <x:c r="D6" s="7"/>
-      <x:c r="E6" s="7"/>
-      <x:c r="F6" s="9"/>
+      <x:c r="D6" s="6"/>
+      <x:c r="E6" s="6"/>
+      <x:c r="F6" s="10"/>
       <x:c r="G6" s="10"/>
-      <x:c r="H6" s="6"/>
-      <x:c r="I6" s="10"/>
+      <x:c r="H6" s="10"/>
+      <x:c r="I6" s="6"/>
       <x:c r="J6" s="10"/>
       <x:c r="K6" s="10"/>
       <x:c r="L6" s="10"/>
-      <x:c r="M6" s="7"/>
+      <x:c r="M6" s="10"/>
+      <x:c r="N6" s="10"/>
+      <x:c r="O6" s="10"/>
+      <x:c r="P6" s="10"/>
+      <x:c r="Q6" s="10"/>
+      <x:c r="R6" s="6"/>
+      <x:c r="S6" s="6"/>
+      <x:c r="T6" s="6"/>
+      <x:c r="U6" s="6"/>
+      <x:c r="V6" s="6"/>
+      <x:c r="W6" s="7"/>
+      <x:c r="X6" s="7"/>
+      <x:c r="Y6" s="9"/>
+      <x:c r="Z6" s="10"/>
+      <x:c r="AA6" s="6"/>
+      <x:c r="AB6" s="10"/>
+      <x:c r="AC6" s="10"/>
+      <x:c r="AD6" s="10"/>
+      <x:c r="AE6" s="10"/>
+      <x:c r="AF6" s="7"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7"/>
       <x:c r="B7" s="7"/>
       <x:c r="C7" s="7"/>
-      <x:c r="D7" s="7"/>
-      <x:c r="E7" s="7"/>
-      <x:c r="F7" s="9"/>
+      <x:c r="D7" s="6"/>
+      <x:c r="E7" s="6"/>
+      <x:c r="F7" s="10"/>
       <x:c r="G7" s="10"/>
-      <x:c r="H7" s="6"/>
-      <x:c r="I7" s="10"/>
+      <x:c r="H7" s="10"/>
+      <x:c r="I7" s="6"/>
       <x:c r="J7" s="10"/>
       <x:c r="K7" s="10"/>
       <x:c r="L7" s="10"/>
-      <x:c r="M7" s="7"/>
+      <x:c r="M7" s="10"/>
+      <x:c r="N7" s="10"/>
+      <x:c r="O7" s="10"/>
+      <x:c r="P7" s="10"/>
+      <x:c r="Q7" s="10"/>
+      <x:c r="R7" s="6"/>
+      <x:c r="S7" s="6"/>
+      <x:c r="T7" s="6"/>
+      <x:c r="U7" s="6"/>
+      <x:c r="V7" s="6"/>
+      <x:c r="W7" s="7"/>
+      <x:c r="X7" s="7"/>
+      <x:c r="Y7" s="9"/>
+      <x:c r="Z7" s="10"/>
+      <x:c r="AA7" s="6"/>
+      <x:c r="AB7" s="10"/>
+      <x:c r="AC7" s="10"/>
+      <x:c r="AD7" s="10"/>
+      <x:c r="AE7" s="10"/>
+      <x:c r="AF7" s="7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7"/>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
-      <x:c r="D8" s="7"/>
-      <x:c r="E8" s="7"/>
-      <x:c r="F8" s="9"/>
+      <x:c r="D8" s="6"/>
+      <x:c r="E8" s="6"/>
+      <x:c r="F8" s="10"/>
       <x:c r="G8" s="10"/>
-      <x:c r="H8" s="6"/>
-      <x:c r="I8" s="10"/>
+      <x:c r="H8" s="10"/>
+      <x:c r="I8" s="6"/>
       <x:c r="J8" s="10"/>
       <x:c r="K8" s="10"/>
       <x:c r="L8" s="10"/>
-      <x:c r="M8" s="7"/>
+      <x:c r="M8" s="10"/>
+      <x:c r="N8" s="10"/>
+      <x:c r="O8" s="10"/>
+      <x:c r="P8" s="10"/>
+      <x:c r="Q8" s="10"/>
+      <x:c r="R8" s="6"/>
+      <x:c r="S8" s="6"/>
+      <x:c r="T8" s="6"/>
+      <x:c r="U8" s="6"/>
+      <x:c r="V8" s="6"/>
+      <x:c r="W8" s="7"/>
+      <x:c r="X8" s="7"/>
+      <x:c r="Y8" s="9"/>
+      <x:c r="Z8" s="10"/>
+      <x:c r="AA8" s="6"/>
+      <x:c r="AB8" s="10"/>
+      <x:c r="AC8" s="10"/>
+      <x:c r="AD8" s="10"/>
+      <x:c r="AE8" s="10"/>
+      <x:c r="AF8" s="7"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7"/>
       <x:c r="B9" s="7"/>
       <x:c r="C9" s="7"/>
-      <x:c r="D9" s="7"/>
-      <x:c r="E9" s="7"/>
-      <x:c r="F9" s="9"/>
+      <x:c r="D9" s="6"/>
+      <x:c r="E9" s="6"/>
+      <x:c r="F9" s="10"/>
       <x:c r="G9" s="10"/>
-      <x:c r="H9" s="6"/>
-      <x:c r="I9" s="10"/>
+      <x:c r="H9" s="10"/>
+      <x:c r="I9" s="6"/>
       <x:c r="J9" s="10"/>
       <x:c r="K9" s="10"/>
       <x:c r="L9" s="10"/>
-      <x:c r="M9" s="7"/>
+      <x:c r="M9" s="10"/>
+      <x:c r="N9" s="10"/>
+      <x:c r="O9" s="10"/>
+      <x:c r="P9" s="10"/>
+      <x:c r="Q9" s="10"/>
+      <x:c r="R9" s="6"/>
+      <x:c r="S9" s="6"/>
+      <x:c r="T9" s="6"/>
+      <x:c r="U9" s="6"/>
+      <x:c r="V9" s="6"/>
+      <x:c r="W9" s="7"/>
+      <x:c r="X9" s="7"/>
+      <x:c r="Y9" s="9"/>
+      <x:c r="Z9" s="10"/>
+      <x:c r="AA9" s="6"/>
+      <x:c r="AB9" s="10"/>
+      <x:c r="AC9" s="10"/>
+      <x:c r="AD9" s="10"/>
+      <x:c r="AE9" s="10"/>
+      <x:c r="AF9" s="7"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7"/>
       <x:c r="B10" s="7"/>
       <x:c r="C10" s="7"/>
-      <x:c r="D10" s="7"/>
-      <x:c r="E10" s="7"/>
-      <x:c r="F10" s="9"/>
+      <x:c r="D10" s="6"/>
+      <x:c r="E10" s="6"/>
+      <x:c r="F10" s="10"/>
       <x:c r="G10" s="10"/>
-      <x:c r="H10" s="6"/>
-      <x:c r="I10" s="10"/>
+      <x:c r="H10" s="10"/>
+      <x:c r="I10" s="6"/>
       <x:c r="J10" s="10"/>
       <x:c r="K10" s="10"/>
       <x:c r="L10" s="10"/>
-      <x:c r="M10" s="7"/>
+      <x:c r="M10" s="10"/>
+      <x:c r="N10" s="10"/>
+      <x:c r="O10" s="10"/>
+      <x:c r="P10" s="10"/>
+      <x:c r="Q10" s="10"/>
+      <x:c r="R10" s="6"/>
+      <x:c r="S10" s="6"/>
+      <x:c r="T10" s="6"/>
+      <x:c r="U10" s="6"/>
+      <x:c r="V10" s="6"/>
+      <x:c r="W10" s="7"/>
+      <x:c r="X10" s="7"/>
+      <x:c r="Y10" s="9"/>
+      <x:c r="Z10" s="10"/>
+      <x:c r="AA10" s="6"/>
+      <x:c r="AB10" s="10"/>
+      <x:c r="AC10" s="10"/>
+      <x:c r="AD10" s="10"/>
+      <x:c r="AE10" s="10"/>
+      <x:c r="AF10" s="7"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7"/>
       <x:c r="B11" s="7"/>
       <x:c r="C11" s="7"/>
-      <x:c r="D11" s="7"/>
-      <x:c r="E11" s="7"/>
-      <x:c r="F11" s="9"/>
+      <x:c r="D11" s="6"/>
+      <x:c r="E11" s="6"/>
+      <x:c r="F11" s="10"/>
       <x:c r="G11" s="10"/>
-      <x:c r="H11" s="6"/>
-      <x:c r="I11" s="10"/>
+      <x:c r="H11" s="10"/>
+      <x:c r="I11" s="6"/>
       <x:c r="J11" s="10"/>
       <x:c r="K11" s="10"/>
       <x:c r="L11" s="10"/>
-      <x:c r="M11" s="7"/>
+      <x:c r="M11" s="10"/>
+      <x:c r="N11" s="10"/>
+      <x:c r="O11" s="10"/>
+      <x:c r="P11" s="10"/>
+      <x:c r="Q11" s="10"/>
+      <x:c r="R11" s="6"/>
+      <x:c r="S11" s="6"/>
+      <x:c r="T11" s="6"/>
+      <x:c r="U11" s="6"/>
+      <x:c r="V11" s="6"/>
+      <x:c r="W11" s="7"/>
+      <x:c r="X11" s="7"/>
+      <x:c r="Y11" s="9"/>
+      <x:c r="Z11" s="10"/>
+      <x:c r="AA11" s="6"/>
+      <x:c r="AB11" s="10"/>
+      <x:c r="AC11" s="10"/>
+      <x:c r="AD11" s="10"/>
+      <x:c r="AE11" s="10"/>
+      <x:c r="AF11" s="7"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7"/>
       <x:c r="B12" s="7"/>
       <x:c r="C12" s="7"/>
-      <x:c r="D12" s="7"/>
-      <x:c r="E12" s="7"/>
-      <x:c r="F12" s="9"/>
+      <x:c r="D12" s="6"/>
+      <x:c r="E12" s="6"/>
+      <x:c r="F12" s="10"/>
       <x:c r="G12" s="10"/>
-      <x:c r="H12" s="6"/>
-      <x:c r="I12" s="10"/>
+      <x:c r="H12" s="10"/>
+      <x:c r="I12" s="6"/>
       <x:c r="J12" s="10"/>
       <x:c r="K12" s="10"/>
       <x:c r="L12" s="10"/>
-      <x:c r="M12" s="7"/>
+      <x:c r="M12" s="10"/>
+      <x:c r="N12" s="10"/>
+      <x:c r="O12" s="10"/>
+      <x:c r="P12" s="10"/>
+      <x:c r="Q12" s="10"/>
+      <x:c r="R12" s="6"/>
+      <x:c r="S12" s="6"/>
+      <x:c r="T12" s="6"/>
+      <x:c r="U12" s="6"/>
+      <x:c r="V12" s="6"/>
+      <x:c r="W12" s="7"/>
+      <x:c r="X12" s="7"/>
+      <x:c r="Y12" s="9"/>
+      <x:c r="Z12" s="10"/>
+      <x:c r="AA12" s="6"/>
+      <x:c r="AB12" s="10"/>
+      <x:c r="AC12" s="10"/>
+      <x:c r="AD12" s="10"/>
+      <x:c r="AE12" s="10"/>
+      <x:c r="AF12" s="7"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7"/>
       <x:c r="B13" s="7"/>
       <x:c r="C13" s="7"/>
-      <x:c r="D13" s="7"/>
-      <x:c r="E13" s="7"/>
-      <x:c r="F13" s="9"/>
+      <x:c r="D13" s="6"/>
+      <x:c r="E13" s="6"/>
+      <x:c r="F13" s="10"/>
       <x:c r="G13" s="10"/>
-      <x:c r="H13" s="6"/>
-      <x:c r="I13" s="10"/>
+      <x:c r="H13" s="10"/>
+      <x:c r="I13" s="6"/>
       <x:c r="J13" s="10"/>
       <x:c r="K13" s="10"/>
       <x:c r="L13" s="10"/>
-      <x:c r="M13" s="7"/>
+      <x:c r="M13" s="10"/>
+      <x:c r="N13" s="10"/>
+      <x:c r="O13" s="10"/>
+      <x:c r="P13" s="10"/>
+      <x:c r="Q13" s="10"/>
+      <x:c r="R13" s="6"/>
+      <x:c r="S13" s="6"/>
+      <x:c r="T13" s="6"/>
+      <x:c r="U13" s="6"/>
+      <x:c r="V13" s="6"/>
+      <x:c r="W13" s="7"/>
+      <x:c r="X13" s="7"/>
+      <x:c r="Y13" s="9"/>
+      <x:c r="Z13" s="10"/>
+      <x:c r="AA13" s="6"/>
+      <x:c r="AB13" s="10"/>
+      <x:c r="AC13" s="10"/>
+      <x:c r="AD13" s="10"/>
+      <x:c r="AE13" s="10"/>
+      <x:c r="AF13" s="7"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7"/>
       <x:c r="B14" s="7"/>
       <x:c r="C14" s="7"/>
-      <x:c r="D14" s="7"/>
-      <x:c r="E14" s="7"/>
-      <x:c r="F14" s="9"/>
+      <x:c r="D14" s="6"/>
+      <x:c r="E14" s="6"/>
+      <x:c r="F14" s="10"/>
       <x:c r="G14" s="10"/>
-      <x:c r="H14" s="6"/>
-      <x:c r="I14" s="10"/>
+      <x:c r="H14" s="10"/>
+      <x:c r="I14" s="6"/>
       <x:c r="J14" s="10"/>
       <x:c r="K14" s="10"/>
       <x:c r="L14" s="10"/>
-      <x:c r="M14" s="7"/>
+      <x:c r="M14" s="10"/>
+      <x:c r="N14" s="10"/>
+      <x:c r="O14" s="10"/>
+      <x:c r="P14" s="10"/>
+      <x:c r="Q14" s="10"/>
+      <x:c r="R14" s="6"/>
+      <x:c r="S14" s="6"/>
+      <x:c r="T14" s="6"/>
+      <x:c r="U14" s="6"/>
+      <x:c r="V14" s="6"/>
+      <x:c r="W14" s="7"/>
+      <x:c r="X14" s="7"/>
+      <x:c r="Y14" s="9"/>
+      <x:c r="Z14" s="10"/>
+      <x:c r="AA14" s="6"/>
+      <x:c r="AB14" s="10"/>
+      <x:c r="AC14" s="10"/>
+      <x:c r="AD14" s="10"/>
+      <x:c r="AE14" s="10"/>
+      <x:c r="AF14" s="7"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7"/>
       <x:c r="B15" s="7"/>
       <x:c r="C15" s="7"/>
-      <x:c r="D15" s="7"/>
-      <x:c r="E15" s="7"/>
-      <x:c r="F15" s="9"/>
+      <x:c r="D15" s="6"/>
+      <x:c r="E15" s="6"/>
+      <x:c r="F15" s="10"/>
       <x:c r="G15" s="10"/>
-      <x:c r="H15" s="6"/>
-      <x:c r="I15" s="10"/>
+      <x:c r="H15" s="10"/>
+      <x:c r="I15" s="6"/>
       <x:c r="J15" s="10"/>
       <x:c r="K15" s="10"/>
       <x:c r="L15" s="10"/>
-      <x:c r="M15" s="7"/>
+      <x:c r="M15" s="10"/>
+      <x:c r="N15" s="10"/>
+      <x:c r="O15" s="10"/>
+      <x:c r="P15" s="10"/>
+      <x:c r="Q15" s="10"/>
+      <x:c r="R15" s="6"/>
+      <x:c r="S15" s="6"/>
+      <x:c r="T15" s="6"/>
+      <x:c r="U15" s="6"/>
+      <x:c r="V15" s="6"/>
+      <x:c r="W15" s="7"/>
+      <x:c r="X15" s="7"/>
+      <x:c r="Y15" s="9"/>
+      <x:c r="Z15" s="10"/>
+      <x:c r="AA15" s="6"/>
+      <x:c r="AB15" s="10"/>
+      <x:c r="AC15" s="10"/>
+      <x:c r="AD15" s="10"/>
+      <x:c r="AE15" s="10"/>
+      <x:c r="AF15" s="7"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7"/>
       <x:c r="B16" s="7"/>
       <x:c r="C16" s="7"/>
-      <x:c r="D16" s="7"/>
-      <x:c r="E16" s="7"/>
-      <x:c r="F16" s="9"/>
+      <x:c r="D16" s="6"/>
+      <x:c r="E16" s="6"/>
+      <x:c r="F16" s="10"/>
       <x:c r="G16" s="10"/>
-      <x:c r="H16" s="6"/>
-      <x:c r="I16" s="10"/>
+      <x:c r="H16" s="10"/>
+      <x:c r="I16" s="6"/>
       <x:c r="J16" s="10"/>
       <x:c r="K16" s="10"/>
       <x:c r="L16" s="10"/>
-      <x:c r="M16" s="7"/>
+      <x:c r="M16" s="10"/>
+      <x:c r="N16" s="10"/>
+      <x:c r="O16" s="10"/>
+      <x:c r="P16" s="10"/>
+      <x:c r="Q16" s="10"/>
+      <x:c r="R16" s="6"/>
+      <x:c r="S16" s="6"/>
+      <x:c r="T16" s="6"/>
+      <x:c r="U16" s="6"/>
+      <x:c r="V16" s="6"/>
+      <x:c r="W16" s="7"/>
+      <x:c r="X16" s="7"/>
+      <x:c r="Y16" s="9"/>
+      <x:c r="Z16" s="10"/>
+      <x:c r="AA16" s="6"/>
+      <x:c r="AB16" s="10"/>
+      <x:c r="AC16" s="10"/>
+      <x:c r="AD16" s="10"/>
+      <x:c r="AE16" s="10"/>
+      <x:c r="AF16" s="7"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7"/>
       <x:c r="B17" s="7"/>
       <x:c r="C17" s="7"/>
-      <x:c r="D17" s="7"/>
-      <x:c r="E17" s="7"/>
-      <x:c r="F17" s="9"/>
+      <x:c r="D17" s="6"/>
+      <x:c r="E17" s="6"/>
+      <x:c r="F17" s="10"/>
       <x:c r="G17" s="10"/>
-      <x:c r="H17" s="6"/>
-      <x:c r="I17" s="10"/>
+      <x:c r="H17" s="10"/>
+      <x:c r="I17" s="6"/>
       <x:c r="J17" s="10"/>
       <x:c r="K17" s="10"/>
       <x:c r="L17" s="10"/>
-      <x:c r="M17" s="7"/>
+      <x:c r="M17" s="10"/>
+      <x:c r="N17" s="10"/>
+      <x:c r="O17" s="10"/>
+      <x:c r="P17" s="10"/>
+      <x:c r="Q17" s="10"/>
+      <x:c r="R17" s="6"/>
+      <x:c r="S17" s="6"/>
+      <x:c r="T17" s="6"/>
+      <x:c r="U17" s="6"/>
+      <x:c r="V17" s="6"/>
+      <x:c r="W17" s="7"/>
+      <x:c r="X17" s="7"/>
+      <x:c r="Y17" s="9"/>
+      <x:c r="Z17" s="10"/>
+      <x:c r="AA17" s="6"/>
+      <x:c r="AB17" s="10"/>
+      <x:c r="AC17" s="10"/>
+      <x:c r="AD17" s="10"/>
+      <x:c r="AE17" s="10"/>
+      <x:c r="AF17" s="7"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7"/>
       <x:c r="B18" s="7"/>
       <x:c r="C18" s="7"/>
-      <x:c r="D18" s="7"/>
-      <x:c r="E18" s="7"/>
-      <x:c r="F18" s="9"/>
+      <x:c r="D18" s="6"/>
+      <x:c r="E18" s="6"/>
+      <x:c r="F18" s="10"/>
       <x:c r="G18" s="10"/>
-      <x:c r="H18" s="6"/>
-      <x:c r="I18" s="10"/>
+      <x:c r="H18" s="10"/>
+      <x:c r="I18" s="6"/>
       <x:c r="J18" s="10"/>
       <x:c r="K18" s="10"/>
       <x:c r="L18" s="10"/>
-      <x:c r="M18" s="7"/>
+      <x:c r="M18" s="10"/>
+      <x:c r="N18" s="10"/>
+      <x:c r="O18" s="10"/>
+      <x:c r="P18" s="10"/>
+      <x:c r="Q18" s="10"/>
+      <x:c r="R18" s="6"/>
+      <x:c r="S18" s="6"/>
+      <x:c r="T18" s="6"/>
+      <x:c r="U18" s="6"/>
+      <x:c r="V18" s="6"/>
+      <x:c r="W18" s="7"/>
+      <x:c r="X18" s="7"/>
+      <x:c r="Y18" s="9"/>
+      <x:c r="Z18" s="10"/>
+      <x:c r="AA18" s="6"/>
+      <x:c r="AB18" s="10"/>
+      <x:c r="AC18" s="10"/>
+      <x:c r="AD18" s="10"/>
+      <x:c r="AE18" s="10"/>
+      <x:c r="AF18" s="7"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7"/>
       <x:c r="B19" s="7"/>
       <x:c r="C19" s="7"/>
-      <x:c r="D19" s="7"/>
-      <x:c r="E19" s="7"/>
-      <x:c r="F19" s="9"/>
+      <x:c r="D19" s="6"/>
+      <x:c r="E19" s="6"/>
+      <x:c r="F19" s="10"/>
       <x:c r="G19" s="10"/>
-      <x:c r="H19" s="6"/>
-      <x:c r="I19" s="10"/>
+      <x:c r="H19" s="10"/>
+      <x:c r="I19" s="6"/>
       <x:c r="J19" s="10"/>
       <x:c r="K19" s="10"/>
       <x:c r="L19" s="10"/>
-      <x:c r="M19" s="7"/>
+      <x:c r="M19" s="10"/>
+      <x:c r="N19" s="10"/>
+      <x:c r="O19" s="10"/>
+      <x:c r="P19" s="10"/>
+      <x:c r="Q19" s="10"/>
+      <x:c r="R19" s="6"/>
+      <x:c r="S19" s="6"/>
+      <x:c r="T19" s="6"/>
+      <x:c r="U19" s="6"/>
+      <x:c r="V19" s="6"/>
+      <x:c r="W19" s="7"/>
+      <x:c r="X19" s="7"/>
+      <x:c r="Y19" s="9"/>
+      <x:c r="Z19" s="10"/>
+      <x:c r="AA19" s="6"/>
+      <x:c r="AB19" s="10"/>
+      <x:c r="AC19" s="10"/>
+      <x:c r="AD19" s="10"/>
+      <x:c r="AE19" s="10"/>
+      <x:c r="AF19" s="7"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7"/>
       <x:c r="B20" s="7"/>
       <x:c r="C20" s="7"/>
-      <x:c r="D20" s="7"/>
-      <x:c r="E20" s="7"/>
-      <x:c r="F20" s="9"/>
+      <x:c r="D20" s="6"/>
+      <x:c r="E20" s="6"/>
+      <x:c r="F20" s="10"/>
       <x:c r="G20" s="10"/>
-      <x:c r="H20" s="6"/>
-      <x:c r="I20" s="10"/>
+      <x:c r="H20" s="10"/>
+      <x:c r="I20" s="6"/>
       <x:c r="J20" s="10"/>
       <x:c r="K20" s="10"/>
       <x:c r="L20" s="10"/>
-      <x:c r="M20" s="7"/>
+      <x:c r="M20" s="10"/>
+      <x:c r="N20" s="10"/>
+      <x:c r="O20" s="10"/>
+      <x:c r="P20" s="10"/>
+      <x:c r="Q20" s="10"/>
+      <x:c r="R20" s="6"/>
+      <x:c r="S20" s="6"/>
+      <x:c r="T20" s="6"/>
+      <x:c r="U20" s="6"/>
+      <x:c r="V20" s="6"/>
+      <x:c r="W20" s="7"/>
+      <x:c r="X20" s="7"/>
+      <x:c r="Y20" s="9"/>
+      <x:c r="Z20" s="10"/>
+      <x:c r="AA20" s="6"/>
+      <x:c r="AB20" s="10"/>
+      <x:c r="AC20" s="10"/>
+      <x:c r="AD20" s="10"/>
+      <x:c r="AE20" s="10"/>
+      <x:c r="AF20" s="7"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7"/>
       <x:c r="B21" s="7"/>
       <x:c r="C21" s="7"/>
-      <x:c r="D21" s="7"/>
-      <x:c r="E21" s="7"/>
-      <x:c r="F21" s="9"/>
+      <x:c r="D21" s="6"/>
+      <x:c r="E21" s="6"/>
+      <x:c r="F21" s="10"/>
       <x:c r="G21" s="10"/>
-      <x:c r="H21" s="6"/>
-      <x:c r="I21" s="10"/>
+      <x:c r="H21" s="10"/>
+      <x:c r="I21" s="6"/>
       <x:c r="J21" s="10"/>
       <x:c r="K21" s="10"/>
       <x:c r="L21" s="10"/>
-      <x:c r="M21" s="7"/>
+      <x:c r="M21" s="10"/>
+      <x:c r="N21" s="10"/>
+      <x:c r="O21" s="10"/>
+      <x:c r="P21" s="10"/>
+      <x:c r="Q21" s="10"/>
+      <x:c r="R21" s="6"/>
+      <x:c r="S21" s="6"/>
+      <x:c r="T21" s="6"/>
+      <x:c r="U21" s="6"/>
+      <x:c r="V21" s="6"/>
+      <x:c r="W21" s="7"/>
+      <x:c r="X21" s="7"/>
+      <x:c r="Y21" s="9"/>
+      <x:c r="Z21" s="10"/>
+      <x:c r="AA21" s="6"/>
+      <x:c r="AB21" s="10"/>
+      <x:c r="AC21" s="10"/>
+      <x:c r="AD21" s="10"/>
+      <x:c r="AE21" s="10"/>
+      <x:c r="AF21" s="7"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="7"/>
       <x:c r="B22" s="7"/>
       <x:c r="C22" s="7"/>
-      <x:c r="D22" s="7"/>
-      <x:c r="E22" s="7"/>
-      <x:c r="F22" s="9"/>
+      <x:c r="D22" s="6"/>
+      <x:c r="E22" s="6"/>
+      <x:c r="F22" s="10"/>
       <x:c r="G22" s="10"/>
-      <x:c r="H22" s="6"/>
-      <x:c r="I22" s="10"/>
+      <x:c r="H22" s="10"/>
+      <x:c r="I22" s="6"/>
       <x:c r="J22" s="10"/>
       <x:c r="K22" s="10"/>
       <x:c r="L22" s="10"/>
-      <x:c r="M22" s="7"/>
+      <x:c r="M22" s="10"/>
+      <x:c r="N22" s="10"/>
+      <x:c r="O22" s="10"/>
+      <x:c r="P22" s="10"/>
+      <x:c r="Q22" s="10"/>
+      <x:c r="R22" s="6"/>
+      <x:c r="S22" s="6"/>
+      <x:c r="T22" s="6"/>
+      <x:c r="U22" s="6"/>
+      <x:c r="V22" s="6"/>
+      <x:c r="W22" s="7"/>
+      <x:c r="X22" s="7"/>
+      <x:c r="Y22" s="9"/>
+      <x:c r="Z22" s="10"/>
+      <x:c r="AA22" s="6"/>
+      <x:c r="AB22" s="10"/>
+      <x:c r="AC22" s="10"/>
+      <x:c r="AD22" s="10"/>
+      <x:c r="AE22" s="10"/>
+      <x:c r="AF22" s="7"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7"/>
       <x:c r="B23" s="7"/>
       <x:c r="C23" s="7"/>
-      <x:c r="D23" s="7"/>
-      <x:c r="E23" s="7"/>
-      <x:c r="F23" s="9"/>
+      <x:c r="D23" s="6"/>
+      <x:c r="E23" s="6"/>
+      <x:c r="F23" s="10"/>
       <x:c r="G23" s="10"/>
-      <x:c r="H23" s="6"/>
-      <x:c r="I23" s="10"/>
+      <x:c r="H23" s="10"/>
+      <x:c r="I23" s="6"/>
       <x:c r="J23" s="10"/>
       <x:c r="K23" s="10"/>
       <x:c r="L23" s="10"/>
-      <x:c r="M23" s="7"/>
+      <x:c r="M23" s="10"/>
+      <x:c r="N23" s="10"/>
+      <x:c r="O23" s="10"/>
+      <x:c r="P23" s="10"/>
+      <x:c r="Q23" s="10"/>
+      <x:c r="R23" s="6"/>
+      <x:c r="S23" s="6"/>
+      <x:c r="T23" s="6"/>
+      <x:c r="U23" s="6"/>
+      <x:c r="V23" s="6"/>
+      <x:c r="W23" s="7"/>
+      <x:c r="X23" s="7"/>
+      <x:c r="Y23" s="9"/>
+      <x:c r="Z23" s="10"/>
+      <x:c r="AA23" s="6"/>
+      <x:c r="AB23" s="10"/>
+      <x:c r="AC23" s="10"/>
+      <x:c r="AD23" s="10"/>
+      <x:c r="AE23" s="10"/>
+      <x:c r="AF23" s="7"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7"/>
       <x:c r="B24" s="7"/>
       <x:c r="C24" s="7"/>
-      <x:c r="D24" s="7"/>
-      <x:c r="E24" s="7"/>
-      <x:c r="F24" s="9"/>
+      <x:c r="D24" s="6"/>
+      <x:c r="E24" s="6"/>
+      <x:c r="F24" s="10"/>
       <x:c r="G24" s="10"/>
-      <x:c r="H24" s="6"/>
-      <x:c r="I24" s="10"/>
+      <x:c r="H24" s="10"/>
+      <x:c r="I24" s="6"/>
       <x:c r="J24" s="10"/>
       <x:c r="K24" s="10"/>
       <x:c r="L24" s="10"/>
-      <x:c r="M24" s="7"/>
+      <x:c r="M24" s="10"/>
+      <x:c r="N24" s="10"/>
+      <x:c r="O24" s="10"/>
+      <x:c r="P24" s="10"/>
+      <x:c r="Q24" s="10"/>
+      <x:c r="R24" s="6"/>
+      <x:c r="S24" s="6"/>
+      <x:c r="T24" s="6"/>
+      <x:c r="U24" s="6"/>
+      <x:c r="V24" s="6"/>
+      <x:c r="W24" s="7"/>
+      <x:c r="X24" s="7"/>
+      <x:c r="Y24" s="9"/>
+      <x:c r="Z24" s="10"/>
+      <x:c r="AA24" s="6"/>
+      <x:c r="AB24" s="10"/>
+      <x:c r="AC24" s="10"/>
+      <x:c r="AD24" s="10"/>
+      <x:c r="AE24" s="10"/>
+      <x:c r="AF24" s="7"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="E5:E24">
+      <x:formula1>"Sí,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I24">
+      <x:formula1>"A,B,C"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Reglas de vidrio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" customHeight="1">
+      <x:c r="A4" s="5" t="str">
+        <x:v>Código de regla</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>Nombre</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Zona de riesgo</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>Antepecho de referencia (mm)</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="str">
+        <x:v>Área de referencia (m²)</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="str">
+        <x:v>Clases admitidas separadas por |</x:v>
+      </x:c>
+      <x:c r="G4" s="5" t="str">
+        <x:v>Obligatoria</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="str">
+        <x:v>Ejemplo sintético</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="7"/>
+      <x:c r="B5" s="7"/>
+      <x:c r="C5" s="7"/>
+      <x:c r="D5" s="10"/>
+      <x:c r="E5" s="10"/>
+      <x:c r="F5" s="7"/>
+      <x:c r="G5" s="7"/>
+      <x:c r="H5" s="7"/>
+      <x:c r="I5" s="7"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="7"/>
+      <x:c r="B6" s="7"/>
+      <x:c r="C6" s="7"/>
+      <x:c r="D6" s="10"/>
+      <x:c r="E6" s="10"/>
+      <x:c r="F6" s="7"/>
+      <x:c r="G6" s="7"/>
+      <x:c r="H6" s="7"/>
+      <x:c r="I6" s="7"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="7"/>
+      <x:c r="B7" s="7"/>
+      <x:c r="C7" s="7"/>
+      <x:c r="D7" s="10"/>
+      <x:c r="E7" s="10"/>
+      <x:c r="F7" s="7"/>
+      <x:c r="G7" s="7"/>
+      <x:c r="H7" s="7"/>
+      <x:c r="I7" s="7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="7"/>
+      <x:c r="B8" s="7"/>
+      <x:c r="C8" s="7"/>
+      <x:c r="D8" s="10"/>
+      <x:c r="E8" s="10"/>
+      <x:c r="F8" s="7"/>
+      <x:c r="G8" s="7"/>
+      <x:c r="H8" s="7"/>
+      <x:c r="I8" s="7"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="7"/>
+      <x:c r="B9" s="7"/>
+      <x:c r="C9" s="7"/>
+      <x:c r="D9" s="10"/>
+      <x:c r="E9" s="10"/>
+      <x:c r="F9" s="7"/>
+      <x:c r="G9" s="7"/>
+      <x:c r="H9" s="7"/>
+      <x:c r="I9" s="7"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="7"/>
+      <x:c r="B10" s="7"/>
+      <x:c r="C10" s="7"/>
+      <x:c r="D10" s="10"/>
+      <x:c r="E10" s="10"/>
+      <x:c r="F10" s="7"/>
+      <x:c r="G10" s="7"/>
+      <x:c r="H10" s="7"/>
+      <x:c r="I10" s="7"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="7"/>
+      <x:c r="B11" s="7"/>
+      <x:c r="C11" s="7"/>
+      <x:c r="D11" s="10"/>
+      <x:c r="E11" s="10"/>
+      <x:c r="F11" s="7"/>
+      <x:c r="G11" s="7"/>
+      <x:c r="H11" s="7"/>
+      <x:c r="I11" s="7"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="7"/>
+      <x:c r="B12" s="7"/>
+      <x:c r="C12" s="7"/>
+      <x:c r="D12" s="10"/>
+      <x:c r="E12" s="10"/>
+      <x:c r="F12" s="7"/>
+      <x:c r="G12" s="7"/>
+      <x:c r="H12" s="7"/>
+      <x:c r="I12" s="7"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="7"/>
+      <x:c r="B13" s="7"/>
+      <x:c r="C13" s="7"/>
+      <x:c r="D13" s="10"/>
+      <x:c r="E13" s="10"/>
+      <x:c r="F13" s="7"/>
+      <x:c r="G13" s="7"/>
+      <x:c r="H13" s="7"/>
+      <x:c r="I13" s="7"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7"/>
+      <x:c r="B14" s="7"/>
+      <x:c r="C14" s="7"/>
+      <x:c r="D14" s="10"/>
+      <x:c r="E14" s="10"/>
+      <x:c r="F14" s="7"/>
+      <x:c r="G14" s="7"/>
+      <x:c r="H14" s="7"/>
+      <x:c r="I14" s="7"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="7"/>
+      <x:c r="B15" s="7"/>
+      <x:c r="C15" s="7"/>
+      <x:c r="D15" s="10"/>
+      <x:c r="E15" s="10"/>
+      <x:c r="F15" s="7"/>
+      <x:c r="G15" s="7"/>
+      <x:c r="H15" s="7"/>
+      <x:c r="I15" s="7"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="7"/>
+      <x:c r="B16" s="7"/>
+      <x:c r="C16" s="7"/>
+      <x:c r="D16" s="10"/>
+      <x:c r="E16" s="10"/>
+      <x:c r="F16" s="7"/>
+      <x:c r="G16" s="7"/>
+      <x:c r="H16" s="7"/>
+      <x:c r="I16" s="7"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="7"/>
+      <x:c r="B17" s="7"/>
+      <x:c r="C17" s="7"/>
+      <x:c r="D17" s="10"/>
+      <x:c r="E17" s="10"/>
+      <x:c r="F17" s="7"/>
+      <x:c r="G17" s="7"/>
+      <x:c r="H17" s="7"/>
+      <x:c r="I17" s="7"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="7"/>
+      <x:c r="B18" s="7"/>
+      <x:c r="C18" s="7"/>
+      <x:c r="D18" s="10"/>
+      <x:c r="E18" s="10"/>
+      <x:c r="F18" s="7"/>
+      <x:c r="G18" s="7"/>
+      <x:c r="H18" s="7"/>
+      <x:c r="I18" s="7"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="7"/>
+      <x:c r="B19" s="7"/>
+      <x:c r="C19" s="7"/>
+      <x:c r="D19" s="10"/>
+      <x:c r="E19" s="10"/>
+      <x:c r="F19" s="7"/>
+      <x:c r="G19" s="7"/>
+      <x:c r="H19" s="7"/>
+      <x:c r="I19" s="7"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="7"/>
+      <x:c r="B20" s="7"/>
+      <x:c r="C20" s="7"/>
+      <x:c r="D20" s="10"/>
+      <x:c r="E20" s="10"/>
+      <x:c r="F20" s="7"/>
+      <x:c r="G20" s="7"/>
+      <x:c r="H20" s="7"/>
+      <x:c r="I20" s="7"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="7"/>
+      <x:c r="B21" s="7"/>
+      <x:c r="C21" s="7"/>
+      <x:c r="D21" s="10"/>
+      <x:c r="E21" s="10"/>
+      <x:c r="F21" s="7"/>
+      <x:c r="G21" s="7"/>
+      <x:c r="H21" s="7"/>
+      <x:c r="I21" s="7"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="7"/>
+      <x:c r="B22" s="7"/>
+      <x:c r="C22" s="7"/>
+      <x:c r="D22" s="10"/>
+      <x:c r="E22" s="10"/>
+      <x:c r="F22" s="7"/>
+      <x:c r="G22" s="7"/>
+      <x:c r="H22" s="7"/>
+      <x:c r="I22" s="7"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="7"/>
+      <x:c r="B23" s="7"/>
+      <x:c r="C23" s="7"/>
+      <x:c r="D23" s="10"/>
+      <x:c r="E23" s="10"/>
+      <x:c r="F23" s="7"/>
+      <x:c r="G23" s="7"/>
+      <x:c r="H23" s="7"/>
+      <x:c r="I23" s="7"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="7"/>
+      <x:c r="B24" s="7"/>
+      <x:c r="C24" s="7"/>
+      <x:c r="D24" s="10"/>
+      <x:c r="E24" s="10"/>
+      <x:c r="F24" s="7"/>
+      <x:c r="G24" s="7"/>
+      <x:c r="H24" s="7"/>
+      <x:c r="I24" s="7"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="C5:C24">
+      <x:formula1>"Puerta,Panel lateral,Paño bajo,Gran ventanal"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G5:G24">
+      <x:formula1>"Sí,No"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H5:H24">
+      <x:formula1>"Sí,No"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3490,342 +4583,4 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>Precios de costo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="2" t="str">
-        <x:v>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="48" customHeight="1">
-      <x:c r="A4" s="5" t="str">
-        <x:v>Código de sistema</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>SKU</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="str">
-        <x:v>Lista de costo</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="str">
-        <x:v>Proveedor</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="str">
-        <x:v>Moneda</x:v>
-      </x:c>
-      <x:c r="F4" s="5" t="str">
-        <x:v>Vigente desde (aaaa-mm-dd)</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="str">
-        <x:v>Vigente hasta (aaaa-mm-dd)</x:v>
-      </x:c>
-      <x:c r="H4" s="5" t="str">
-        <x:v>Tipo de artículo</x:v>
-      </x:c>
-      <x:c r="I4" s="5" t="str">
-        <x:v>Unidad</x:v>
-      </x:c>
-      <x:c r="J4" s="5" t="str">
-        <x:v>Costo unitario</x:v>
-      </x:c>
-      <x:c r="K4" s="5" t="str">
-        <x:v>Fuente</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="7"/>
-      <x:c r="B5" s="7"/>
-      <x:c r="C5" s="7"/>
-      <x:c r="D5" s="7"/>
-      <x:c r="E5" s="7"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="13"/>
-      <x:c r="H5" s="7"/>
-      <x:c r="I5" s="7"/>
-      <x:c r="J5" s="8"/>
-      <x:c r="K5" s="7"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="7"/>
-      <x:c r="B6" s="7"/>
-      <x:c r="C6" s="7"/>
-      <x:c r="D6" s="7"/>
-      <x:c r="E6" s="7"/>
-      <x:c r="F6" s="12"/>
-      <x:c r="G6" s="13"/>
-      <x:c r="H6" s="7"/>
-      <x:c r="I6" s="7"/>
-      <x:c r="J6" s="8"/>
-      <x:c r="K6" s="7"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="7"/>
-      <x:c r="B7" s="7"/>
-      <x:c r="C7" s="7"/>
-      <x:c r="D7" s="7"/>
-      <x:c r="E7" s="7"/>
-      <x:c r="F7" s="12"/>
-      <x:c r="G7" s="13"/>
-      <x:c r="H7" s="7"/>
-      <x:c r="I7" s="7"/>
-      <x:c r="J7" s="8"/>
-      <x:c r="K7" s="7"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="7"/>
-      <x:c r="B8" s="7"/>
-      <x:c r="C8" s="7"/>
-      <x:c r="D8" s="7"/>
-      <x:c r="E8" s="7"/>
-      <x:c r="F8" s="12"/>
-      <x:c r="G8" s="13"/>
-      <x:c r="H8" s="7"/>
-      <x:c r="I8" s="7"/>
-      <x:c r="J8" s="8"/>
-      <x:c r="K8" s="7"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="7"/>
-      <x:c r="B9" s="7"/>
-      <x:c r="C9" s="7"/>
-      <x:c r="D9" s="7"/>
-      <x:c r="E9" s="7"/>
-      <x:c r="F9" s="12"/>
-      <x:c r="G9" s="13"/>
-      <x:c r="H9" s="7"/>
-      <x:c r="I9" s="7"/>
-      <x:c r="J9" s="8"/>
-      <x:c r="K9" s="7"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="7"/>
-      <x:c r="B10" s="7"/>
-      <x:c r="C10" s="7"/>
-      <x:c r="D10" s="7"/>
-      <x:c r="E10" s="7"/>
-      <x:c r="F10" s="12"/>
-      <x:c r="G10" s="13"/>
-      <x:c r="H10" s="7"/>
-      <x:c r="I10" s="7"/>
-      <x:c r="J10" s="8"/>
-      <x:c r="K10" s="7"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="7"/>
-      <x:c r="B11" s="7"/>
-      <x:c r="C11" s="7"/>
-      <x:c r="D11" s="7"/>
-      <x:c r="E11" s="7"/>
-      <x:c r="F11" s="12"/>
-      <x:c r="G11" s="13"/>
-      <x:c r="H11" s="7"/>
-      <x:c r="I11" s="7"/>
-      <x:c r="J11" s="8"/>
-      <x:c r="K11" s="7"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="7"/>
-      <x:c r="B12" s="7"/>
-      <x:c r="C12" s="7"/>
-      <x:c r="D12" s="7"/>
-      <x:c r="E12" s="7"/>
-      <x:c r="F12" s="12"/>
-      <x:c r="G12" s="13"/>
-      <x:c r="H12" s="7"/>
-      <x:c r="I12" s="7"/>
-      <x:c r="J12" s="8"/>
-      <x:c r="K12" s="7"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="7"/>
-      <x:c r="B13" s="7"/>
-      <x:c r="C13" s="7"/>
-      <x:c r="D13" s="7"/>
-      <x:c r="E13" s="7"/>
-      <x:c r="F13" s="12"/>
-      <x:c r="G13" s="13"/>
-      <x:c r="H13" s="7"/>
-      <x:c r="I13" s="7"/>
-      <x:c r="J13" s="8"/>
-      <x:c r="K13" s="7"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="7"/>
-      <x:c r="B14" s="7"/>
-      <x:c r="C14" s="7"/>
-      <x:c r="D14" s="7"/>
-      <x:c r="E14" s="7"/>
-      <x:c r="F14" s="12"/>
-      <x:c r="G14" s="13"/>
-      <x:c r="H14" s="7"/>
-      <x:c r="I14" s="7"/>
-      <x:c r="J14" s="8"/>
-      <x:c r="K14" s="7"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="7"/>
-      <x:c r="B15" s="7"/>
-      <x:c r="C15" s="7"/>
-      <x:c r="D15" s="7"/>
-      <x:c r="E15" s="7"/>
-      <x:c r="F15" s="12"/>
-      <x:c r="G15" s="13"/>
-      <x:c r="H15" s="7"/>
-      <x:c r="I15" s="7"/>
-      <x:c r="J15" s="8"/>
-      <x:c r="K15" s="7"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="7"/>
-      <x:c r="B16" s="7"/>
-      <x:c r="C16" s="7"/>
-      <x:c r="D16" s="7"/>
-      <x:c r="E16" s="7"/>
-      <x:c r="F16" s="12"/>
-      <x:c r="G16" s="13"/>
-      <x:c r="H16" s="7"/>
-      <x:c r="I16" s="7"/>
-      <x:c r="J16" s="8"/>
-      <x:c r="K16" s="7"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="7"/>
-      <x:c r="B17" s="7"/>
-      <x:c r="C17" s="7"/>
-      <x:c r="D17" s="7"/>
-      <x:c r="E17" s="7"/>
-      <x:c r="F17" s="12"/>
-      <x:c r="G17" s="13"/>
-      <x:c r="H17" s="7"/>
-      <x:c r="I17" s="7"/>
-      <x:c r="J17" s="8"/>
-      <x:c r="K17" s="7"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="7"/>
-      <x:c r="B18" s="7"/>
-      <x:c r="C18" s="7"/>
-      <x:c r="D18" s="7"/>
-      <x:c r="E18" s="7"/>
-      <x:c r="F18" s="12"/>
-      <x:c r="G18" s="13"/>
-      <x:c r="H18" s="7"/>
-      <x:c r="I18" s="7"/>
-      <x:c r="J18" s="8"/>
-      <x:c r="K18" s="7"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="7"/>
-      <x:c r="B19" s="7"/>
-      <x:c r="C19" s="7"/>
-      <x:c r="D19" s="7"/>
-      <x:c r="E19" s="7"/>
-      <x:c r="F19" s="12"/>
-      <x:c r="G19" s="13"/>
-      <x:c r="H19" s="7"/>
-      <x:c r="I19" s="7"/>
-      <x:c r="J19" s="8"/>
-      <x:c r="K19" s="7"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="7"/>
-      <x:c r="B20" s="7"/>
-      <x:c r="C20" s="7"/>
-      <x:c r="D20" s="7"/>
-      <x:c r="E20" s="7"/>
-      <x:c r="F20" s="12"/>
-      <x:c r="G20" s="13"/>
-      <x:c r="H20" s="7"/>
-      <x:c r="I20" s="7"/>
-      <x:c r="J20" s="8"/>
-      <x:c r="K20" s="7"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="7"/>
-      <x:c r="B21" s="7"/>
-      <x:c r="C21" s="7"/>
-      <x:c r="D21" s="7"/>
-      <x:c r="E21" s="7"/>
-      <x:c r="F21" s="12"/>
-      <x:c r="G21" s="13"/>
-      <x:c r="H21" s="7"/>
-      <x:c r="I21" s="7"/>
-      <x:c r="J21" s="8"/>
-      <x:c r="K21" s="7"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="7"/>
-      <x:c r="B22" s="7"/>
-      <x:c r="C22" s="7"/>
-      <x:c r="D22" s="7"/>
-      <x:c r="E22" s="7"/>
-      <x:c r="F22" s="12"/>
-      <x:c r="G22" s="13"/>
-      <x:c r="H22" s="7"/>
-      <x:c r="I22" s="7"/>
-      <x:c r="J22" s="8"/>
-      <x:c r="K22" s="7"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="7"/>
-      <x:c r="B23" s="7"/>
-      <x:c r="C23" s="7"/>
-      <x:c r="D23" s="7"/>
-      <x:c r="E23" s="7"/>
-      <x:c r="F23" s="12"/>
-      <x:c r="G23" s="13"/>
-      <x:c r="H23" s="7"/>
-      <x:c r="I23" s="7"/>
-      <x:c r="J23" s="8"/>
-      <x:c r="K23" s="7"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="7"/>
-      <x:c r="B24" s="7"/>
-      <x:c r="C24" s="7"/>
-      <x:c r="D24" s="7"/>
-      <x:c r="E24" s="7"/>
-      <x:c r="F24" s="12"/>
-      <x:c r="G24" s="13"/>
-      <x:c r="H24" s="7"/>
-      <x:c r="I24" s="7"/>
-      <x:c r="J24" s="8"/>
-      <x:c r="K24" s="7"/>
-    </x:row>
-  </x:sheetData>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="E5:E24">
-      <x:formula1>"CLP,USD"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="H5:H24">
-      <x:formula1>"Perfil,Refuerzo,Vidrio,Herraje,Otro"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="I5:I24">
-      <x:formula1>"Barra,Metro,Metro cuadrado,Kit,Unidad"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
D04: resolver herrajes por clase y sellar componentes de fabricación
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$F$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$Q$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Precios de costo'!$A$4:$K$24</definedName>
   </definedNames>
 </workbook>
@@ -1711,8 +1711,8 @@
   </sheetData>
   <autoFilter ref="A4:K24"/>
   <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
@@ -4640,7 +4640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4658,8 +4658,9 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="47" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4755,10 +4756,15 @@
       </c>
       <c r="P4" s="14" t="inlineStr">
         <is>
-          <t>Componentes (JSON)</t>
+          <t>Componentes históricos (JSON)</t>
         </is>
       </c>
       <c r="Q4" s="14" t="inlineStr">
+        <is>
+          <t>Familia, clase y reglas de componentes (JSON)</t>
+        </is>
+      </c>
+      <c r="R4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -4782,6 +4788,7 @@
       <c r="O5" s="15" t="n"/>
       <c r="P5" s="15" t="n"/>
       <c r="Q5" s="15" t="n"/>
+      <c r="R5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -4801,6 +4808,7 @@
       <c r="O6" s="15" t="n"/>
       <c r="P6" s="15" t="n"/>
       <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -4820,6 +4828,7 @@
       <c r="O7" s="15" t="n"/>
       <c r="P7" s="15" t="n"/>
       <c r="Q7" s="15" t="n"/>
+      <c r="R7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -4839,6 +4848,7 @@
       <c r="O8" s="15" t="n"/>
       <c r="P8" s="15" t="n"/>
       <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -4858,6 +4868,7 @@
       <c r="O9" s="15" t="n"/>
       <c r="P9" s="15" t="n"/>
       <c r="Q9" s="15" t="n"/>
+      <c r="R9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -4877,6 +4888,7 @@
       <c r="O10" s="15" t="n"/>
       <c r="P10" s="15" t="n"/>
       <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -4896,6 +4908,7 @@
       <c r="O11" s="15" t="n"/>
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -4915,6 +4928,7 @@
       <c r="O12" s="15" t="n"/>
       <c r="P12" s="15" t="n"/>
       <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -4934,6 +4948,7 @@
       <c r="O13" s="15" t="n"/>
       <c r="P13" s="15" t="n"/>
       <c r="Q13" s="15" t="n"/>
+      <c r="R13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -4953,6 +4968,7 @@
       <c r="O14" s="15" t="n"/>
       <c r="P14" s="15" t="n"/>
       <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -4972,6 +4988,7 @@
       <c r="O15" s="15" t="n"/>
       <c r="P15" s="15" t="n"/>
       <c r="Q15" s="15" t="n"/>
+      <c r="R15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -4991,6 +5008,7 @@
       <c r="O16" s="15" t="n"/>
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -5010,6 +5028,7 @@
       <c r="O17" s="15" t="n"/>
       <c r="P17" s="15" t="n"/>
       <c r="Q17" s="15" t="n"/>
+      <c r="R17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -5029,6 +5048,7 @@
       <c r="O18" s="15" t="n"/>
       <c r="P18" s="15" t="n"/>
       <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -5048,6 +5068,7 @@
       <c r="O19" s="15" t="n"/>
       <c r="P19" s="15" t="n"/>
       <c r="Q19" s="15" t="n"/>
+      <c r="R19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -5067,6 +5088,7 @@
       <c r="O20" s="15" t="n"/>
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="15" t="n"/>
+      <c r="R20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -5086,6 +5108,7 @@
       <c r="O21" s="15" t="n"/>
       <c r="P21" s="15" t="n"/>
       <c r="Q21" s="15" t="n"/>
+      <c r="R21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -5105,6 +5128,7 @@
       <c r="O22" s="15" t="n"/>
       <c r="P22" s="15" t="n"/>
       <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -5124,6 +5148,7 @@
       <c r="O23" s="15" t="n"/>
       <c r="P23" s="15" t="n"/>
       <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -5143,12 +5168,13 @@
       <c r="O24" s="15" t="n"/>
       <c r="P24" s="15" t="n"/>
       <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q24"/>
+  <autoFilter ref="A4:R24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">

</xml_diff>

<commit_message>
D04: resolver herrajes por clase y sellar componentes de fabricación (#122)
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$F$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$Q$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Precios de costo'!$A$4:$K$24</definedName>
   </definedNames>
 </workbook>
@@ -1711,8 +1711,8 @@
   </sheetData>
   <autoFilter ref="A4:K24"/>
   <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
@@ -4640,7 +4640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4658,8 +4658,9 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="47" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4755,10 +4756,15 @@
       </c>
       <c r="P4" s="14" t="inlineStr">
         <is>
-          <t>Componentes (JSON)</t>
+          <t>Componentes históricos (JSON)</t>
         </is>
       </c>
       <c r="Q4" s="14" t="inlineStr">
+        <is>
+          <t>Familia, clase y reglas de componentes (JSON)</t>
+        </is>
+      </c>
+      <c r="R4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -4782,6 +4788,7 @@
       <c r="O5" s="15" t="n"/>
       <c r="P5" s="15" t="n"/>
       <c r="Q5" s="15" t="n"/>
+      <c r="R5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -4801,6 +4808,7 @@
       <c r="O6" s="15" t="n"/>
       <c r="P6" s="15" t="n"/>
       <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -4820,6 +4828,7 @@
       <c r="O7" s="15" t="n"/>
       <c r="P7" s="15" t="n"/>
       <c r="Q7" s="15" t="n"/>
+      <c r="R7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -4839,6 +4848,7 @@
       <c r="O8" s="15" t="n"/>
       <c r="P8" s="15" t="n"/>
       <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -4858,6 +4868,7 @@
       <c r="O9" s="15" t="n"/>
       <c r="P9" s="15" t="n"/>
       <c r="Q9" s="15" t="n"/>
+      <c r="R9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -4877,6 +4888,7 @@
       <c r="O10" s="15" t="n"/>
       <c r="P10" s="15" t="n"/>
       <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -4896,6 +4908,7 @@
       <c r="O11" s="15" t="n"/>
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -4915,6 +4928,7 @@
       <c r="O12" s="15" t="n"/>
       <c r="P12" s="15" t="n"/>
       <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -4934,6 +4948,7 @@
       <c r="O13" s="15" t="n"/>
       <c r="P13" s="15" t="n"/>
       <c r="Q13" s="15" t="n"/>
+      <c r="R13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -4953,6 +4968,7 @@
       <c r="O14" s="15" t="n"/>
       <c r="P14" s="15" t="n"/>
       <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -4972,6 +4988,7 @@
       <c r="O15" s="15" t="n"/>
       <c r="P15" s="15" t="n"/>
       <c r="Q15" s="15" t="n"/>
+      <c r="R15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -4991,6 +5008,7 @@
       <c r="O16" s="15" t="n"/>
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -5010,6 +5028,7 @@
       <c r="O17" s="15" t="n"/>
       <c r="P17" s="15" t="n"/>
       <c r="Q17" s="15" t="n"/>
+      <c r="R17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -5029,6 +5048,7 @@
       <c r="O18" s="15" t="n"/>
       <c r="P18" s="15" t="n"/>
       <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -5048,6 +5068,7 @@
       <c r="O19" s="15" t="n"/>
       <c r="P19" s="15" t="n"/>
       <c r="Q19" s="15" t="n"/>
+      <c r="R19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -5067,6 +5088,7 @@
       <c r="O20" s="15" t="n"/>
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="15" t="n"/>
+      <c r="R20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -5086,6 +5108,7 @@
       <c r="O21" s="15" t="n"/>
       <c r="P21" s="15" t="n"/>
       <c r="Q21" s="15" t="n"/>
+      <c r="R21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -5105,6 +5128,7 @@
       <c r="O22" s="15" t="n"/>
       <c r="P22" s="15" t="n"/>
       <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -5124,6 +5148,7 @@
       <c r="O23" s="15" t="n"/>
       <c r="P23" s="15" t="n"/>
       <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -5143,12 +5168,13 @@
       <c r="O24" s="15" t="n"/>
       <c r="P24" s="15" t="n"/>
       <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q24"/>
+  <autoFilter ref="A4:R24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">

</xml_diff>

<commit_message>
D05: carta de acabados por caras y continuidad comercial
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AH$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AI$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$F$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$M$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
@@ -378,7 +378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH24"/>
+  <dimension ref="A1:AI24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -402,19 +402,20 @@
     <col width="22" customWidth="1" min="19" max="19"/>
     <col width="36" customWidth="1" min="20" max="20"/>
     <col width="33" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="39" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="23" customWidth="1" min="25" max="25"/>
-    <col width="32" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="29" customWidth="1" min="28" max="28"/>
-    <col width="28" customWidth="1" min="29" max="29"/>
-    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="23" customWidth="1" min="26" max="26"/>
+    <col width="32" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="29" customWidth="1" min="29" max="29"/>
+    <col width="28" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,65 +541,70 @@
       </c>
       <c r="V4" s="14" t="inlineStr">
         <is>
+          <t>Carta de colores por caras con fuente</t>
+        </is>
+      </c>
+      <c r="W4" s="14" t="inlineStr">
+        <is>
           <t>Versión</t>
         </is>
       </c>
-      <c r="W4" s="14" t="inlineStr">
+      <c r="X4" s="14" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="X4" s="14" t="inlineStr">
+      <c r="Y4" s="14" t="inlineStr">
         <is>
           <t>Altura rodamiento (mm)</t>
         </is>
       </c>
-      <c r="Y4" s="14" t="inlineStr">
+      <c r="Z4" s="14" t="inlineStr">
         <is>
           <t>Traslape central (mm)</t>
         </is>
       </c>
-      <c r="Z4" s="14" t="inlineStr">
+      <c r="AA4" s="14" t="inlineStr">
         <is>
           <t>Holgura lateral corredera (mm)</t>
         </is>
       </c>
-      <c r="AA4" s="14" t="inlineStr">
+      <c r="AB4" s="14" t="inlineStr">
         <is>
           <t>Adición corredera (mm)</t>
         </is>
       </c>
-      <c r="AB4" s="14" t="inlineStr">
+      <c r="AC4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio ancho (mm)</t>
         </is>
       </c>
-      <c r="AC4" s="14" t="inlineStr">
+      <c r="AD4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio alto (mm)</t>
         </is>
       </c>
-      <c r="AD4" s="14" t="inlineStr">
+      <c r="AE4" s="14" t="inlineStr">
         <is>
           <t>Tipo de riel</t>
         </is>
       </c>
-      <c r="AE4" s="14" t="inlineStr">
+      <c r="AF4" s="14" t="inlineStr">
         <is>
           <t>Cantidad de carriles</t>
         </is>
       </c>
-      <c r="AF4" s="14" t="inlineStr">
+      <c r="AG4" s="14" t="inlineStr">
         <is>
           <t>Riel separado</t>
         </is>
       </c>
-      <c r="AG4" s="14" t="inlineStr">
+      <c r="AH4" s="14" t="inlineStr">
         <is>
           <t>Encuentro requerido</t>
         </is>
       </c>
-      <c r="AH4" s="14" t="inlineStr">
+      <c r="AI4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -639,6 +645,7 @@
       <c r="AF5" s="15" t="n"/>
       <c r="AG5" s="15" t="n"/>
       <c r="AH5" s="15" t="n"/>
+      <c r="AI5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -675,6 +682,7 @@
       <c r="AF6" s="15" t="n"/>
       <c r="AG6" s="15" t="n"/>
       <c r="AH6" s="15" t="n"/>
+      <c r="AI6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -711,6 +719,7 @@
       <c r="AF7" s="15" t="n"/>
       <c r="AG7" s="15" t="n"/>
       <c r="AH7" s="15" t="n"/>
+      <c r="AI7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -747,6 +756,7 @@
       <c r="AF8" s="15" t="n"/>
       <c r="AG8" s="15" t="n"/>
       <c r="AH8" s="15" t="n"/>
+      <c r="AI8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -783,6 +793,7 @@
       <c r="AF9" s="15" t="n"/>
       <c r="AG9" s="15" t="n"/>
       <c r="AH9" s="15" t="n"/>
+      <c r="AI9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -819,6 +830,7 @@
       <c r="AF10" s="15" t="n"/>
       <c r="AG10" s="15" t="n"/>
       <c r="AH10" s="15" t="n"/>
+      <c r="AI10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -855,6 +867,7 @@
       <c r="AF11" s="15" t="n"/>
       <c r="AG11" s="15" t="n"/>
       <c r="AH11" s="15" t="n"/>
+      <c r="AI11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -891,6 +904,7 @@
       <c r="AF12" s="15" t="n"/>
       <c r="AG12" s="15" t="n"/>
       <c r="AH12" s="15" t="n"/>
+      <c r="AI12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -927,6 +941,7 @@
       <c r="AF13" s="15" t="n"/>
       <c r="AG13" s="15" t="n"/>
       <c r="AH13" s="15" t="n"/>
+      <c r="AI13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -963,6 +978,7 @@
       <c r="AF14" s="15" t="n"/>
       <c r="AG14" s="15" t="n"/>
       <c r="AH14" s="15" t="n"/>
+      <c r="AI14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -999,6 +1015,7 @@
       <c r="AF15" s="15" t="n"/>
       <c r="AG15" s="15" t="n"/>
       <c r="AH15" s="15" t="n"/>
+      <c r="AI15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -1035,6 +1052,7 @@
       <c r="AF16" s="15" t="n"/>
       <c r="AG16" s="15" t="n"/>
       <c r="AH16" s="15" t="n"/>
+      <c r="AI16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -1071,6 +1089,7 @@
       <c r="AF17" s="15" t="n"/>
       <c r="AG17" s="15" t="n"/>
       <c r="AH17" s="15" t="n"/>
+      <c r="AI17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -1107,6 +1126,7 @@
       <c r="AF18" s="15" t="n"/>
       <c r="AG18" s="15" t="n"/>
       <c r="AH18" s="15" t="n"/>
+      <c r="AI18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -1143,6 +1163,7 @@
       <c r="AF19" s="15" t="n"/>
       <c r="AG19" s="15" t="n"/>
       <c r="AH19" s="15" t="n"/>
+      <c r="AI19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -1179,6 +1200,7 @@
       <c r="AF20" s="15" t="n"/>
       <c r="AG20" s="15" t="n"/>
       <c r="AH20" s="15" t="n"/>
+      <c r="AI20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -1215,6 +1237,7 @@
       <c r="AF21" s="15" t="n"/>
       <c r="AG21" s="15" t="n"/>
       <c r="AH21" s="15" t="n"/>
+      <c r="AI21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -1251,6 +1274,7 @@
       <c r="AF22" s="15" t="n"/>
       <c r="AG22" s="15" t="n"/>
       <c r="AH22" s="15" t="n"/>
+      <c r="AI22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -1287,6 +1311,7 @@
       <c r="AF23" s="15" t="n"/>
       <c r="AG23" s="15" t="n"/>
       <c r="AH23" s="15" t="n"/>
+      <c r="AI23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -1323,12 +1348,13 @@
       <c r="AF24" s="15" t="n"/>
       <c r="AG24" s="15" t="n"/>
       <c r="AH24" s="15" t="n"/>
+      <c r="AI24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AH24"/>
+  <autoFilter ref="A4:AI24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:AH2"/>
-    <mergeCell ref="A1:AH1"/>
+    <mergeCell ref="A2:AI2"/>
+    <mergeCell ref="A1:AI1"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation sqref="C5:C24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
@@ -1337,16 +1363,16 @@
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"PVC,Aluminio"</formula1>
     </dataValidation>
-    <dataValidation sqref="W5:W24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="X5:X24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AD5:AD24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AE5:AE24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Un carril,Doble carril"</formula1>
     </dataValidation>
-    <dataValidation sqref="AF5:AF24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AG5:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AG5:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AH5:AH24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3165,7 +3191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3174,6 +3200,13 @@
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3218,6 +3251,41 @@
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Fabricante de barra</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Proveedor de barra</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Combinación de caras del stock</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Código de regla de corte</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Versión de stock</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Unidad de compra</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Stock vigente</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -3230,6 +3298,13 @@
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="15" t="n"/>
       <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -3238,6 +3313,13 @@
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="15" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -3246,6 +3328,13 @@
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="15" t="n"/>
       <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
+      <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -3254,6 +3343,13 @@
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -3262,6 +3358,13 @@
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="15" t="n"/>
       <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -3270,6 +3373,13 @@
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -3278,6 +3388,13 @@
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
       <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -3286,6 +3403,13 @@
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -3294,6 +3418,13 @@
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -3302,6 +3433,13 @@
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -3310,6 +3448,13 @@
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="15" t="n"/>
       <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -3318,6 +3463,13 @@
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -3326,6 +3478,13 @@
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="15" t="n"/>
       <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -3334,6 +3493,13 @@
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -3342,6 +3508,13 @@
       <c r="D19" s="15" t="n"/>
       <c r="E19" s="15" t="n"/>
       <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -3350,6 +3523,13 @@
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="15" t="n"/>
       <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -3358,6 +3538,13 @@
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="15" t="n"/>
       <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -3366,6 +3553,13 @@
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="15" t="n"/>
       <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -3374,6 +3568,13 @@
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="15" t="n"/>
       <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -3382,13 +3583,28 @@
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="15" t="n"/>
       <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F24"/>
+  <autoFilter ref="A4:M24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="K5:K24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Barra"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L5:L24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
D05: colores por caras, SKU y recargos con autoridad (#123)
* D05: carta de acabados por caras y continuidad comercial

* D05: alinear delta y readiness con autoridad comercial

* test: preserve real response bodies across project navigation

* test: bind project body capture to the triggering request

* test: capture fresh project responses without intercepting traffic
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AH$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AI$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$F$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$M$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
@@ -378,7 +378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH24"/>
+  <dimension ref="A1:AI24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -402,19 +402,20 @@
     <col width="22" customWidth="1" min="19" max="19"/>
     <col width="36" customWidth="1" min="20" max="20"/>
     <col width="33" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="39" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="23" customWidth="1" min="25" max="25"/>
-    <col width="32" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="29" customWidth="1" min="28" max="28"/>
-    <col width="28" customWidth="1" min="29" max="29"/>
-    <col width="22" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="23" customWidth="1" min="26" max="26"/>
+    <col width="32" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="29" customWidth="1" min="29" max="29"/>
+    <col width="28" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,65 +541,70 @@
       </c>
       <c r="V4" s="14" t="inlineStr">
         <is>
+          <t>Carta de colores por caras con fuente</t>
+        </is>
+      </c>
+      <c r="W4" s="14" t="inlineStr">
+        <is>
           <t>Versión</t>
         </is>
       </c>
-      <c r="W4" s="14" t="inlineStr">
+      <c r="X4" s="14" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="X4" s="14" t="inlineStr">
+      <c r="Y4" s="14" t="inlineStr">
         <is>
           <t>Altura rodamiento (mm)</t>
         </is>
       </c>
-      <c r="Y4" s="14" t="inlineStr">
+      <c r="Z4" s="14" t="inlineStr">
         <is>
           <t>Traslape central (mm)</t>
         </is>
       </c>
-      <c r="Z4" s="14" t="inlineStr">
+      <c r="AA4" s="14" t="inlineStr">
         <is>
           <t>Holgura lateral corredera (mm)</t>
         </is>
       </c>
-      <c r="AA4" s="14" t="inlineStr">
+      <c r="AB4" s="14" t="inlineStr">
         <is>
           <t>Adición corredera (mm)</t>
         </is>
       </c>
-      <c r="AB4" s="14" t="inlineStr">
+      <c r="AC4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio ancho (mm)</t>
         </is>
       </c>
-      <c r="AC4" s="14" t="inlineStr">
+      <c r="AD4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio alto (mm)</t>
         </is>
       </c>
-      <c r="AD4" s="14" t="inlineStr">
+      <c r="AE4" s="14" t="inlineStr">
         <is>
           <t>Tipo de riel</t>
         </is>
       </c>
-      <c r="AE4" s="14" t="inlineStr">
+      <c r="AF4" s="14" t="inlineStr">
         <is>
           <t>Cantidad de carriles</t>
         </is>
       </c>
-      <c r="AF4" s="14" t="inlineStr">
+      <c r="AG4" s="14" t="inlineStr">
         <is>
           <t>Riel separado</t>
         </is>
       </c>
-      <c r="AG4" s="14" t="inlineStr">
+      <c r="AH4" s="14" t="inlineStr">
         <is>
           <t>Encuentro requerido</t>
         </is>
       </c>
-      <c r="AH4" s="14" t="inlineStr">
+      <c r="AI4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -639,6 +645,7 @@
       <c r="AF5" s="15" t="n"/>
       <c r="AG5" s="15" t="n"/>
       <c r="AH5" s="15" t="n"/>
+      <c r="AI5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -675,6 +682,7 @@
       <c r="AF6" s="15" t="n"/>
       <c r="AG6" s="15" t="n"/>
       <c r="AH6" s="15" t="n"/>
+      <c r="AI6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -711,6 +719,7 @@
       <c r="AF7" s="15" t="n"/>
       <c r="AG7" s="15" t="n"/>
       <c r="AH7" s="15" t="n"/>
+      <c r="AI7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -747,6 +756,7 @@
       <c r="AF8" s="15" t="n"/>
       <c r="AG8" s="15" t="n"/>
       <c r="AH8" s="15" t="n"/>
+      <c r="AI8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -783,6 +793,7 @@
       <c r="AF9" s="15" t="n"/>
       <c r="AG9" s="15" t="n"/>
       <c r="AH9" s="15" t="n"/>
+      <c r="AI9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -819,6 +830,7 @@
       <c r="AF10" s="15" t="n"/>
       <c r="AG10" s="15" t="n"/>
       <c r="AH10" s="15" t="n"/>
+      <c r="AI10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -855,6 +867,7 @@
       <c r="AF11" s="15" t="n"/>
       <c r="AG11" s="15" t="n"/>
       <c r="AH11" s="15" t="n"/>
+      <c r="AI11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -891,6 +904,7 @@
       <c r="AF12" s="15" t="n"/>
       <c r="AG12" s="15" t="n"/>
       <c r="AH12" s="15" t="n"/>
+      <c r="AI12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -927,6 +941,7 @@
       <c r="AF13" s="15" t="n"/>
       <c r="AG13" s="15" t="n"/>
       <c r="AH13" s="15" t="n"/>
+      <c r="AI13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -963,6 +978,7 @@
       <c r="AF14" s="15" t="n"/>
       <c r="AG14" s="15" t="n"/>
       <c r="AH14" s="15" t="n"/>
+      <c r="AI14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -999,6 +1015,7 @@
       <c r="AF15" s="15" t="n"/>
       <c r="AG15" s="15" t="n"/>
       <c r="AH15" s="15" t="n"/>
+      <c r="AI15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -1035,6 +1052,7 @@
       <c r="AF16" s="15" t="n"/>
       <c r="AG16" s="15" t="n"/>
       <c r="AH16" s="15" t="n"/>
+      <c r="AI16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -1071,6 +1089,7 @@
       <c r="AF17" s="15" t="n"/>
       <c r="AG17" s="15" t="n"/>
       <c r="AH17" s="15" t="n"/>
+      <c r="AI17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -1107,6 +1126,7 @@
       <c r="AF18" s="15" t="n"/>
       <c r="AG18" s="15" t="n"/>
       <c r="AH18" s="15" t="n"/>
+      <c r="AI18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -1143,6 +1163,7 @@
       <c r="AF19" s="15" t="n"/>
       <c r="AG19" s="15" t="n"/>
       <c r="AH19" s="15" t="n"/>
+      <c r="AI19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -1179,6 +1200,7 @@
       <c r="AF20" s="15" t="n"/>
       <c r="AG20" s="15" t="n"/>
       <c r="AH20" s="15" t="n"/>
+      <c r="AI20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -1215,6 +1237,7 @@
       <c r="AF21" s="15" t="n"/>
       <c r="AG21" s="15" t="n"/>
       <c r="AH21" s="15" t="n"/>
+      <c r="AI21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -1251,6 +1274,7 @@
       <c r="AF22" s="15" t="n"/>
       <c r="AG22" s="15" t="n"/>
       <c r="AH22" s="15" t="n"/>
+      <c r="AI22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -1287,6 +1311,7 @@
       <c r="AF23" s="15" t="n"/>
       <c r="AG23" s="15" t="n"/>
       <c r="AH23" s="15" t="n"/>
+      <c r="AI23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -1323,12 +1348,13 @@
       <c r="AF24" s="15" t="n"/>
       <c r="AG24" s="15" t="n"/>
       <c r="AH24" s="15" t="n"/>
+      <c r="AI24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AH24"/>
+  <autoFilter ref="A4:AI24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:AH2"/>
-    <mergeCell ref="A1:AH1"/>
+    <mergeCell ref="A2:AI2"/>
+    <mergeCell ref="A1:AI1"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation sqref="C5:C24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
@@ -1337,16 +1363,16 @@
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"PVC,Aluminio"</formula1>
     </dataValidation>
-    <dataValidation sqref="W5:W24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="X5:X24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AD5:AD24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AE5:AE24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Un carril,Doble carril"</formula1>
     </dataValidation>
-    <dataValidation sqref="AF5:AF24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AG5:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AG5:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AH5:AH24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3165,7 +3191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3174,6 +3200,13 @@
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3218,6 +3251,41 @@
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Fabricante de barra</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Proveedor de barra</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Combinación de caras del stock</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Código de regla de corte</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Versión de stock</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Unidad de compra</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Stock vigente</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -3230,6 +3298,13 @@
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="15" t="n"/>
       <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -3238,6 +3313,13 @@
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="15" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -3246,6 +3328,13 @@
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="15" t="n"/>
       <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
+      <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -3254,6 +3343,13 @@
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -3262,6 +3358,13 @@
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="15" t="n"/>
       <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -3270,6 +3373,13 @@
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -3278,6 +3388,13 @@
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
       <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -3286,6 +3403,13 @@
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -3294,6 +3418,13 @@
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="15" t="n"/>
       <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -3302,6 +3433,13 @@
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -3310,6 +3448,13 @@
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="15" t="n"/>
       <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -3318,6 +3463,13 @@
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -3326,6 +3478,13 @@
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="15" t="n"/>
       <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -3334,6 +3493,13 @@
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -3342,6 +3508,13 @@
       <c r="D19" s="15" t="n"/>
       <c r="E19" s="15" t="n"/>
       <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -3350,6 +3523,13 @@
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="15" t="n"/>
       <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -3358,6 +3538,13 @@
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="15" t="n"/>
       <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -3366,6 +3553,13 @@
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="15" t="n"/>
       <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -3374,6 +3568,13 @@
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="15" t="n"/>
       <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -3382,13 +3583,28 @@
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="15" t="n"/>
       <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F24"/>
+  <autoFilter ref="A4:M24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="K5:K24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Barra"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L5:L24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
D06: accesorios derivados, servicios y sublineas selladas
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AI$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
@@ -378,7 +378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI24"/>
+  <dimension ref="A1:AJ24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -403,19 +403,20 @@
     <col width="36" customWidth="1" min="20" max="20"/>
     <col width="33" customWidth="1" min="21" max="21"/>
     <col width="39" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="42" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
-    <col width="23" customWidth="1" min="26" max="26"/>
-    <col width="32" customWidth="1" min="27" max="27"/>
-    <col width="24" customWidth="1" min="28" max="28"/>
-    <col width="29" customWidth="1" min="29" max="29"/>
-    <col width="28" customWidth="1" min="30" max="30"/>
-    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="32" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="29" customWidth="1" min="30" max="30"/>
+    <col width="28" customWidth="1" min="31" max="31"/>
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,65 +547,70 @@
       </c>
       <c r="W4" s="14" t="inlineStr">
         <is>
+          <t>Accesorios y extras con tarifas y fuente</t>
+        </is>
+      </c>
+      <c r="X4" s="14" t="inlineStr">
+        <is>
           <t>Versión</t>
         </is>
       </c>
-      <c r="X4" s="14" t="inlineStr">
+      <c r="Y4" s="14" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="Y4" s="14" t="inlineStr">
+      <c r="Z4" s="14" t="inlineStr">
         <is>
           <t>Altura rodamiento (mm)</t>
         </is>
       </c>
-      <c r="Z4" s="14" t="inlineStr">
+      <c r="AA4" s="14" t="inlineStr">
         <is>
           <t>Traslape central (mm)</t>
         </is>
       </c>
-      <c r="AA4" s="14" t="inlineStr">
+      <c r="AB4" s="14" t="inlineStr">
         <is>
           <t>Holgura lateral corredera (mm)</t>
         </is>
       </c>
-      <c r="AB4" s="14" t="inlineStr">
+      <c r="AC4" s="14" t="inlineStr">
         <is>
           <t>Adición corredera (mm)</t>
         </is>
       </c>
-      <c r="AC4" s="14" t="inlineStr">
+      <c r="AD4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio ancho (mm)</t>
         </is>
       </c>
-      <c r="AD4" s="14" t="inlineStr">
+      <c r="AE4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio alto (mm)</t>
         </is>
       </c>
-      <c r="AE4" s="14" t="inlineStr">
+      <c r="AF4" s="14" t="inlineStr">
         <is>
           <t>Tipo de riel</t>
         </is>
       </c>
-      <c r="AF4" s="14" t="inlineStr">
+      <c r="AG4" s="14" t="inlineStr">
         <is>
           <t>Cantidad de carriles</t>
         </is>
       </c>
-      <c r="AG4" s="14" t="inlineStr">
+      <c r="AH4" s="14" t="inlineStr">
         <is>
           <t>Riel separado</t>
         </is>
       </c>
-      <c r="AH4" s="14" t="inlineStr">
+      <c r="AI4" s="14" t="inlineStr">
         <is>
           <t>Encuentro requerido</t>
         </is>
       </c>
-      <c r="AI4" s="14" t="inlineStr">
+      <c r="AJ4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -646,6 +652,7 @@
       <c r="AG5" s="15" t="n"/>
       <c r="AH5" s="15" t="n"/>
       <c r="AI5" s="15" t="n"/>
+      <c r="AJ5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -683,6 +690,7 @@
       <c r="AG6" s="15" t="n"/>
       <c r="AH6" s="15" t="n"/>
       <c r="AI6" s="15" t="n"/>
+      <c r="AJ6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -720,6 +728,7 @@
       <c r="AG7" s="15" t="n"/>
       <c r="AH7" s="15" t="n"/>
       <c r="AI7" s="15" t="n"/>
+      <c r="AJ7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -757,6 +766,7 @@
       <c r="AG8" s="15" t="n"/>
       <c r="AH8" s="15" t="n"/>
       <c r="AI8" s="15" t="n"/>
+      <c r="AJ8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -794,6 +804,7 @@
       <c r="AG9" s="15" t="n"/>
       <c r="AH9" s="15" t="n"/>
       <c r="AI9" s="15" t="n"/>
+      <c r="AJ9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -831,6 +842,7 @@
       <c r="AG10" s="15" t="n"/>
       <c r="AH10" s="15" t="n"/>
       <c r="AI10" s="15" t="n"/>
+      <c r="AJ10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -868,6 +880,7 @@
       <c r="AG11" s="15" t="n"/>
       <c r="AH11" s="15" t="n"/>
       <c r="AI11" s="15" t="n"/>
+      <c r="AJ11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -905,6 +918,7 @@
       <c r="AG12" s="15" t="n"/>
       <c r="AH12" s="15" t="n"/>
       <c r="AI12" s="15" t="n"/>
+      <c r="AJ12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -942,6 +956,7 @@
       <c r="AG13" s="15" t="n"/>
       <c r="AH13" s="15" t="n"/>
       <c r="AI13" s="15" t="n"/>
+      <c r="AJ13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -979,6 +994,7 @@
       <c r="AG14" s="15" t="n"/>
       <c r="AH14" s="15" t="n"/>
       <c r="AI14" s="15" t="n"/>
+      <c r="AJ14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -1016,6 +1032,7 @@
       <c r="AG15" s="15" t="n"/>
       <c r="AH15" s="15" t="n"/>
       <c r="AI15" s="15" t="n"/>
+      <c r="AJ15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -1053,6 +1070,7 @@
       <c r="AG16" s="15" t="n"/>
       <c r="AH16" s="15" t="n"/>
       <c r="AI16" s="15" t="n"/>
+      <c r="AJ16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -1090,6 +1108,7 @@
       <c r="AG17" s="15" t="n"/>
       <c r="AH17" s="15" t="n"/>
       <c r="AI17" s="15" t="n"/>
+      <c r="AJ17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -1127,6 +1146,7 @@
       <c r="AG18" s="15" t="n"/>
       <c r="AH18" s="15" t="n"/>
       <c r="AI18" s="15" t="n"/>
+      <c r="AJ18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -1164,6 +1184,7 @@
       <c r="AG19" s="15" t="n"/>
       <c r="AH19" s="15" t="n"/>
       <c r="AI19" s="15" t="n"/>
+      <c r="AJ19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -1201,6 +1222,7 @@
       <c r="AG20" s="15" t="n"/>
       <c r="AH20" s="15" t="n"/>
       <c r="AI20" s="15" t="n"/>
+      <c r="AJ20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -1238,6 +1260,7 @@
       <c r="AG21" s="15" t="n"/>
       <c r="AH21" s="15" t="n"/>
       <c r="AI21" s="15" t="n"/>
+      <c r="AJ21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -1275,6 +1298,7 @@
       <c r="AG22" s="15" t="n"/>
       <c r="AH22" s="15" t="n"/>
       <c r="AI22" s="15" t="n"/>
+      <c r="AJ22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -1312,6 +1336,7 @@
       <c r="AG23" s="15" t="n"/>
       <c r="AH23" s="15" t="n"/>
       <c r="AI23" s="15" t="n"/>
+      <c r="AJ23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -1349,12 +1374,13 @@
       <c r="AG24" s="15" t="n"/>
       <c r="AH24" s="15" t="n"/>
       <c r="AI24" s="15" t="n"/>
+      <c r="AJ24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AI24"/>
+  <autoFilter ref="A4:AJ24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:AI2"/>
-    <mergeCell ref="A1:AI1"/>
+    <mergeCell ref="A2:AJ2"/>
+    <mergeCell ref="A1:AJ1"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation sqref="C5:C24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
@@ -1363,16 +1389,16 @@
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"PVC,Aluminio"</formula1>
     </dataValidation>
-    <dataValidation sqref="X5:X24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="Y5:Y24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AE5:AE24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AF5:AF24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Un carril,Doble carril"</formula1>
     </dataValidation>
-    <dataValidation sqref="AG5:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AH5:AH24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AH5:AH24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AI5:AI24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
D06: accesorios y servicios con cantidades del motor y sublineas selladas (#124)
* D06: accesorios derivados, servicios y sublineas selladas

* D06: aislar borradores y deshacer por entidad

* D06: registrar gate final aislado y aceptacion

* D06: explicar servicios sin autoridad de moneda

* fix: aislar sugerencias por modulo y costos por rol

* fix: proteger tarifas de accesorios en catalogo y RLS

* fix: mantener lectura tecnica y atestaciones privadas de extras

* test: sincronizar lectura real del catalogo antes de verificar permisos

* docs: cerrar evidencia del gate y privacidad de D06
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AI$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
@@ -378,7 +378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI24"/>
+  <dimension ref="A1:AJ24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -403,19 +403,20 @@
     <col width="36" customWidth="1" min="20" max="20"/>
     <col width="33" customWidth="1" min="21" max="21"/>
     <col width="39" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="42" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
-    <col width="23" customWidth="1" min="26" max="26"/>
-    <col width="32" customWidth="1" min="27" max="27"/>
-    <col width="24" customWidth="1" min="28" max="28"/>
-    <col width="29" customWidth="1" min="29" max="29"/>
-    <col width="28" customWidth="1" min="30" max="30"/>
-    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="32" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="29" customWidth="1" min="30" max="30"/>
+    <col width="28" customWidth="1" min="31" max="31"/>
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
     <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,65 +547,70 @@
       </c>
       <c r="W4" s="14" t="inlineStr">
         <is>
+          <t>Accesorios y extras con tarifas y fuente</t>
+        </is>
+      </c>
+      <c r="X4" s="14" t="inlineStr">
+        <is>
           <t>Versión</t>
         </is>
       </c>
-      <c r="X4" s="14" t="inlineStr">
+      <c r="Y4" s="14" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="Y4" s="14" t="inlineStr">
+      <c r="Z4" s="14" t="inlineStr">
         <is>
           <t>Altura rodamiento (mm)</t>
         </is>
       </c>
-      <c r="Z4" s="14" t="inlineStr">
+      <c r="AA4" s="14" t="inlineStr">
         <is>
           <t>Traslape central (mm)</t>
         </is>
       </c>
-      <c r="AA4" s="14" t="inlineStr">
+      <c r="AB4" s="14" t="inlineStr">
         <is>
           <t>Holgura lateral corredera (mm)</t>
         </is>
       </c>
-      <c r="AB4" s="14" t="inlineStr">
+      <c r="AC4" s="14" t="inlineStr">
         <is>
           <t>Adición corredera (mm)</t>
         </is>
       </c>
-      <c r="AC4" s="14" t="inlineStr">
+      <c r="AD4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio ancho (mm)</t>
         </is>
       </c>
-      <c r="AD4" s="14" t="inlineStr">
+      <c r="AE4" s="14" t="inlineStr">
         <is>
           <t>Descuento vidrio alto (mm)</t>
         </is>
       </c>
-      <c r="AE4" s="14" t="inlineStr">
+      <c r="AF4" s="14" t="inlineStr">
         <is>
           <t>Tipo de riel</t>
         </is>
       </c>
-      <c r="AF4" s="14" t="inlineStr">
+      <c r="AG4" s="14" t="inlineStr">
         <is>
           <t>Cantidad de carriles</t>
         </is>
       </c>
-      <c r="AG4" s="14" t="inlineStr">
+      <c r="AH4" s="14" t="inlineStr">
         <is>
           <t>Riel separado</t>
         </is>
       </c>
-      <c r="AH4" s="14" t="inlineStr">
+      <c r="AI4" s="14" t="inlineStr">
         <is>
           <t>Encuentro requerido</t>
         </is>
       </c>
-      <c r="AI4" s="14" t="inlineStr">
+      <c r="AJ4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -646,6 +652,7 @@
       <c r="AG5" s="15" t="n"/>
       <c r="AH5" s="15" t="n"/>
       <c r="AI5" s="15" t="n"/>
+      <c r="AJ5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -683,6 +690,7 @@
       <c r="AG6" s="15" t="n"/>
       <c r="AH6" s="15" t="n"/>
       <c r="AI6" s="15" t="n"/>
+      <c r="AJ6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -720,6 +728,7 @@
       <c r="AG7" s="15" t="n"/>
       <c r="AH7" s="15" t="n"/>
       <c r="AI7" s="15" t="n"/>
+      <c r="AJ7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -757,6 +766,7 @@
       <c r="AG8" s="15" t="n"/>
       <c r="AH8" s="15" t="n"/>
       <c r="AI8" s="15" t="n"/>
+      <c r="AJ8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -794,6 +804,7 @@
       <c r="AG9" s="15" t="n"/>
       <c r="AH9" s="15" t="n"/>
       <c r="AI9" s="15" t="n"/>
+      <c r="AJ9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -831,6 +842,7 @@
       <c r="AG10" s="15" t="n"/>
       <c r="AH10" s="15" t="n"/>
       <c r="AI10" s="15" t="n"/>
+      <c r="AJ10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -868,6 +880,7 @@
       <c r="AG11" s="15" t="n"/>
       <c r="AH11" s="15" t="n"/>
       <c r="AI11" s="15" t="n"/>
+      <c r="AJ11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -905,6 +918,7 @@
       <c r="AG12" s="15" t="n"/>
       <c r="AH12" s="15" t="n"/>
       <c r="AI12" s="15" t="n"/>
+      <c r="AJ12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -942,6 +956,7 @@
       <c r="AG13" s="15" t="n"/>
       <c r="AH13" s="15" t="n"/>
       <c r="AI13" s="15" t="n"/>
+      <c r="AJ13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -979,6 +994,7 @@
       <c r="AG14" s="15" t="n"/>
       <c r="AH14" s="15" t="n"/>
       <c r="AI14" s="15" t="n"/>
+      <c r="AJ14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -1016,6 +1032,7 @@
       <c r="AG15" s="15" t="n"/>
       <c r="AH15" s="15" t="n"/>
       <c r="AI15" s="15" t="n"/>
+      <c r="AJ15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -1053,6 +1070,7 @@
       <c r="AG16" s="15" t="n"/>
       <c r="AH16" s="15" t="n"/>
       <c r="AI16" s="15" t="n"/>
+      <c r="AJ16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -1090,6 +1108,7 @@
       <c r="AG17" s="15" t="n"/>
       <c r="AH17" s="15" t="n"/>
       <c r="AI17" s="15" t="n"/>
+      <c r="AJ17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -1127,6 +1146,7 @@
       <c r="AG18" s="15" t="n"/>
       <c r="AH18" s="15" t="n"/>
       <c r="AI18" s="15" t="n"/>
+      <c r="AJ18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -1164,6 +1184,7 @@
       <c r="AG19" s="15" t="n"/>
       <c r="AH19" s="15" t="n"/>
       <c r="AI19" s="15" t="n"/>
+      <c r="AJ19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -1201,6 +1222,7 @@
       <c r="AG20" s="15" t="n"/>
       <c r="AH20" s="15" t="n"/>
       <c r="AI20" s="15" t="n"/>
+      <c r="AJ20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -1238,6 +1260,7 @@
       <c r="AG21" s="15" t="n"/>
       <c r="AH21" s="15" t="n"/>
       <c r="AI21" s="15" t="n"/>
+      <c r="AJ21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -1275,6 +1298,7 @@
       <c r="AG22" s="15" t="n"/>
       <c r="AH22" s="15" t="n"/>
       <c r="AI22" s="15" t="n"/>
+      <c r="AJ22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -1312,6 +1336,7 @@
       <c r="AG23" s="15" t="n"/>
       <c r="AH23" s="15" t="n"/>
       <c r="AI23" s="15" t="n"/>
+      <c r="AJ23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -1349,12 +1374,13 @@
       <c r="AG24" s="15" t="n"/>
       <c r="AH24" s="15" t="n"/>
       <c r="AI24" s="15" t="n"/>
+      <c r="AJ24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AI24"/>
+  <autoFilter ref="A4:AJ24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:AI2"/>
-    <mergeCell ref="A1:AI1"/>
+    <mergeCell ref="A2:AJ2"/>
+    <mergeCell ref="A1:AJ1"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation sqref="C5:C24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
@@ -1363,16 +1389,16 @@
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"PVC,Aluminio"</formula1>
     </dataValidation>
-    <dataValidation sqref="X5:X24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="Y5:Y24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AE5:AE24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AF5:AF24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Un carril,Doble carril"</formula1>
     </dataValidation>
-    <dataValidation sqref="AG5:AG24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AH5:AH24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="AH5:AH24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+    <dataValidation sqref="AI5:AI24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(P06): conjuntos con planta y autoridad de acoples
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$K$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
@@ -1787,7 +1787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1799,7 +1799,8 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1864,6 +1865,11 @@
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Ángulos y aporte desarrollado con fuente (JSON)</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -1880,6 +1886,7 @@
       <c r="H5" s="15" t="n"/>
       <c r="I5" s="15" t="n"/>
       <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -1892,6 +1899,7 @@
       <c r="H6" s="15" t="n"/>
       <c r="I6" s="15" t="n"/>
       <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -1904,6 +1912,7 @@
       <c r="H7" s="15" t="n"/>
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -1916,6 +1925,7 @@
       <c r="H8" s="15" t="n"/>
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -1928,6 +1938,7 @@
       <c r="H9" s="15" t="n"/>
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -1940,6 +1951,7 @@
       <c r="H10" s="15" t="n"/>
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -1952,6 +1964,7 @@
       <c r="H11" s="15" t="n"/>
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -1964,6 +1977,7 @@
       <c r="H12" s="15" t="n"/>
       <c r="I12" s="15" t="n"/>
       <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -1976,6 +1990,7 @@
       <c r="H13" s="15" t="n"/>
       <c r="I13" s="15" t="n"/>
       <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -1988,6 +2003,7 @@
       <c r="H14" s="15" t="n"/>
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -2000,6 +2016,7 @@
       <c r="H15" s="15" t="n"/>
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -2012,6 +2029,7 @@
       <c r="H16" s="15" t="n"/>
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -2024,6 +2042,7 @@
       <c r="H17" s="15" t="n"/>
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -2036,6 +2055,7 @@
       <c r="H18" s="15" t="n"/>
       <c r="I18" s="15" t="n"/>
       <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -2048,6 +2068,7 @@
       <c r="H19" s="15" t="n"/>
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -2060,6 +2081,7 @@
       <c r="H20" s="15" t="n"/>
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -2072,6 +2094,7 @@
       <c r="H21" s="15" t="n"/>
       <c r="I21" s="15" t="n"/>
       <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -2084,6 +2107,7 @@
       <c r="H22" s="15" t="n"/>
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -2096,6 +2120,7 @@
       <c r="H23" s="15" t="n"/>
       <c r="I23" s="15" t="n"/>
       <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -2108,12 +2133,13 @@
       <c r="H24" s="15" t="n"/>
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J24"/>
+  <autoFilter ref="A4:K24"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">

</xml_diff>

<commit_message>
P06: conjuntos con planta, ángulos y autoridad de acoples (#138)
* feat(P06): conjuntos con planta y autoridad de acoples

* docs(P06): evidencia y conocimiento verificado

* test(P06): espera vidrio antes de confirmar importación

* test(P06): actualiza expectativa del catálogo vigente

* test(P06): selecciona serie v7 en el flujo comercial

* test(P06): usa serie vigente en fixture de proyectos

* docs(P06): registra aceptación y Database Gate completo
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$K$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
@@ -1787,7 +1787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1799,7 +1799,8 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1864,6 +1865,11 @@
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Ángulos y aporte desarrollado con fuente (JSON)</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -1880,6 +1886,7 @@
       <c r="H5" s="15" t="n"/>
       <c r="I5" s="15" t="n"/>
       <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -1892,6 +1899,7 @@
       <c r="H6" s="15" t="n"/>
       <c r="I6" s="15" t="n"/>
       <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -1904,6 +1912,7 @@
       <c r="H7" s="15" t="n"/>
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -1916,6 +1925,7 @@
       <c r="H8" s="15" t="n"/>
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -1928,6 +1938,7 @@
       <c r="H9" s="15" t="n"/>
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -1940,6 +1951,7 @@
       <c r="H10" s="15" t="n"/>
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -1952,6 +1964,7 @@
       <c r="H11" s="15" t="n"/>
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -1964,6 +1977,7 @@
       <c r="H12" s="15" t="n"/>
       <c r="I12" s="15" t="n"/>
       <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -1976,6 +1990,7 @@
       <c r="H13" s="15" t="n"/>
       <c r="I13" s="15" t="n"/>
       <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -1988,6 +2003,7 @@
       <c r="H14" s="15" t="n"/>
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -2000,6 +2016,7 @@
       <c r="H15" s="15" t="n"/>
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -2012,6 +2029,7 @@
       <c r="H16" s="15" t="n"/>
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -2024,6 +2042,7 @@
       <c r="H17" s="15" t="n"/>
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -2036,6 +2055,7 @@
       <c r="H18" s="15" t="n"/>
       <c r="I18" s="15" t="n"/>
       <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -2048,6 +2068,7 @@
       <c r="H19" s="15" t="n"/>
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -2060,6 +2081,7 @@
       <c r="H20" s="15" t="n"/>
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -2072,6 +2094,7 @@
       <c r="H21" s="15" t="n"/>
       <c r="I21" s="15" t="n"/>
       <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -2084,6 +2107,7 @@
       <c r="H22" s="15" t="n"/>
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -2096,6 +2120,7 @@
       <c r="H23" s="15" t="n"/>
       <c r="I23" s="15" t="n"/>
       <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -2108,12 +2133,13 @@
       <c r="H24" s="15" t="n"/>
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J24"/>
+  <autoFilter ref="A4:K24"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">

</xml_diff>

<commit_message>
P16: autoridad visible y fuentes inmutables del catálogo
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$N$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
@@ -1787,7 +1787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1799,8 +1799,11 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1866,10 +1869,25 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
+          <t>Pérdida de soldadura del perfil (mm)</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Holgura de refuerzo (mm)</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Geometría, origen y orientación de sección</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
           <t>Ángulos y aporte desarrollado con fuente (JSON)</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -1887,6 +1905,9 @@
       <c r="I5" s="15" t="n"/>
       <c r="J5" s="15" t="n"/>
       <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
+      <c r="N5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -1900,6 +1921,9 @@
       <c r="I6" s="15" t="n"/>
       <c r="J6" s="15" t="n"/>
       <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
+      <c r="N6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -1913,6 +1937,9 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="15" t="n"/>
       <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
+      <c r="N7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -1926,6 +1953,9 @@
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="15" t="n"/>
       <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -1939,6 +1969,9 @@
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="15" t="n"/>
       <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
+      <c r="N9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -1952,6 +1985,9 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
+      <c r="N10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -1965,6 +2001,9 @@
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="15" t="n"/>
       <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -1978,6 +2017,9 @@
       <c r="I12" s="15" t="n"/>
       <c r="J12" s="15" t="n"/>
       <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -1991,6 +2033,9 @@
       <c r="I13" s="15" t="n"/>
       <c r="J13" s="15" t="n"/>
       <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
+      <c r="N13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -2004,6 +2049,9 @@
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="15" t="n"/>
       <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
+      <c r="N14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -2017,6 +2065,9 @@
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="15" t="n"/>
       <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
+      <c r="N15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -2030,6 +2081,9 @@
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="15" t="n"/>
       <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -2043,6 +2097,9 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -2056,6 +2113,9 @@
       <c r="I18" s="15" t="n"/>
       <c r="J18" s="15" t="n"/>
       <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -2069,6 +2129,9 @@
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="15" t="n"/>
       <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -2082,6 +2145,9 @@
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="15" t="n"/>
       <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -2095,6 +2161,9 @@
       <c r="I21" s="15" t="n"/>
       <c r="J21" s="15" t="n"/>
       <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
+      <c r="N21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -2108,6 +2177,9 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -2121,6 +2193,9 @@
       <c r="I23" s="15" t="n"/>
       <c r="J23" s="15" t="n"/>
       <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -2134,12 +2209,15 @@
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="15" t="n"/>
       <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K24"/>
+  <autoFilter ref="A4:N24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">

</xml_diff>

<commit_message>
P16: autoridad visible y fuentes inmutables del catálogo (#144)
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$N$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
@@ -1787,7 +1787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1799,8 +1799,11 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1866,10 +1869,25 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
+          <t>Pérdida de soldadura del perfil (mm)</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Holgura de refuerzo (mm)</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Geometría, origen y orientación de sección</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
           <t>Ángulos y aporte desarrollado con fuente (JSON)</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
@@ -1887,6 +1905,9 @@
       <c r="I5" s="15" t="n"/>
       <c r="J5" s="15" t="n"/>
       <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
+      <c r="N5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -1900,6 +1921,9 @@
       <c r="I6" s="15" t="n"/>
       <c r="J6" s="15" t="n"/>
       <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
+      <c r="N6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -1913,6 +1937,9 @@
       <c r="I7" s="15" t="n"/>
       <c r="J7" s="15" t="n"/>
       <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
+      <c r="N7" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -1926,6 +1953,9 @@
       <c r="I8" s="15" t="n"/>
       <c r="J8" s="15" t="n"/>
       <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -1939,6 +1969,9 @@
       <c r="I9" s="15" t="n"/>
       <c r="J9" s="15" t="n"/>
       <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
+      <c r="N9" s="15" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -1952,6 +1985,9 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
+      <c r="N10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -1965,6 +2001,9 @@
       <c r="I11" s="15" t="n"/>
       <c r="J11" s="15" t="n"/>
       <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -1978,6 +2017,9 @@
       <c r="I12" s="15" t="n"/>
       <c r="J12" s="15" t="n"/>
       <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -1991,6 +2033,9 @@
       <c r="I13" s="15" t="n"/>
       <c r="J13" s="15" t="n"/>
       <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
+      <c r="N13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -2004,6 +2049,9 @@
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="15" t="n"/>
       <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
+      <c r="N14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -2017,6 +2065,9 @@
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="15" t="n"/>
       <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
+      <c r="N15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -2030,6 +2081,9 @@
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="15" t="n"/>
       <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -2043,6 +2097,9 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -2056,6 +2113,9 @@
       <c r="I18" s="15" t="n"/>
       <c r="J18" s="15" t="n"/>
       <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -2069,6 +2129,9 @@
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="15" t="n"/>
       <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -2082,6 +2145,9 @@
       <c r="I20" s="15" t="n"/>
       <c r="J20" s="15" t="n"/>
       <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -2095,6 +2161,9 @@
       <c r="I21" s="15" t="n"/>
       <c r="J21" s="15" t="n"/>
       <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
+      <c r="N21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -2108,6 +2177,9 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -2121,6 +2193,9 @@
       <c r="I23" s="15" t="n"/>
       <c r="J23" s="15" t="n"/>
       <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -2134,12 +2209,15 @@
       <c r="I24" s="15" t="n"/>
       <c r="J24" s="15" t="n"/>
       <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K24"/>
+  <autoFilter ref="A4:N24"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">

</xml_diff>

<commit_message>
P10: la aceptación Proline llega del registro a la aprobación del cliente
- Plantilla oficial: hoja «Barras de refuerzo»; la importación del taller
  declara la compra de acero (migración + pgTAP 263). La cobertura ya no
  promete «cotizable» si una regla de refuerzo no tiene su barra.
- Primer uso: la biblioteca va primero si el taller no tiene serie propia;
  columnas que encogen a 390 px; el botón Asistente conserva su nombre en
  móvil; Documentos ignora una lectura superada.
- E2E proline-acceptance (1440 y 390): registro, taller, 2FA, empresa,
  PRO6004, ficha sintética, precios, ventana de prueba, 3 ventanas,
  emisión por correo y aprobación en el portal, con tiempos por paso.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -7,24 +7,26 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfiles" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles y reglas de corte" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refuerzos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Límites" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colores y SKU por color" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas de vidrio" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Barras de refuerzo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Límites" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colores y SKU por color" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas de vidrio" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Perfiles'!$A$4:$N$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Roles y reglas de corte'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Refuerzos'!$A$4:$L$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Límites'!$A$4:$J$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Colores y SKU por color'!$A$4:$M$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Precios de costo'!$A$4:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Barras de refuerzo'!$A$4:$N$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Límites'!$A$4:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Colores y SKU por color'!$A$4:$M$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Precios de costo'!$A$4:$K$24</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1412,6 +1414,563 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="47" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Herrajes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Código de sistema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Apertura</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Ancho mínimo de hoja (mm)</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Ancho máximo de hoja (mm)</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Alto mínimo de hoja (mm)</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Alto máximo de hoja (mm)</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Peso máximo de hoja (kg)</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Masa de kit (kg)</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de riel</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Capacidad de carros (kg)</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>Cantidad de carros</t>
+        </is>
+      </c>
+      <c r="N4" s="14" t="inlineStr">
+        <is>
+          <t>Cantidad de compases</t>
+        </is>
+      </c>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="P4" s="14" t="inlineStr">
+        <is>
+          <t>Componentes históricos (JSON)</t>
+        </is>
+      </c>
+      <c r="Q4" s="14" t="inlineStr">
+        <is>
+          <t>Familia, clase y reglas de componentes (JSON)</t>
+        </is>
+      </c>
+      <c r="R4" s="14" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="n"/>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
+      <c r="N5" s="15" t="n"/>
+      <c r="O5" s="15" t="n"/>
+      <c r="P5" s="15" t="n"/>
+      <c r="Q5" s="15" t="n"/>
+      <c r="R5" s="15" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
+      <c r="N6" s="15" t="n"/>
+      <c r="O6" s="15" t="n"/>
+      <c r="P6" s="15" t="n"/>
+      <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="15" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="15" t="n"/>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
+      <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
+      <c r="N7" s="15" t="n"/>
+      <c r="O7" s="15" t="n"/>
+      <c r="P7" s="15" t="n"/>
+      <c r="Q7" s="15" t="n"/>
+      <c r="R7" s="15" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="15" t="n"/>
+      <c r="O8" s="15" t="n"/>
+      <c r="P8" s="15" t="n"/>
+      <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="15" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
+      <c r="N9" s="15" t="n"/>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="15" t="n"/>
+      <c r="Q9" s="15" t="n"/>
+      <c r="R9" s="15" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
+      <c r="N10" s="15" t="n"/>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="15" t="n"/>
+      <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="15" t="n"/>
+      <c r="O11" s="15" t="n"/>
+      <c r="P11" s="15" t="n"/>
+      <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="15" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="15" t="n"/>
+      <c r="O12" s="15" t="n"/>
+      <c r="P12" s="15" t="n"/>
+      <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
+      <c r="N13" s="15" t="n"/>
+      <c r="O13" s="15" t="n"/>
+      <c r="P13" s="15" t="n"/>
+      <c r="Q13" s="15" t="n"/>
+      <c r="R13" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
+      <c r="N14" s="15" t="n"/>
+      <c r="O14" s="15" t="n"/>
+      <c r="P14" s="15" t="n"/>
+      <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="15" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
+      <c r="N15" s="15" t="n"/>
+      <c r="O15" s="15" t="n"/>
+      <c r="P15" s="15" t="n"/>
+      <c r="Q15" s="15" t="n"/>
+      <c r="R15" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
+      <c r="P16" s="15" t="n"/>
+      <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
+      <c r="P17" s="15" t="n"/>
+      <c r="Q17" s="15" t="n"/>
+      <c r="R17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
+      <c r="O19" s="15" t="n"/>
+      <c r="P19" s="15" t="n"/>
+      <c r="Q19" s="15" t="n"/>
+      <c r="R19" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
+      <c r="O20" s="15" t="n"/>
+      <c r="P20" s="15" t="n"/>
+      <c r="Q20" s="15" t="n"/>
+      <c r="R20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
+      <c r="N21" s="15" t="n"/>
+      <c r="O21" s="15" t="n"/>
+      <c r="P21" s="15" t="n"/>
+      <c r="Q21" s="15" t="n"/>
+      <c r="R21" s="15" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
+      <c r="O22" s="15" t="n"/>
+      <c r="P22" s="15" t="n"/>
+      <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="n"/>
+      <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="15" t="n"/>
+      <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:R24"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Practicable,Oscilobatiente,Corredera,Puerta,Proyectante"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K5:K24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Un carril,Doble carril"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O5:O24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2978,6 +3537,456 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Barras de refuerzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Código de sistema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>SKU de refuerzo</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>SKU comercial del refuerzo</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Nombre del refuerzo</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Largo de barra (mm)</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Unidad de compra</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Fabricante de barra</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Proveedor de barra</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Color del stock</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Código de regla de corte</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Versión de stock</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>Barra vigente</t>
+        </is>
+      </c>
+      <c r="N4" s="14" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="n"/>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
+      <c r="N5" s="15" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
+      <c r="N6" s="15" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="15" t="n"/>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
+      <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
+      <c r="N7" s="15" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="15" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
+      <c r="N9" s="15" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
+      <c r="N10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="15" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
+      <c r="N13" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
+      <c r="N14" s="15" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
+      <c r="N15" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
+      <c r="N21" s="15" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:N24"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="G5:G24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Barra"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M5:M24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3315,7 +4324,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3739,7 +4748,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4657,7 +5666,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4978,561 +5987,4 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="31" customWidth="1" min="16" max="16"/>
-    <col width="47" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Herrajes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Código de sistema</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Apertura</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>Ancho mínimo de hoja (mm)</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Ancho máximo de hoja (mm)</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>Alto mínimo de hoja (mm)</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>Alto máximo de hoja (mm)</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>Peso máximo de hoja (kg)</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>Masa de kit (kg)</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Tipo de riel</t>
-        </is>
-      </c>
-      <c r="L4" s="14" t="inlineStr">
-        <is>
-          <t>Capacidad de carros (kg)</t>
-        </is>
-      </c>
-      <c r="M4" s="14" t="inlineStr">
-        <is>
-          <t>Cantidad de carros</t>
-        </is>
-      </c>
-      <c r="N4" s="14" t="inlineStr">
-        <is>
-          <t>Cantidad de compases</t>
-        </is>
-      </c>
-      <c r="O4" s="14" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="P4" s="14" t="inlineStr">
-        <is>
-          <t>Componentes históricos (JSON)</t>
-        </is>
-      </c>
-      <c r="Q4" s="14" t="inlineStr">
-        <is>
-          <t>Familia, clase y reglas de componentes (JSON)</t>
-        </is>
-      </c>
-      <c r="R4" s="14" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="n"/>
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="15" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="15" t="n"/>
-      <c r="J5" s="15" t="n"/>
-      <c r="K5" s="15" t="n"/>
-      <c r="L5" s="15" t="n"/>
-      <c r="M5" s="15" t="n"/>
-      <c r="N5" s="15" t="n"/>
-      <c r="O5" s="15" t="n"/>
-      <c r="P5" s="15" t="n"/>
-      <c r="Q5" s="15" t="n"/>
-      <c r="R5" s="15" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="n"/>
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
-      <c r="H6" s="15" t="n"/>
-      <c r="I6" s="15" t="n"/>
-      <c r="J6" s="15" t="n"/>
-      <c r="K6" s="15" t="n"/>
-      <c r="L6" s="15" t="n"/>
-      <c r="M6" s="15" t="n"/>
-      <c r="N6" s="15" t="n"/>
-      <c r="O6" s="15" t="n"/>
-      <c r="P6" s="15" t="n"/>
-      <c r="Q6" s="15" t="n"/>
-      <c r="R6" s="15" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="n"/>
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="15" t="n"/>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="15" t="n"/>
-      <c r="J7" s="15" t="n"/>
-      <c r="K7" s="15" t="n"/>
-      <c r="L7" s="15" t="n"/>
-      <c r="M7" s="15" t="n"/>
-      <c r="N7" s="15" t="n"/>
-      <c r="O7" s="15" t="n"/>
-      <c r="P7" s="15" t="n"/>
-      <c r="Q7" s="15" t="n"/>
-      <c r="R7" s="15" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="n"/>
-      <c r="B8" s="15" t="n"/>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="15" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="15" t="n"/>
-      <c r="K8" s="15" t="n"/>
-      <c r="L8" s="15" t="n"/>
-      <c r="M8" s="15" t="n"/>
-      <c r="N8" s="15" t="n"/>
-      <c r="O8" s="15" t="n"/>
-      <c r="P8" s="15" t="n"/>
-      <c r="Q8" s="15" t="n"/>
-      <c r="R8" s="15" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="n"/>
-      <c r="B9" s="15" t="n"/>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
-      <c r="H9" s="15" t="n"/>
-      <c r="I9" s="15" t="n"/>
-      <c r="J9" s="15" t="n"/>
-      <c r="K9" s="15" t="n"/>
-      <c r="L9" s="15" t="n"/>
-      <c r="M9" s="15" t="n"/>
-      <c r="N9" s="15" t="n"/>
-      <c r="O9" s="15" t="n"/>
-      <c r="P9" s="15" t="n"/>
-      <c r="Q9" s="15" t="n"/>
-      <c r="R9" s="15" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="n"/>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="15" t="n"/>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="15" t="n"/>
-      <c r="J10" s="15" t="n"/>
-      <c r="K10" s="15" t="n"/>
-      <c r="L10" s="15" t="n"/>
-      <c r="M10" s="15" t="n"/>
-      <c r="N10" s="15" t="n"/>
-      <c r="O10" s="15" t="n"/>
-      <c r="P10" s="15" t="n"/>
-      <c r="Q10" s="15" t="n"/>
-      <c r="R10" s="15" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="n"/>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
-      <c r="H11" s="15" t="n"/>
-      <c r="I11" s="15" t="n"/>
-      <c r="J11" s="15" t="n"/>
-      <c r="K11" s="15" t="n"/>
-      <c r="L11" s="15" t="n"/>
-      <c r="M11" s="15" t="n"/>
-      <c r="N11" s="15" t="n"/>
-      <c r="O11" s="15" t="n"/>
-      <c r="P11" s="15" t="n"/>
-      <c r="Q11" s="15" t="n"/>
-      <c r="R11" s="15" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="n"/>
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="15" t="n"/>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="15" t="n"/>
-      <c r="K12" s="15" t="n"/>
-      <c r="L12" s="15" t="n"/>
-      <c r="M12" s="15" t="n"/>
-      <c r="N12" s="15" t="n"/>
-      <c r="O12" s="15" t="n"/>
-      <c r="P12" s="15" t="n"/>
-      <c r="Q12" s="15" t="n"/>
-      <c r="R12" s="15" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="n"/>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="15" t="n"/>
-      <c r="I13" s="15" t="n"/>
-      <c r="J13" s="15" t="n"/>
-      <c r="K13" s="15" t="n"/>
-      <c r="L13" s="15" t="n"/>
-      <c r="M13" s="15" t="n"/>
-      <c r="N13" s="15" t="n"/>
-      <c r="O13" s="15" t="n"/>
-      <c r="P13" s="15" t="n"/>
-      <c r="Q13" s="15" t="n"/>
-      <c r="R13" s="15" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="n"/>
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="15" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="15" t="n"/>
-      <c r="H14" s="15" t="n"/>
-      <c r="I14" s="15" t="n"/>
-      <c r="J14" s="15" t="n"/>
-      <c r="K14" s="15" t="n"/>
-      <c r="L14" s="15" t="n"/>
-      <c r="M14" s="15" t="n"/>
-      <c r="N14" s="15" t="n"/>
-      <c r="O14" s="15" t="n"/>
-      <c r="P14" s="15" t="n"/>
-      <c r="Q14" s="15" t="n"/>
-      <c r="R14" s="15" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="n"/>
-      <c r="B15" s="15" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="15" t="n"/>
-      <c r="I15" s="15" t="n"/>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="15" t="n"/>
-      <c r="L15" s="15" t="n"/>
-      <c r="M15" s="15" t="n"/>
-      <c r="N15" s="15" t="n"/>
-      <c r="O15" s="15" t="n"/>
-      <c r="P15" s="15" t="n"/>
-      <c r="Q15" s="15" t="n"/>
-      <c r="R15" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="15" t="n"/>
-      <c r="I16" s="15" t="n"/>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="15" t="n"/>
-      <c r="L16" s="15" t="n"/>
-      <c r="M16" s="15" t="n"/>
-      <c r="N16" s="15" t="n"/>
-      <c r="O16" s="15" t="n"/>
-      <c r="P16" s="15" t="n"/>
-      <c r="Q16" s="15" t="n"/>
-      <c r="R16" s="15" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="n"/>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="15" t="n"/>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="15" t="n"/>
-      <c r="M17" s="15" t="n"/>
-      <c r="N17" s="15" t="n"/>
-      <c r="O17" s="15" t="n"/>
-      <c r="P17" s="15" t="n"/>
-      <c r="Q17" s="15" t="n"/>
-      <c r="R17" s="15" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="n"/>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n"/>
-      <c r="H18" s="15" t="n"/>
-      <c r="I18" s="15" t="n"/>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="15" t="n"/>
-      <c r="M18" s="15" t="n"/>
-      <c r="N18" s="15" t="n"/>
-      <c r="O18" s="15" t="n"/>
-      <c r="P18" s="15" t="n"/>
-      <c r="Q18" s="15" t="n"/>
-      <c r="R18" s="15" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="n"/>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="15" t="n"/>
-      <c r="I19" s="15" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="15" t="n"/>
-      <c r="M19" s="15" t="n"/>
-      <c r="N19" s="15" t="n"/>
-      <c r="O19" s="15" t="n"/>
-      <c r="P19" s="15" t="n"/>
-      <c r="Q19" s="15" t="n"/>
-      <c r="R19" s="15" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="15" t="n"/>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="15" t="n"/>
-      <c r="I20" s="15" t="n"/>
-      <c r="J20" s="15" t="n"/>
-      <c r="K20" s="15" t="n"/>
-      <c r="L20" s="15" t="n"/>
-      <c r="M20" s="15" t="n"/>
-      <c r="N20" s="15" t="n"/>
-      <c r="O20" s="15" t="n"/>
-      <c r="P20" s="15" t="n"/>
-      <c r="Q20" s="15" t="n"/>
-      <c r="R20" s="15" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="n"/>
-      <c r="B21" s="15" t="n"/>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="15" t="n"/>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="15" t="n"/>
-      <c r="I21" s="15" t="n"/>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="15" t="n"/>
-      <c r="L21" s="15" t="n"/>
-      <c r="M21" s="15" t="n"/>
-      <c r="N21" s="15" t="n"/>
-      <c r="O21" s="15" t="n"/>
-      <c r="P21" s="15" t="n"/>
-      <c r="Q21" s="15" t="n"/>
-      <c r="R21" s="15" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="n"/>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
-      <c r="G22" s="15" t="n"/>
-      <c r="H22" s="15" t="n"/>
-      <c r="I22" s="15" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="15" t="n"/>
-      <c r="L22" s="15" t="n"/>
-      <c r="M22" s="15" t="n"/>
-      <c r="N22" s="15" t="n"/>
-      <c r="O22" s="15" t="n"/>
-      <c r="P22" s="15" t="n"/>
-      <c r="Q22" s="15" t="n"/>
-      <c r="R22" s="15" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="n"/>
-      <c r="B23" s="15" t="n"/>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="15" t="n"/>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="15" t="n"/>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="n"/>
-      <c r="L23" s="15" t="n"/>
-      <c r="M23" s="15" t="n"/>
-      <c r="N23" s="15" t="n"/>
-      <c r="O23" s="15" t="n"/>
-      <c r="P23" s="15" t="n"/>
-      <c r="Q23" s="15" t="n"/>
-      <c r="R23" s="15" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="n"/>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
-      <c r="L24" s="15" t="n"/>
-      <c r="M24" s="15" t="n"/>
-      <c r="N24" s="15" t="n"/>
-      <c r="O24" s="15" t="n"/>
-      <c r="P24" s="15" t="n"/>
-      <c r="Q24" s="15" t="n"/>
-      <c r="R24" s="15" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:R24"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
-  </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
-      <formula1>"Practicable,Oscilobatiente,Corredera,Puerta,Proyectante"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K5:K24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
-      <formula1>"Un carril,Doble carril"</formula1>
-    </dataValidation>
-    <dataValidation sqref="O5:O24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Revise la opción" error="Elija un valor de la lista de esta columna." type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Compra completa para taller: aceros, kits, fijaciones y correos legibles
- Un mismo acero que refuerza marco y travesaño es una sola barra de
  compra, no una ambigüedad.
- Los componentes de un kit pueden declarar su código de compra y su
  fabricante; los kits Vorne de PRO6004 traen los de la OT 385.
- Nueva hoja «Fijaciones» en la planilla oficial: el tornillo del acero
  llega a la orden de compra (migración 20270214000100).
- Las barras compradas lisas toman el perfil de corte por defecto del
  taller; una posición sin compra completa se sella solo cotización y
  queda registrado por qué.
- Los correos muestran «Obra N° 44 · revisión A», nunca «P-000044 · REV-A».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/ingest/templates/catalogo-v1.xlsx
+++ b/backend/ingest/templates/catalogo-v1.xlsx
@@ -13,7 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidrios" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas de vidrio" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Herrajes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fijaciones" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios de costo" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sistemas'!$A$4:$AJ$24</definedName>
@@ -26,7 +27,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Vidrios'!$A$4:$AF$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Reglas de vidrio'!$A$4:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Herrajes'!$A$4:$R$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Precios de costo'!$A$4:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Fijaciones'!$A$4:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Precios de costo'!$A$4:$K$24</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1971,6 +1973,508 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="47" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fijaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Completa los datos del proveedor. Vacío = Sin dato. Indica la fuente de cada fila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Código de sistema</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>SKU de compra</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Fabricante</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Versión</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="14" t="n"/>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="14" t="n"/>
+      <c r="L4" s="14" t="n"/>
+      <c r="M4" s="14" t="n"/>
+      <c r="N4" s="14" t="n"/>
+      <c r="O4" s="14" t="n"/>
+      <c r="P4" s="14" t="n"/>
+      <c r="Q4" s="14" t="n"/>
+      <c r="R4" s="14" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="n"/>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="15" t="n"/>
+      <c r="N5" s="15" t="n"/>
+      <c r="O5" s="15" t="n"/>
+      <c r="P5" s="15" t="n"/>
+      <c r="Q5" s="15" t="n"/>
+      <c r="R5" s="15" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="15" t="n"/>
+      <c r="D6" s="15" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="n"/>
+      <c r="N6" s="15" t="n"/>
+      <c r="O6" s="15" t="n"/>
+      <c r="P6" s="15" t="n"/>
+      <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="15" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="15" t="n"/>
+      <c r="C7" s="15" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
+      <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="15" t="n"/>
+      <c r="M7" s="15" t="n"/>
+      <c r="N7" s="15" t="n"/>
+      <c r="O7" s="15" t="n"/>
+      <c r="P7" s="15" t="n"/>
+      <c r="Q7" s="15" t="n"/>
+      <c r="R7" s="15" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="n"/>
+      <c r="N8" s="15" t="n"/>
+      <c r="O8" s="15" t="n"/>
+      <c r="P8" s="15" t="n"/>
+      <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="15" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="15" t="n"/>
+      <c r="N9" s="15" t="n"/>
+      <c r="O9" s="15" t="n"/>
+      <c r="P9" s="15" t="n"/>
+      <c r="Q9" s="15" t="n"/>
+      <c r="R9" s="15" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="n"/>
+      <c r="N10" s="15" t="n"/>
+      <c r="O10" s="15" t="n"/>
+      <c r="P10" s="15" t="n"/>
+      <c r="Q10" s="15" t="n"/>
+      <c r="R10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="15" t="n"/>
+      <c r="O11" s="15" t="n"/>
+      <c r="P11" s="15" t="n"/>
+      <c r="Q11" s="15" t="n"/>
+      <c r="R11" s="15" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="15" t="n"/>
+      <c r="O12" s="15" t="n"/>
+      <c r="P12" s="15" t="n"/>
+      <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+      <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="15" t="n"/>
+      <c r="N13" s="15" t="n"/>
+      <c r="O13" s="15" t="n"/>
+      <c r="P13" s="15" t="n"/>
+      <c r="Q13" s="15" t="n"/>
+      <c r="R13" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="n"/>
+      <c r="N14" s="15" t="n"/>
+      <c r="O14" s="15" t="n"/>
+      <c r="P14" s="15" t="n"/>
+      <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="15" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="15" t="n"/>
+      <c r="H15" s="15" t="n"/>
+      <c r="I15" s="15" t="n"/>
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="15" t="n"/>
+      <c r="N15" s="15" t="n"/>
+      <c r="O15" s="15" t="n"/>
+      <c r="P15" s="15" t="n"/>
+      <c r="Q15" s="15" t="n"/>
+      <c r="R15" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
+      <c r="P16" s="15" t="n"/>
+      <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
+      <c r="P17" s="15" t="n"/>
+      <c r="Q17" s="15" t="n"/>
+      <c r="R17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="15" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
+      <c r="O19" s="15" t="n"/>
+      <c r="P19" s="15" t="n"/>
+      <c r="Q19" s="15" t="n"/>
+      <c r="R19" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
+      <c r="O20" s="15" t="n"/>
+      <c r="P20" s="15" t="n"/>
+      <c r="Q20" s="15" t="n"/>
+      <c r="R20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="15" t="n"/>
+      <c r="N21" s="15" t="n"/>
+      <c r="O21" s="15" t="n"/>
+      <c r="P21" s="15" t="n"/>
+      <c r="Q21" s="15" t="n"/>
+      <c r="R21" s="15" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
+      <c r="O22" s="15" t="n"/>
+      <c r="P22" s="15" t="n"/>
+      <c r="Q22" s="15" t="n"/>
+      <c r="R22" s="15" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="15" t="n"/>
+      <c r="N23" s="15" t="n"/>
+      <c r="O23" s="15" t="n"/>
+      <c r="P23" s="15" t="n"/>
+      <c r="Q23" s="15" t="n"/>
+      <c r="R23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="15" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="15" t="n"/>
+      <c r="P24" s="15" t="n"/>
+      <c r="Q24" s="15" t="n"/>
+      <c r="R24" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G24"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>